<commit_message>
Generate game descriptions worksheet
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -1,8 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run of Show" sheetId="1" r:id="Rce59c564791d443e"/>
+    <x:sheet name="Run of Show" sheetId="1" r:id="Rce59c564791d443e"/>
+    <x:sheet name="descriptions" sheetId="2" r:id="rIdDescriptions"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2260,4 +2261,3494 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:P44"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+    <col min="7" max="7" width="31" customWidth="1"/>
+    <col min="8" max="8" width="56" customWidth="1"/>
+    <col min="9" max="9" width="82" customWidth="1"/>
+    <col min="10" max="10" width="42" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="13" max="13" width="25" customWidth="1"/>
+    <col min="14" max="14" width="25" customWidth="1"/>
+    <col min="15" max="15" width="13" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>SIX 2026 | Game Guide Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Editable game metadata currently mirrored from src/App.tsx and src/fullDescriptions.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Developer / Publisher</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Platforms (source)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Platforms (shown)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Availability</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Demo / Build</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Quick Overview</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>Full Description</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Official URL</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>Steam App ID</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>YouTube Video ID</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Media Slug</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>Media Folder</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>Online flag</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>Legacy source status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Ascent Rivals</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>GENUN Games</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>Competitive multiplayer racing blending driving, combat, ship upgrades, and four tactical heats.</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>A competitive multiplayer racing game that combines high-speed driving, ship-to-ship combat, and vehicle customization. Four heats give racers opportunities to earn currency through placement, eliminations, and objectives, then improve their ships between rounds. Success depends on mechanical skill, tactical decisions, and adapting in multiplayer or time trials.</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>https://www.ascentrivals.com/</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>2748420</t>
+        </is>
+      </c>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>lQkBSUMFlnk</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>ascentrivals</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>ascentrivals</t>
+        </is>
+      </c>
+      <c r="O4" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P4" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Breach Of Contract</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Fern Sprout Studios</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>itch.io</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>June 20, 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>Beta on itch.io</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>Fast tactical action: plan each breach, wield eldritch powers, and eliminate enemies to recharge.</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>A fast tactical action game built around planning a breach and then surviving the chaos that follows. Players study each room, choose an approach, and use strange eldritch abilities against the enemies inside. Eliminations restore energy, encouraging an aggressive rhythm once the plan goes into motion.</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>https://fern-sprout-studios.itch.io/breach-of-contract</t>
+        </is>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" s="17" t="inlineStr">
+        <is>
+          <t>D8xRftvI5iU</t>
+        </is>
+      </c>
+      <c r="M5" s="17" t="inlineStr">
+        <is>
+          <t>breachofcontract</t>
+        </is>
+      </c>
+      <c r="N5" s="17" t="inlineStr">
+        <is>
+          <t>breachofcontract</t>
+        </is>
+      </c>
+      <c r="O5" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>BroomSweeper</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>BandWidth Games</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>January 19, 2026</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>Minesweeper gone roguelike, with 150+ items, dust bunnies, and 16 floors of janitorial danger.</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>A roguelike spin on Minesweeper in which players stock a cleaning cart with more than 150 useful items while dealing with troublesome Dust Bunnies. Sixteen floors of Tentateq Tower stand between the player and the end of the shift, including seven hazardous materials that alter the familiar logic rules.</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K6" s="17" t="inlineStr">
+        <is>
+          <t>3473250</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="inlineStr">
+        <is>
+          <t>JCCfUywh9iY</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>broomsweeper</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>broomsweeper</t>
+        </is>
+      </c>
+      <c r="O6" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P6" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Cooking Fist</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Spaghetti Code LLC</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>A cooking fighting game with no health bars—fight for ingredients, pause to cook, and win by making the most food.</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>A cooking-focused fighting game without traditional health bars. Players battle over ingredients, but collecting three forces them to pause the fight and cook. Victory goes to the competitor who manages the brawl, ingredient gathering, and cooking windows well enough to produce the most food.</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>https://cookingfist.com/</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="inlineStr">
+        <is>
+          <t>3941360</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="inlineStr">
+        <is>
+          <t>oxuyE_pWvXw</t>
+        </is>
+      </c>
+      <c r="M7" s="17" t="inlineStr">
+        <is>
+          <t>cookingfist</t>
+        </is>
+      </c>
+      <c r="N7" s="17" t="inlineStr">
+        <is>
+          <t>cookingfist</t>
+        </is>
+      </c>
+      <c r="O7" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P7" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Creature Kitchen</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>The Rat Zone</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>February 6, 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and itch.io</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>A creepy-cozy cooking simulator about exploring a strange house and feeding local wildlife.</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>A creepy-cozy cooking simulator about befriending wildlife and preparing their favorite snacks. Players search a strange house, explore the surrounding forest, and learn more about its unusual inhabitants as the witching hour approaches.</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" s="17" t="inlineStr">
+        <is>
+          <t>3097300</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>3U8V5RcFSqs</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>creaturekitchen</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>creaturekitchen</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Desolus</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Mark J. Mayers</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam, PS5, Switch 2, Xbox Series</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Steam, PlayStation, Xbox, Switch</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Q3 2026 / Steam lists coming soon</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and Xbox</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>A Gothic first-person puzzle game about black holes, impossible architecture, and rebuilding a city across time.</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>A first-person puzzle game set in a Gothic city fractured between its past and future. Players create and manipulate black holes to solve impossible, Escher-like spatial puzzles. Traveling through time allows damaged structures to become whole again and may offer a way to save the city from ruin.</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>https://www.desolus.com</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>1003460</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>HxfV0AvwSIs</t>
+        </is>
+      </c>
+      <c r="M9" s="17" t="inlineStr">
+        <is>
+          <t>desolus</t>
+        </is>
+      </c>
+      <c r="N9" s="17" t="inlineStr">
+        <is>
+          <t>desolus</t>
+        </is>
+      </c>
+      <c r="O9" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" s="17" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Diabolocracy</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Chaos Gremlin Games</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Hellish corporate politics become a roguelite turn-based tactics game starring a team of Sins.</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>A roguelite turn-based tactics game where Hell's corporate bureaucracy runs on violence. Players assemble a team of Sins, fight for influence, endure meetings, and combine complementary abilities into powerful SIN-ergies. The goal is to complete a hostile takeover before the boss returns from vacation.</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t>4143850</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>xdvk8IQBGWI</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>diabolocracy</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>diabolocracy</t>
+        </is>
+      </c>
+      <c r="O10" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P10" s="17" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Dig Too Deep</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Punch Up Games</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Throw goblins at every problem in an action tower-defense roguelite where minions are also ammunition.</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>An action tower-defense roguelite where goblins solve nearly every problem. They mine scrap, build defenses, fight enemies, and can even be launched as ammunition. Players upgrade their goblin workforce and defend their troll against increasingly dangerous waves.</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>4280850</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>JSwNG2A444M</t>
+        </is>
+      </c>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t>digtoodeep</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="inlineStr">
+        <is>
+          <t>digtoodeep</t>
+        </is>
+      </c>
+      <c r="O11" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P11" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Dittori</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Blookerstein</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>A reality-breaking game with 200+ puzzles built around splitting objects into two linked copies.</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>A puzzle adventure set beneath the world, where an awakening ancient god threatens everything. The player can split an object so it exists in two places at once, with every change to one copy affecting the other. More than 200 handcrafted puzzles explore the increasingly reality-breaking consequences of that power.</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K12" s="17" t="inlineStr">
+        <is>
+          <t>4311980</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>0xXuZZ7F8Vs</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>dittori</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>dittori</t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P12" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="84" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Dungeon Bodega Simulator</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Alien Fruit Games</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>PC, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>March 23, 2026</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Grow crops, brew potions, forge weapons, serve customers, and investigate a dungeon mystery.</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>A narrative-driven shop game about growing crops, brewing potions, and forging weapons for customers. Running the business is only part of the job, because a mystery connected to the nearby dungeon gradually demands investigation.</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
+        <is>
+          <t>3458180</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>Hpbdtqusk3c</t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>dungeonbodegasimulator</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>dungeonbodegasimulator</t>
+        </is>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P13" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="84" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>End of Garbage</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Joshua Rosen (Rakelock LLC)</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>PC, Mac, Steam</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>March 13, 2026</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>A short first-person puzzle game about the dark surreality of endings, documents, bodies, and deduction.</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>A short first-person puzzle game about the dark surrealism of endings. Players sign documents, identify bodies, observe the stars, and work through a sequence of deduction and logic puzzles that turn ordinary bureaucratic tasks into something stranger.</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K14" s="17" t="inlineStr">
+        <is>
+          <t>4256210</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t>Eh56--dqBK4</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>endofgarbage</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>endofgarbage</t>
+        </is>
+      </c>
+      <c r="O14" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P14" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="84" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Fairy Circle</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Play Hooky</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>March 26, 2026</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>A bag-building roguelike where a Forest Keeper protects a fairytale home from the Gloom.</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>A bag-building roguelike set in a fairytale world. As a Forest Keeper, the player builds a collection of useful pieces and abilities while protecting their home from an encroaching shadow force known as the Gloom.</t>
+        </is>
+      </c>
+      <c r="J15" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>3962850</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="inlineStr">
+        <is>
+          <t>_QT6JHIRf1w</t>
+        </is>
+      </c>
+      <c r="M15" s="17" t="inlineStr">
+        <is>
+          <t>fairycircle</t>
+        </is>
+      </c>
+      <c r="N15" s="17" t="inlineStr">
+        <is>
+          <t>fairycircle</t>
+        </is>
+      </c>
+      <c r="O15" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P15" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Feeding Gooble</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Displacer Labs</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>itch.io</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>In development</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>No public download confirmed</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>A conveyor-belt roguelite about keeping Gooble fed while lab experiments complicate the test forever.</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>A roguelite experiment in which the player has volunteered—whether they like it or not—to keep Gooble fed. Food travels through a belt system while other laboratory experiments complicate the test. Players must balance the required calories, push their luck, and discover combinations that create useful synergies.</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" s="17" t="inlineStr">
+        <is>
+          <t>za-kJSvx9vA</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>feedinggooble</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>feedinggooble</t>
+        </is>
+      </c>
+      <c r="O16" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P16" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="84" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Gravity Goblins</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>The Rat Zone</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>A gravity-bending roguelite collectathon through an ever-shifting tower packed with coins and trinkets.</t>
+        </is>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>A gravity-bending roguelite collectathon set inside an ever-changing tower. Players manipulate geometry, collect coins, gather upgrades and trinkets, and spend time at the local arcade. Reaching the top requires mastering the tower's shifting spaces and uncovering the secret hidden there.</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>4102030</t>
+        </is>
+      </c>
+      <c r="L17" s="17" t="inlineStr">
+        <is>
+          <t>IUN1QLruuJ8</t>
+        </is>
+      </c>
+      <c r="M17" s="17" t="inlineStr">
+        <is>
+          <t>gravitygoblins</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>gravitygoblins</t>
+        </is>
+      </c>
+      <c r="O17" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P17" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="84" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Hamsteria</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>2WheelerDev</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>PC, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>A difficult two-player co-op game starring hamsters in attached wheels, with online, local, and solo play.</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>A demanding cooperative game about two hamsters moving in attached wheels. It supports online co-op, local co-op, and a single-player option, turning coordination and momentum into the central challenge.</t>
+        </is>
+      </c>
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>4430020</t>
+        </is>
+      </c>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>8wjcCM3xKQM</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>hamsteria</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>hamsteria</t>
+        </is>
+      </c>
+      <c r="O18" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P18" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="84" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Haunted Heist</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>autotroph games</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>PC, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>A 3–10 player PvP horror party game: heisters steal gems while tricksters weaponize a procedural mansion.</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>A round-based PvP horror party game for three to ten players. Heisters search a procedurally generated mansion for gems, while Tricksters deploy disruptive and dangerous abilities to frighten them, break their plans, and protect the haunted home.</t>
+        </is>
+      </c>
+      <c r="J19" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>4024440</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="inlineStr">
+        <is>
+          <t>QM9Ztbm9EjQ</t>
+        </is>
+      </c>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>hauntedheist</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>hauntedheist</t>
+        </is>
+      </c>
+      <c r="O19" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P19" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="84" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Hit &amp; Haunted</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Amnesiac Ghost</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>A murder mystery where you play both the hitman and the victim’s ghost to uncover who ordered the hit.</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>A top-down murder mystery told from both sides of the same killing. Players alternate between Ace, the hitman, and Eli, the victim's ghost. Their unlikely partnership must uncover who hired Ace and determine the motive behind the contract.</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>3574060</t>
+        </is>
+      </c>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>eRlyPFMJ1qs</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>hithaunted</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>hithaunted</t>
+        </is>
+      </c>
+      <c r="O20" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P20" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="84" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Hogen</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Scrappyard Games</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>April 2, 2025</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>A grid-based card battler where you face Death, craft powerful builds, and uncover what lies behind the game.</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>A grid-based card battler that begins after the player crosses to the other side and finds Death waiting with a deck. What initially appears to be a simple match may hide something deeper. Strategic positioning, carefully constructed builds, and powerful card combinations determine how far the player gets.</t>
+        </is>
+      </c>
+      <c r="J21" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>3575520</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="inlineStr">
+        <is>
+          <t>gGKx2EghID8</t>
+        </is>
+      </c>
+      <c r="M21" s="17" t="inlineStr">
+        <is>
+          <t>hogen</t>
+        </is>
+      </c>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>hogen</t>
+        </is>
+      </c>
+      <c r="O21" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P21" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>HYPERFIST</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Chirality</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>July 10, 2026</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Comic-styled first-person action focused on fast, fluid punching, grabbing, and mecha-fist combat.</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>A fast first-person melee action game presented with a comic-book style. Players control Heath, a local punk equipped with mechanical fists, and fight robotic enemies through a fluid combat system focused on punching, grabbing, and other close-range techniques.</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>3689210</t>
+        </is>
+      </c>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>m-P1E2uCtbM</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>hyperfist</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>hyperfist</t>
+        </is>
+      </c>
+      <c r="O22" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P22" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="84" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Killing Baby Hitler</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>The Coffee Industrial Complex</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and itch.io</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>A retro FPS through corrupted timelines using resistance art, grenades, dinosaurs, and a wicked guitar.</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>A retro-inspired first-person shooter about repairing timelines corrupted after a time-travel experiment goes wrong. Players fight fascism across altered versions of history, recover banned art to inspire resistance, throw grenades, ride dinosaurs, and use an extremely loud guitar against Nazi enemies.</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>3317230</t>
+        </is>
+      </c>
+      <c r="L23" s="17" t="inlineStr">
+        <is>
+          <t>p2ENhCALff0</t>
+        </is>
+      </c>
+      <c r="M23" s="17" t="inlineStr">
+        <is>
+          <t>killingbabyhitler</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>killingbabyhitler</t>
+        </is>
+      </c>
+      <c r="O23" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P23" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Knockout 2: Wrath of the Karen</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>ExceptioNULL Games</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam, Mobile</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Steam, Mobile</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>In development</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t>A comedic boxing adventure where the Federal Boxing Investigations settles every argument in the ring.</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>A comedic boxing adventure set in a world where disputes and laws are settled in the ring. The player joins the Federal Boxing Investigations and faces a rising threat to national security, the world, and—perhaps most importantly—the bureau's quarterly performance bonus.</t>
+        </is>
+      </c>
+      <c r="J24" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>2349350</t>
+        </is>
+      </c>
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>7qiAh0rK458</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>knockout2wrathofthekaren</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>knockout2wrathofthekaren</t>
+        </is>
+      </c>
+      <c r="O24" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P24" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="84" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Malice In Wonderland</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Slyglass Games</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>A fast action roguelike based on the original Wonderland stories, where time itself is your health.</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>A fast action roguelike inspired by the original Wonderland stories. The player fights the Hatter while trapped in an endlessly repeating tea time, with remaining time replacing a conventional health bar. Taking damage shortens the clock, failure rewinds the run, and Decrees can combine with existing abilities to create destructive new builds.</t>
+        </is>
+      </c>
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>4552140</t>
+        </is>
+      </c>
+      <c r="L25" s="17" t="inlineStr">
+        <is>
+          <t>PYI_usmMim8</t>
+        </is>
+      </c>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>maliceinwonderland</t>
+        </is>
+      </c>
+      <c r="N25" s="17" t="inlineStr">
+        <is>
+          <t>maliceinwonderland</t>
+        </is>
+      </c>
+      <c r="O25" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P25" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Manafinder II</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Wolfsden LLC</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>A console-style turn-based RPG emphasizing party roles, weapon choices, and elemental affinities.</t>
+        </is>
+      </c>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>A console-style role-playing game with turn-based battles emphasizing party roles, weapon choices, and elemental relationships. Players travel through varied locations including fungal wilderness, the Luperci town of Alba, and the human ruins of Cuauhtla while confronting beasts, the Purged, and other dangers.</t>
+        </is>
+      </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>4568010</t>
+        </is>
+      </c>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>uR8CokKtDYw</t>
+        </is>
+      </c>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t>manafinderii</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t>manafinderii</t>
+        </is>
+      </c>
+      <c r="O26" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P26" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>MYRIORAMA</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>J&amp;K Games</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>A stop-motion-styled top-down adventure where players rearrange dungeon rooms to solve puzzles.</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>A top-down adventure inspired by classic 2D Zelda games, with dungeons that can be rearranged room by room. Moving the dungeon itself becomes the key to solving puzzles and navigating its challenges. Low-frame-rate animation and handcrafted-looking environments give the world the appearance of a living stop-motion diorama.</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>4663150</t>
+        </is>
+      </c>
+      <c r="L27" s="17" t="inlineStr">
+        <is>
+          <t>ubZqNnt4tlo</t>
+        </is>
+      </c>
+      <c r="M27" s="17" t="inlineStr">
+        <is>
+          <t>myriorama</t>
+        </is>
+      </c>
+      <c r="N27" s="17" t="inlineStr">
+        <is>
+          <t>myriorama</t>
+        </is>
+      </c>
+      <c r="O27" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P27" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="84" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Nightmare Kitchen</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Byteback Studios</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>A co-op FPS roguelite where chefs fight monstrous food with ridiculous culinary weapons.</t>
+        </is>
+      </c>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>A cooperative first-person roguelite where the food is trying to eat the chefs. Teams explore restaurant-themed dungeons, fight deranged culinary monsters, and wield absurd food-inspired weapons. Between runs, players improve their chefs and rebuild the food court at Tater Hills Mall in preparation for the Food-Pocalypse.</t>
+        </is>
+      </c>
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>3077140</t>
+        </is>
+      </c>
+      <c r="L28" s="17" t="inlineStr">
+        <is>
+          <t>VVkEj57OxVc</t>
+        </is>
+      </c>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>nightmarekitchen</t>
+        </is>
+      </c>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>nightmarekitchen</t>
+        </is>
+      </c>
+      <c r="O28" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P28" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="84" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Nimbit Frontier</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Megasploot</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>A cozy creature-collecting life sim with detailed care, custom habitats, conservation, and roguelite expeditions.</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>A cozy creature-collecting life simulation with detailed creature care and roguelite exploration. Players raise Nimbits, design comfortable habitats, and venture into the changing Underwild to find rare species. Nurturing, discovery, atmosphere, and conservation are central to the experience.</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>2477710</t>
+        </is>
+      </c>
+      <c r="L29" s="17" t="inlineStr">
+        <is>
+          <t>YJxnDCrTqyM</t>
+        </is>
+      </c>
+      <c r="M29" s="17" t="inlineStr">
+        <is>
+          <t>nimbitfrontier</t>
+        </is>
+      </c>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>nimbitfrontier</t>
+        </is>
+      </c>
+      <c r="O29" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P29" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="84" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>RUNE GUNNER</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>False Summit</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>A 1–4 player co-op roguelite shooter where guns and magic fuse into chaotic, build-breaking runs.</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>A cooperative roguelite shooter for one to four players that combines firearms and magic. Classes can be mixed during a run, while stacking major upgrades creates increasingly powerful builds. Teams must survive chaotic encounters across a shattered world occupied by hostile Constructs.</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
+        <is>
+          <t>3769870</t>
+        </is>
+      </c>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>AdDfigLpSjg</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>runegunner</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>runegunner</t>
+        </is>
+      </c>
+      <c r="O30" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P30" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="84" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>SCP: Antimemetics Division</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Quadrant Five</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>In development</t>
+        </is>
+      </c>
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="H31" s="17" t="inlineStr">
+        <is>
+          <t>Tactile survival horror inside a locked-down SCP site where memory and reality are dangerous resources.</t>
+        </is>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>A tactile survival-horror game set after amnestics have taken effect and Site-48 has gone into lockdown. Players scavenge restricted equipment, earn access to forgotten areas, and manipulate reality while escaping lethal SCP anomalies. Memory itself is dangerous, because understanding too much can be fatal.</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr">
+        <is>
+          <t>4385740</t>
+        </is>
+      </c>
+      <c r="L31" s="17" t="inlineStr">
+        <is>
+          <t>3ENXLCf6c2o</t>
+        </is>
+      </c>
+      <c r="M31" s="17" t="inlineStr">
+        <is>
+          <t>scpantimemeticsdivision</t>
+        </is>
+      </c>
+      <c r="N31" s="17" t="inlineStr">
+        <is>
+          <t>scpantimemeticsdivision</t>
+        </is>
+      </c>
+      <c r="O31" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P31" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="84" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Seedborne Soldiers</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Hat Wobble Games</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>June 1, 2026</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>An auto-battler roguelike about growing heroes across time and space and assembling wild synergies.</t>
+        </is>
+      </c>
+      <c r="I32" s="17" t="inlineStr">
+        <is>
+          <t>An auto-battler roguelike about growing a team of heroes drawn from different points in time and space. Players level their recruits, equip new gear, and assemble powerful synergies while searching for an exit from a surreal dreamworld.</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr">
+        <is>
+          <t>3039930</t>
+        </is>
+      </c>
+      <c r="L32" s="17" t="inlineStr">
+        <is>
+          <t>ejA_7I6fPTk</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="inlineStr">
+        <is>
+          <t>seedbornesoldiers</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>seedbornesoldiers</t>
+        </is>
+      </c>
+      <c r="O32" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P32" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="84" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Shroomwood</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Sporelite Games</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>PC, Mac, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>Demo and playtest available on Steam</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>Play a tiny mushroom warrior in a transforming wilderness, mixing melee and ranged weapons.</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>A run-based action adventure set in a wilderness that changes and transforms. The player controls a small but determined mushroom warrior, combining melee and ranged weapons to battle the forest's peculiar creatures. The shifting environment is designed to make every run feel different.</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
+        <is>
+          <t>3504020</t>
+        </is>
+      </c>
+      <c r="L33" s="17" t="inlineStr">
+        <is>
+          <t>qZtAtZZIl_w</t>
+        </is>
+      </c>
+      <c r="M33" s="17" t="inlineStr">
+        <is>
+          <t>Martin%20Hundrup</t>
+        </is>
+      </c>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t>Martin%20Hundrup</t>
+        </is>
+      </c>
+      <c r="O33" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P33" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="84" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Steel Swarm: SURVIVOR</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Clay Token Game Studio, Inc.</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>PC, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and itch.io</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>A fast survivors-like where customizable drone formations overwhelm metal hordes solo or in co-op.</t>
+        </is>
+      </c>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>A fast survivors-style roguelite centered on commanding drones against enormous mechanical hordes. Players arrange formations, upgrade individual drones, and refine their setup during each run. Enemy waves can be challenged alone or with other players in cooperative multiplayer.</t>
+        </is>
+      </c>
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>4307100</t>
+        </is>
+      </c>
+      <c r="L34" s="17" t="inlineStr">
+        <is>
+          <t>poEK4BFvMYA</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="inlineStr">
+        <is>
+          <t>steelswarmsurvivor</t>
+        </is>
+      </c>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>steelswarmsurvivor</t>
+        </is>
+      </c>
+      <c r="O34" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P34" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="84" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Super Choppy</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Sumoshell Bombfunk</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>PC, Mac, Linux, Steam</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and itch.io</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>A pixel-art action platformer where Choppy uses an axe to throw, fly, climb, and chop.</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>A challenging action platformer with colorful retro pixel artwork and a deliberately silly revenge story. Choppy's axe is more than a weapon: it supports throwing, flying, climbing, chopping, and the advanced movement required to master each stage.</t>
+        </is>
+      </c>
+      <c r="J35" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr">
+        <is>
+          <t>3616860</t>
+        </is>
+      </c>
+      <c r="L35" s="17" t="inlineStr">
+        <is>
+          <t>b6UtITtVuxk</t>
+        </is>
+      </c>
+      <c r="M35" s="17" t="inlineStr">
+        <is>
+          <t>superchoppy</t>
+        </is>
+      </c>
+      <c r="N35" s="17" t="inlineStr">
+        <is>
+          <t>superchoppy</t>
+        </is>
+      </c>
+      <c r="O35" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P35" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="84" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Telera</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Entropico</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H36" s="17" t="inlineStr">
+        <is>
+          <t>A roguelike dice-builder about rolling, scoring, upgrading, combining magic items, and out-thinking luck.</t>
+        </is>
+      </c>
+      <c r="I36" s="17" t="inlineStr">
+        <is>
+          <t>A roguelike dice-building game for players who enjoy large scores and calculated risks. Each round involves rolling dice, earning points, and clearing levels; between rounds, players upgrade dice, acquire new ones, and combine magical items. Every run mixes luck, planning, and player choices on the path toward legendary bosses and a new high score.</t>
+        </is>
+      </c>
+      <c r="J36" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>4079370</t>
+        </is>
+      </c>
+      <c r="L36" s="17" t="inlineStr">
+        <is>
+          <t>Qv9GY_9RpGo</t>
+        </is>
+      </c>
+      <c r="M36" s="17" t="inlineStr">
+        <is>
+          <t>telera</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>telera</t>
+        </is>
+      </c>
+      <c r="O36" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P36" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="84" customHeight="1">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>The Assessment</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Miga Games</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="inlineStr">
+        <is>
+          <t>An archaeologist explores a forgotten castle, performs rituals, releases souls, and confronts corrupted memories.</t>
+        </is>
+      </c>
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>A narrative horror game about an archaeologist hired to examine a forgotten castle. The assignment reveals the truth behind human sacrifices sealed within its walls. Players perform rituals, free trapped souls, and experience Gabrielle's most painful memories as the castle's spirits distort them.</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>4081850</t>
+        </is>
+      </c>
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t>JR4hXyOlywQ</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>theassessment</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>theassessment</t>
+        </is>
+      </c>
+      <c r="O37" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P37" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="84" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>TileShire</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Boss Blob</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>PC, Mac, Steam</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H38" s="17" t="inlineStr">
+        <is>
+          <t>A minimalist townbuilder where placing and transforming tiles earns points, cards, and townsfolk.</t>
+        </is>
+      </c>
+      <c r="I38" s="17" t="inlineStr">
+        <is>
+          <t>A minimalist town-building game where placing and transforming tiles produces points and expands the settlement. As the shire develops, players draft new cards and recruit townsfolk whose abilities help turn a simple arrangement of tiles into a home filled with life.</t>
+        </is>
+      </c>
+      <c r="J38" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K38" s="17" t="inlineStr">
+        <is>
+          <t>4370780</t>
+        </is>
+      </c>
+      <c r="L38" s="17" t="inlineStr">
+        <is>
+          <t>C1afDQkrrLg</t>
+        </is>
+      </c>
+      <c r="M38" s="17" t="inlineStr">
+        <is>
+          <t>tileshire</t>
+        </is>
+      </c>
+      <c r="N38" s="17" t="inlineStr">
+        <is>
+          <t>tileshire</t>
+        </is>
+      </c>
+      <c r="O38" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P38" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="84" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>Tower Lab</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Play Tug Studio</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H39" s="17" t="inlineStr">
+        <is>
+          <t>A physics tower-defense roguelite: shrink, grow, split, and clone objects to push enemies away.</t>
+        </is>
+      </c>
+      <c r="I39" s="17" t="inlineStr">
+        <is>
+          <t>A physics-driven roguelite tower-defense game where enemies do not use traditional health. Projectiles and units are physical objects that can be enlarged, reduced, duplicated, or divided. Players combine towers into unusual contraptions designed to push entire enemy formations off the level.</t>
+        </is>
+      </c>
+      <c r="J39" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K39" s="17" t="inlineStr">
+        <is>
+          <t>3084810</t>
+        </is>
+      </c>
+      <c r="L39" s="17" t="inlineStr">
+        <is>
+          <t>FCEoowKglGA</t>
+        </is>
+      </c>
+      <c r="M39" s="17" t="inlineStr">
+        <is>
+          <t>towerlab</t>
+        </is>
+      </c>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>towerlab</t>
+        </is>
+      </c>
+      <c r="O39" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P39" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="84" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Tricky and the Dream Caster</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>PossQueen</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam</t>
+        </is>
+      </c>
+      <c r="H40" s="17" t="inlineStr">
+        <is>
+          <t>A colorful platforming adventure starring Tricky O’Possum and Volt the Mouse on a wizard-punching mission.</t>
+        </is>
+      </c>
+      <c r="I40" s="17" t="inlineStr">
+        <is>
+          <t>A platforming adventure about breaking a curse of eternal sleep by invading the responsible wizard's castle and beating him up. Players control Tricky O'Possum and Volt the Mouse as they run, jump, collect keys, and battle through the Dream Caster's realm on the way to his stronghold.</t>
+        </is>
+      </c>
+      <c r="J40" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K40" s="17" t="inlineStr">
+        <is>
+          <t>3564580</t>
+        </is>
+      </c>
+      <c r="L40" s="17" t="inlineStr">
+        <is>
+          <t>nzQXQ_nIGFk</t>
+        </is>
+      </c>
+      <c r="M40" s="17" t="inlineStr">
+        <is>
+          <t>trickyandthedreamcaster</t>
+        </is>
+      </c>
+      <c r="N40" s="17" t="inlineStr">
+        <is>
+          <t>trickyandthedreamcaster</t>
+        </is>
+      </c>
+      <c r="O40" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P40" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="84" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Turning Manor</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Sabbatical Games</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>Demo available on Steam and itch.io</t>
+        </is>
+      </c>
+      <c r="H41" s="17" t="inlineStr">
+        <is>
+          <t>An anomaly-spotting horror game with no resets, more lore, and leaderboards inside a suspicious workplace.</t>
+        </is>
+      </c>
+      <c r="I41" s="17" t="inlineStr">
+        <is>
+          <t>An anomaly-observation game that begins when unsettling events follow the signing of a new job contract. Players compare rooms and count differences while investigating the mystery of Turning Manor. The design expands the familiar anomaly format with persistent progress, additional story, and leaderboards rather than constant resets.</t>
+        </is>
+      </c>
+      <c r="J41" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K41" s="17" t="inlineStr">
+        <is>
+          <t>3855530</t>
+        </is>
+      </c>
+      <c r="L41" s="17" t="inlineStr">
+        <is>
+          <t>5JvE5PJ6-Bk</t>
+        </is>
+      </c>
+      <c r="M41" s="17" t="inlineStr">
+        <is>
+          <t>turningmanor</t>
+        </is>
+      </c>
+      <c r="N41" s="17" t="inlineStr">
+        <is>
+          <t>turningmanor</t>
+        </is>
+      </c>
+      <c r="O41" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P41" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="84" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>We Need An Army</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Elder Bear Games</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F42" s="17" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="G42" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H42" s="17" t="inlineStr">
+        <is>
+          <t>A tactical slots-based roguelike battler about collecting units, finding relics, and shuffling an army.</t>
+        </is>
+      </c>
+      <c r="I42" s="17" t="inlineStr">
+        <is>
+          <t>A tactical, slots-based roguelike battler about constructing the strongest possible army. Players collect units, uncover relics, and complete minigames that affect their forces. Success comes from making good combinations and shuffling the available pieces into a winning formation.</t>
+        </is>
+      </c>
+      <c r="J42" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K42" s="17" t="inlineStr">
+        <is>
+          <t>3671320</t>
+        </is>
+      </c>
+      <c r="L42" s="17" t="inlineStr">
+        <is>
+          <t>qagBhjgCvs0</t>
+        </is>
+      </c>
+      <c r="M42" s="17" t="inlineStr">
+        <is>
+          <t>weneedanarmy</t>
+        </is>
+      </c>
+      <c r="N42" s="17" t="inlineStr">
+        <is>
+          <t>weneedanarmy</t>
+        </is>
+      </c>
+      <c r="O42" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P42" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="84" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>WILL: Follow The Light</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>TomorrowHead Studio</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>PC, PlayStation, Steam</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>Steam, PlayStation</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>May 7, 2026</t>
+        </is>
+      </c>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>No public demo currently available</t>
+        </is>
+      </c>
+      <c r="H43" s="17" t="inlineStr">
+        <is>
+          <t>A story-driven first-person adventure puzzle about sailing harsh northern waters to reunite with family.</t>
+        </is>
+      </c>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>A story-driven first-person puzzle adventure about a dangerous personal journey through northern waters. Will sails across harsh, isolated landscapes while confronting environmental challenges and puzzles. His voyage is ultimately about finding peace, returning to his family, and understanding himself.</t>
+        </is>
+      </c>
+      <c r="J43" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K43" s="17" t="inlineStr">
+        <is>
+          <t>3144860</t>
+        </is>
+      </c>
+      <c r="L43" s="17" t="inlineStr">
+        <is>
+          <t>I7Scpm5vRIU</t>
+        </is>
+      </c>
+      <c r="M43" s="17" t="inlineStr">
+        <is>
+          <t>Roman%20Novikov</t>
+        </is>
+      </c>
+      <c r="N43" s="17" t="inlineStr">
+        <is>
+          <t>Roman%20Novikov</t>
+        </is>
+      </c>
+      <c r="O43" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P43" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="84" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Wrestle Story</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
+          <t>Tic Toc Games</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>PC, Steam</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>Not yet released</t>
+        </is>
+      </c>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="G44" s="17" t="inlineStr">
+        <is>
+          <t>No public demo listed</t>
+        </is>
+      </c>
+      <c r="H44" s="17" t="inlineStr">
+        <is>
+          <t>A smack-talking 3D wrestling RPG about creating a wrestler, building a tag team, and living the story.</t>
+        </is>
+      </c>
+      <c r="I44" s="17" t="inlineStr">
+        <is>
+          <t>A wrestling role-playing adventure filled with hard hits and louder personalities. Players design their own wrestler, assemble a tag team, and explore a large 3D world built around the spectacle and culture of professional wrestling.</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K44" s="17" t="inlineStr">
+        <is>
+          <t>2357610</t>
+        </is>
+      </c>
+      <c r="L44" s="17" t="inlineStr">
+        <is>
+          <t>Pbii7_HpooQ</t>
+        </is>
+      </c>
+      <c r="M44" s="17" t="inlineStr">
+        <is>
+          <t>wrestlestory</t>
+        </is>
+      </c>
+      <c r="N44" s="17" t="inlineStr">
+        <is>
+          <t>wrestlestory</t>
+        </is>
+      </c>
+      <c r="O44" s="17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P44" s="17" t="inlineStr">
+        <is>
+          <t>Verify status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:P44"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Drive app data from XLSX workbook
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -2265,25 +2265,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="7" max="7" width="31" customWidth="1"/>
-    <col min="8" max="8" width="56" customWidth="1"/>
-    <col min="9" max="9" width="82" customWidth="1"/>
-    <col min="10" max="10" width="42" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="19" customWidth="1"/>
-    <col min="13" max="13" width="25" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="31" customWidth="1"/>
+    <col min="9" max="9" width="56" customWidth="1"/>
+    <col min="10" max="10" width="82" customWidth="1"/>
+    <col min="11" max="11" width="42" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="19" customWidth="1"/>
     <col min="14" max="14" width="25" customWidth="1"/>
-    <col min="15" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="15" max="15" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2303,3452 +2302,3242 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>Game ID</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Developer / Publisher</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Platforms (source)</t>
-        </is>
-      </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Platforms (shown)</t>
+          <t>Platforms</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>Display Platforms</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
           <t>Availability</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Demo / Build</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Quick Overview</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>Full Description</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Official URL</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>Steam App ID</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>YouTube Video ID</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>Media Slug</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>Media Folder</t>
-        </is>
-      </c>
-      <c r="O3" s="9" t="inlineStr">
-        <is>
-          <t>Online flag</t>
-        </is>
-      </c>
-      <c r="P3" s="9" t="inlineStr">
-        <is>
-          <t>Legacy source status</t>
         </is>
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
+          <t>ascent-rivals</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
           <t>Ascent Rivals</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>GENUN Games</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Q4 2026</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>Competitive multiplayer racing blending driving, combat, ship upgrades, and four tactical heats.</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>A competitive multiplayer racing game that combines high-speed driving, ship-to-ship combat, and vehicle customization. Four heats give racers opportunities to earn currency through placement, eliminations, and objectives, then improve their ships between rounds. Success depends on mechanical skill, tactical decisions, and adapting in multiplayer or time trials.</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>https://www.ascentrivals.com/</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>2748420</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>lQkBSUMFlnk</t>
         </is>
       </c>
-      <c r="M4" s="17" t="inlineStr">
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>ascentrivals</t>
         </is>
       </c>
-      <c r="N4" s="17" t="inlineStr">
+      <c r="O4" s="17" t="inlineStr">
         <is>
           <t>ascentrivals</t>
-        </is>
-      </c>
-      <c r="O4" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P4" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
+          <t>breach-of-contract</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
           <t>Breach Of Contract</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Fern Sprout Studios</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>itch.io</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>June 20, 2026</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Beta on itch.io</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>Fast tactical action: plan each breach, wield eldritch powers, and eliminate enemies to recharge.</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>A fast tactical action game built around planning a breach and then surviving the chaos that follows. Players study each room, choose an approach, and use strange eldritch abilities against the enemies inside. Eliminations restore energy, encouraging an aggressive rhythm once the plan goes into motion.</t>
         </is>
       </c>
-      <c r="J5" s="17" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>https://fern-sprout-studios.itch.io/breach-of-contract</t>
         </is>
       </c>
-      <c r="K5" s="17" t="inlineStr">
+      <c r="L5" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="L5" s="17" t="inlineStr">
+      <c r="M5" s="17" t="inlineStr">
         <is>
           <t>D8xRftvI5iU</t>
         </is>
       </c>
-      <c r="M5" s="17" t="inlineStr">
+      <c r="N5" s="17" t="inlineStr">
         <is>
           <t>breachofcontract</t>
         </is>
       </c>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="O5" s="17" t="inlineStr">
         <is>
           <t>breachofcontract</t>
-        </is>
-      </c>
-      <c r="O5" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P5" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
+          <t>broomsweeper</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
           <t>BroomSweeper</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>BandWidth Games</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F6" s="17" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>January 19, 2026</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>Minesweeper gone roguelike, with 150+ items, dust bunnies, and 16 floors of janitorial danger.</t>
         </is>
       </c>
-      <c r="I6" s="17" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>A roguelike spin on Minesweeper in which players stock a cleaning cart with more than 150 useful items while dealing with troublesome Dust Bunnies. Sixteen floors of Tentateq Tower stand between the player and the end of the shift, including seven hazardous materials that alter the familiar logic rules.</t>
         </is>
       </c>
-      <c r="J6" s="17" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K6" s="17" t="inlineStr">
+      <c r="L6" s="17" t="inlineStr">
         <is>
           <t>3473250</t>
         </is>
       </c>
-      <c r="L6" s="17" t="inlineStr">
+      <c r="M6" s="17" t="inlineStr">
         <is>
           <t>JCCfUywh9iY</t>
         </is>
       </c>
-      <c r="M6" s="17" t="inlineStr">
+      <c r="N6" s="17" t="inlineStr">
         <is>
           <t>broomsweeper</t>
         </is>
       </c>
-      <c r="N6" s="17" t="inlineStr">
+      <c r="O6" s="17" t="inlineStr">
         <is>
           <t>broomsweeper</t>
-        </is>
-      </c>
-      <c r="O6" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P6" s="17" t="inlineStr">
-        <is>
-          <t>Released</t>
         </is>
       </c>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
+          <t>cooking-fist</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
           <t>Cooking Fist</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Spaghetti Code LLC</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>A cooking fighting game with no health bars—fight for ingredients, pause to cook, and win by making the most food.</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>A cooking-focused fighting game without traditional health bars. Players battle over ingredients, but collecting three forces them to pause the fight and cook. Victory goes to the competitor who manages the brawl, ingredient gathering, and cooking windows well enough to produce the most food.</t>
         </is>
       </c>
-      <c r="J7" s="17" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>https://cookingfist.com/</t>
         </is>
       </c>
-      <c r="K7" s="17" t="inlineStr">
+      <c r="L7" s="17" t="inlineStr">
         <is>
           <t>3941360</t>
         </is>
       </c>
-      <c r="L7" s="17" t="inlineStr">
+      <c r="M7" s="17" t="inlineStr">
         <is>
           <t>oxuyE_pWvXw</t>
         </is>
       </c>
-      <c r="M7" s="17" t="inlineStr">
+      <c r="N7" s="17" t="inlineStr">
         <is>
           <t>cookingfist</t>
         </is>
       </c>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="O7" s="17" t="inlineStr">
         <is>
           <t>cookingfist</t>
-        </is>
-      </c>
-      <c r="O7" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P7" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
+          <t>creature-kitchen</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
           <t>Creature Kitchen</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>The Rat Zone</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>February 6, 2026</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and itch.io</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>A creepy-cozy cooking simulator about exploring a strange house and feeding local wildlife.</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>A creepy-cozy cooking simulator about befriending wildlife and preparing their favorite snacks. Players search a strange house, explore the surrounding forest, and learn more about its unusual inhabitants as the witching hour approaches.</t>
         </is>
       </c>
-      <c r="J8" s="17" t="inlineStr">
+      <c r="K8" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K8" s="17" t="inlineStr">
+      <c r="L8" s="17" t="inlineStr">
         <is>
           <t>3097300</t>
         </is>
       </c>
-      <c r="L8" s="17" t="inlineStr">
+      <c r="M8" s="17" t="inlineStr">
         <is>
           <t>3U8V5RcFSqs</t>
         </is>
       </c>
-      <c r="M8" s="17" t="inlineStr">
+      <c r="N8" s="17" t="inlineStr">
         <is>
           <t>creaturekitchen</t>
         </is>
       </c>
-      <c r="N8" s="17" t="inlineStr">
+      <c r="O8" s="17" t="inlineStr">
         <is>
           <t>creaturekitchen</t>
-        </is>
-      </c>
-      <c r="O8" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P8" s="17" t="inlineStr">
-        <is>
-          <t>Released</t>
         </is>
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
+          <t>desolus</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
           <t>Desolus</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Mark J. Mayers</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>PC, Steam, PS5, Switch 2, Xbox Series</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Steam, PlayStation, Xbox, Switch</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Q3 2026 / Steam lists coming soon</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and Xbox</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>A Gothic first-person puzzle game about black holes, impossible architecture, and rebuilding a city across time.</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>A first-person puzzle game set in a Gothic city fractured between its past and future. Players create and manipulate black holes to solve impossible, Escher-like spatial puzzles. Traveling through time allows damaged structures to become whole again and may offer a way to save the city from ruin.</t>
         </is>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>https://www.desolus.com</t>
         </is>
       </c>
-      <c r="K9" s="17" t="inlineStr">
+      <c r="L9" s="17" t="inlineStr">
         <is>
           <t>1003460</t>
         </is>
       </c>
-      <c r="L9" s="17" t="inlineStr">
+      <c r="M9" s="17" t="inlineStr">
         <is>
           <t>HxfV0AvwSIs</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr">
+      <c r="N9" s="17" t="inlineStr">
         <is>
           <t>desolus</t>
         </is>
       </c>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="O9" s="17" t="inlineStr">
         <is>
           <t>desolus</t>
-        </is>
-      </c>
-      <c r="O9" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P9" s="17" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
         </is>
       </c>
     </row>
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
+          <t>diabolocracy</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
           <t>Diabolocracy</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Chaos Gremlin Games</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F10" s="17" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>Hellish corporate politics become a roguelite turn-based tactics game starring a team of Sins.</t>
         </is>
       </c>
-      <c r="I10" s="17" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr">
         <is>
           <t>A roguelite turn-based tactics game where Hell's corporate bureaucracy runs on violence. Players assemble a team of Sins, fight for influence, endure meetings, and combine complementary abilities into powerful SIN-ergies. The goal is to complete a hostile takeover before the boss returns from vacation.</t>
         </is>
       </c>
-      <c r="J10" s="17" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K10" s="17" t="inlineStr">
+      <c r="L10" s="17" t="inlineStr">
         <is>
           <t>4143850</t>
         </is>
       </c>
-      <c r="L10" s="17" t="inlineStr">
+      <c r="M10" s="17" t="inlineStr">
         <is>
           <t>xdvk8IQBGWI</t>
         </is>
       </c>
-      <c r="M10" s="17" t="inlineStr">
+      <c r="N10" s="17" t="inlineStr">
         <is>
           <t>diabolocracy</t>
         </is>
       </c>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="O10" s="17" t="inlineStr">
         <is>
           <t>diabolocracy</t>
-        </is>
-      </c>
-      <c r="O10" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P10" s="17" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
         </is>
       </c>
     </row>
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
+          <t>dig-too-deep</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
           <t>Dig Too Deep</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>Punch Up Games</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Throw goblins at every problem in an action tower-defense roguelite where minions are also ammunition.</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>An action tower-defense roguelite where goblins solve nearly every problem. They mine scrap, build defenses, fight enemies, and can even be launched as ammunition. Players upgrade their goblin workforce and defend their troll against increasingly dangerous waves.</t>
         </is>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K11" s="17" t="inlineStr">
+      <c r="L11" s="17" t="inlineStr">
         <is>
           <t>4280850</t>
         </is>
       </c>
-      <c r="L11" s="17" t="inlineStr">
+      <c r="M11" s="17" t="inlineStr">
         <is>
           <t>JSwNG2A444M</t>
         </is>
       </c>
-      <c r="M11" s="17" t="inlineStr">
+      <c r="N11" s="17" t="inlineStr">
         <is>
           <t>digtoodeep</t>
         </is>
       </c>
-      <c r="N11" s="17" t="inlineStr">
+      <c r="O11" s="17" t="inlineStr">
         <is>
           <t>digtoodeep</t>
-        </is>
-      </c>
-      <c r="O11" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P11" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
+          <t>dittori</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
           <t>Dittori</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>Blookerstein</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>A reality-breaking game with 200+ puzzles built around splitting objects into two linked copies.</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr">
         <is>
           <t>A puzzle adventure set beneath the world, where an awakening ancient god threatens everything. The player can split an object so it exists in two places at once, with every change to one copy affecting the other. More than 200 handcrafted puzzles explore the increasingly reality-breaking consequences of that power.</t>
         </is>
       </c>
-      <c r="J12" s="17" t="inlineStr">
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K12" s="17" t="inlineStr">
+      <c r="L12" s="17" t="inlineStr">
         <is>
           <t>4311980</t>
         </is>
       </c>
-      <c r="L12" s="17" t="inlineStr">
+      <c r="M12" s="17" t="inlineStr">
         <is>
           <t>0xXuZZ7F8Vs</t>
         </is>
       </c>
-      <c r="M12" s="17" t="inlineStr">
+      <c r="N12" s="17" t="inlineStr">
         <is>
           <t>dittori</t>
         </is>
       </c>
-      <c r="N12" s="17" t="inlineStr">
+      <c r="O12" s="17" t="inlineStr">
         <is>
           <t>dittori</t>
-        </is>
-      </c>
-      <c r="O12" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P12" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
+          <t>dungeon-bodega-simulator</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
           <t>Dungeon Bodega Simulator</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>Alien Fruit Games</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>PC, Linux, Steam</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>March 23, 2026</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>Grow crops, brew potions, forge weapons, serve customers, and investigate a dungeon mystery.</t>
         </is>
       </c>
-      <c r="I13" s="17" t="inlineStr">
+      <c r="J13" s="17" t="inlineStr">
         <is>
           <t>A narrative-driven shop game about growing crops, brewing potions, and forging weapons for customers. Running the business is only part of the job, because a mystery connected to the nearby dungeon gradually demands investigation.</t>
         </is>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K13" s="17" t="inlineStr">
+      <c r="L13" s="17" t="inlineStr">
         <is>
           <t>3458180</t>
         </is>
       </c>
-      <c r="L13" s="17" t="inlineStr">
+      <c r="M13" s="17" t="inlineStr">
         <is>
           <t>Hpbdtqusk3c</t>
         </is>
       </c>
-      <c r="M13" s="17" t="inlineStr">
+      <c r="N13" s="17" t="inlineStr">
         <is>
           <t>dungeonbodegasimulator</t>
         </is>
       </c>
-      <c r="N13" s="17" t="inlineStr">
+      <c r="O13" s="17" t="inlineStr">
         <is>
           <t>dungeonbodegasimulator</t>
-        </is>
-      </c>
-      <c r="O13" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P13" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
+          <t>end-of-garbage</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
           <t>End of Garbage</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>Joshua Rosen (Rakelock LLC)</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>PC, Mac, Steam</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>March 13, 2026</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="I14" s="17" t="inlineStr">
         <is>
           <t>A short first-person puzzle game about the dark surreality of endings, documents, bodies, and deduction.</t>
         </is>
       </c>
-      <c r="I14" s="17" t="inlineStr">
+      <c r="J14" s="17" t="inlineStr">
         <is>
           <t>A short first-person puzzle game about the dark surrealism of endings. Players sign documents, identify bodies, observe the stars, and work through a sequence of deduction and logic puzzles that turn ordinary bureaucratic tasks into something stranger.</t>
         </is>
       </c>
-      <c r="J14" s="17" t="inlineStr">
+      <c r="K14" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K14" s="17" t="inlineStr">
+      <c r="L14" s="17" t="inlineStr">
         <is>
           <t>4256210</t>
         </is>
       </c>
-      <c r="L14" s="17" t="inlineStr">
+      <c r="M14" s="17" t="inlineStr">
         <is>
           <t>Eh56--dqBK4</t>
         </is>
       </c>
-      <c r="M14" s="17" t="inlineStr">
+      <c r="N14" s="17" t="inlineStr">
         <is>
           <t>endofgarbage</t>
         </is>
       </c>
-      <c r="N14" s="17" t="inlineStr">
+      <c r="O14" s="17" t="inlineStr">
         <is>
           <t>endofgarbage</t>
-        </is>
-      </c>
-      <c r="O14" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P14" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="15" ht="84" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
+          <t>fairy-circle</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
           <t>Fairy Circle</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Play Hooky</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>March 26, 2026</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="I15" s="17" t="inlineStr">
         <is>
           <t>A bag-building roguelike where a Forest Keeper protects a fairytale home from the Gloom.</t>
         </is>
       </c>
-      <c r="I15" s="17" t="inlineStr">
+      <c r="J15" s="17" t="inlineStr">
         <is>
           <t>A bag-building roguelike set in a fairytale world. As a Forest Keeper, the player builds a collection of useful pieces and abilities while protecting their home from an encroaching shadow force known as the Gloom.</t>
         </is>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K15" s="17" t="inlineStr">
+      <c r="L15" s="17" t="inlineStr">
         <is>
           <t>3962850</t>
         </is>
       </c>
-      <c r="L15" s="17" t="inlineStr">
+      <c r="M15" s="17" t="inlineStr">
         <is>
           <t>_QT6JHIRf1w</t>
         </is>
       </c>
-      <c r="M15" s="17" t="inlineStr">
+      <c r="N15" s="17" t="inlineStr">
         <is>
           <t>fairycircle</t>
         </is>
       </c>
-      <c r="N15" s="17" t="inlineStr">
+      <c r="O15" s="17" t="inlineStr">
         <is>
           <t>fairycircle</t>
-        </is>
-      </c>
-      <c r="O15" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P15" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="16" ht="84" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
+          <t>feeding-gooble</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
           <t>Feeding Gooble</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>Displacer Labs</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>itch.io</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>In development</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>No public download confirmed</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
         <is>
           <t>A conveyor-belt roguelite about keeping Gooble fed while lab experiments complicate the test forever.</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr">
         <is>
           <t>A roguelite experiment in which the player has volunteered—whether they like it or not—to keep Gooble fed. Food travels through a belt system while other laboratory experiments complicate the test. Players must balance the required calories, push their luck, and discover combinations that create useful synergies.</t>
         </is>
       </c>
-      <c r="J16" s="17" t="inlineStr">
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K16" s="17" t="inlineStr">
+      <c r="L16" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="L16" s="17" t="inlineStr">
+      <c r="M16" s="17" t="inlineStr">
         <is>
           <t>za-kJSvx9vA</t>
         </is>
       </c>
-      <c r="M16" s="17" t="inlineStr">
+      <c r="N16" s="17" t="inlineStr">
         <is>
           <t>feedinggooble</t>
         </is>
       </c>
-      <c r="N16" s="17" t="inlineStr">
+      <c r="O16" s="17" t="inlineStr">
         <is>
           <t>feedinggooble</t>
-        </is>
-      </c>
-      <c r="O16" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P16" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="17" ht="84" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
+          <t>gravity-goblins</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
           <t>Gravity Goblins</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>The Rat Zone</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="I17" s="17" t="inlineStr">
         <is>
           <t>A gravity-bending roguelite collectathon through an ever-shifting tower packed with coins and trinkets.</t>
         </is>
       </c>
-      <c r="I17" s="17" t="inlineStr">
+      <c r="J17" s="17" t="inlineStr">
         <is>
           <t>A gravity-bending roguelite collectathon set inside an ever-changing tower. Players manipulate geometry, collect coins, gather upgrades and trinkets, and spend time at the local arcade. Reaching the top requires mastering the tower's shifting spaces and uncovering the secret hidden there.</t>
         </is>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K17" s="17" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t>4102030</t>
         </is>
       </c>
-      <c r="L17" s="17" t="inlineStr">
+      <c r="M17" s="17" t="inlineStr">
         <is>
           <t>IUN1QLruuJ8</t>
         </is>
       </c>
-      <c r="M17" s="17" t="inlineStr">
+      <c r="N17" s="17" t="inlineStr">
         <is>
           <t>gravitygoblins</t>
         </is>
       </c>
-      <c r="N17" s="17" t="inlineStr">
+      <c r="O17" s="17" t="inlineStr">
         <is>
           <t>gravitygoblins</t>
-        </is>
-      </c>
-      <c r="O17" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P17" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
+          <t>hamsteria</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
           <t>Hamsteria</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>2WheelerDev</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>PC, Linux, Steam</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>A difficult two-player co-op game starring hamsters in attached wheels, with online, local, and solo play.</t>
         </is>
       </c>
-      <c r="I18" s="17" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
         <is>
           <t>A demanding cooperative game about two hamsters moving in attached wheels. It supports online co-op, local co-op, and a single-player option, turning coordination and momentum into the central challenge.</t>
         </is>
       </c>
-      <c r="J18" s="17" t="inlineStr">
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K18" s="17" t="inlineStr">
+      <c r="L18" s="17" t="inlineStr">
         <is>
           <t>4430020</t>
         </is>
       </c>
-      <c r="L18" s="17" t="inlineStr">
+      <c r="M18" s="17" t="inlineStr">
         <is>
           <t>8wjcCM3xKQM</t>
         </is>
       </c>
-      <c r="M18" s="17" t="inlineStr">
+      <c r="N18" s="17" t="inlineStr">
         <is>
           <t>hamsteria</t>
         </is>
       </c>
-      <c r="N18" s="17" t="inlineStr">
+      <c r="O18" s="17" t="inlineStr">
         <is>
           <t>hamsteria</t>
-        </is>
-      </c>
-      <c r="O18" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P18" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="19" ht="84" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
+          <t>haunted-heist</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
           <t>Haunted Heist</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>autotroph games</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>PC, Linux, Steam</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="I19" s="17" t="inlineStr">
         <is>
           <t>A 3–10 player PvP horror party game: heisters steal gems while tricksters weaponize a procedural mansion.</t>
         </is>
       </c>
-      <c r="I19" s="17" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>A round-based PvP horror party game for three to ten players. Heisters search a procedurally generated mansion for gems, while Tricksters deploy disruptive and dangerous abilities to frighten them, break their plans, and protect the haunted home.</t>
         </is>
       </c>
-      <c r="J19" s="17" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K19" s="17" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr">
         <is>
           <t>4024440</t>
         </is>
       </c>
-      <c r="L19" s="17" t="inlineStr">
+      <c r="M19" s="17" t="inlineStr">
         <is>
           <t>QM9Ztbm9EjQ</t>
         </is>
       </c>
-      <c r="M19" s="17" t="inlineStr">
+      <c r="N19" s="17" t="inlineStr">
         <is>
           <t>hauntedheist</t>
         </is>
       </c>
-      <c r="N19" s="17" t="inlineStr">
+      <c r="O19" s="17" t="inlineStr">
         <is>
           <t>hauntedheist</t>
-        </is>
-      </c>
-      <c r="O19" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P19" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="20" ht="84" customHeight="1">
       <c r="A20" s="17" t="inlineStr">
         <is>
+          <t>hit-haunted</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
           <t>Hit &amp; Haunted</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Amnesiac Ghost</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="I20" s="17" t="inlineStr">
         <is>
           <t>A murder mystery where you play both the hitman and the victim’s ghost to uncover who ordered the hit.</t>
         </is>
       </c>
-      <c r="I20" s="17" t="inlineStr">
+      <c r="J20" s="17" t="inlineStr">
         <is>
           <t>A top-down murder mystery told from both sides of the same killing. Players alternate between Ace, the hitman, and Eli, the victim's ghost. Their unlikely partnership must uncover who hired Ace and determine the motive behind the contract.</t>
         </is>
       </c>
-      <c r="J20" s="17" t="inlineStr">
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K20" s="17" t="inlineStr">
+      <c r="L20" s="17" t="inlineStr">
         <is>
           <t>3574060</t>
         </is>
       </c>
-      <c r="L20" s="17" t="inlineStr">
+      <c r="M20" s="17" t="inlineStr">
         <is>
           <t>eRlyPFMJ1qs</t>
         </is>
       </c>
-      <c r="M20" s="17" t="inlineStr">
+      <c r="N20" s="17" t="inlineStr">
         <is>
           <t>hithaunted</t>
         </is>
       </c>
-      <c r="N20" s="17" t="inlineStr">
+      <c r="O20" s="17" t="inlineStr">
         <is>
           <t>hithaunted</t>
-        </is>
-      </c>
-      <c r="O20" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P20" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="21" ht="84" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
+          <t>hogen</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
           <t>Hogen</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>Scrappyard Games</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>April 2, 2025</t>
         </is>
       </c>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="I21" s="17" t="inlineStr">
         <is>
           <t>A grid-based card battler where you face Death, craft powerful builds, and uncover what lies behind the game.</t>
         </is>
       </c>
-      <c r="I21" s="17" t="inlineStr">
+      <c r="J21" s="17" t="inlineStr">
         <is>
           <t>A grid-based card battler that begins after the player crosses to the other side and finds Death waiting with a deck. What initially appears to be a simple match may hide something deeper. Strategic positioning, carefully constructed builds, and powerful card combinations determine how far the player gets.</t>
         </is>
       </c>
-      <c r="J21" s="17" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K21" s="17" t="inlineStr">
+      <c r="L21" s="17" t="inlineStr">
         <is>
           <t>3575520</t>
         </is>
       </c>
-      <c r="L21" s="17" t="inlineStr">
+      <c r="M21" s="17" t="inlineStr">
         <is>
           <t>gGKx2EghID8</t>
         </is>
       </c>
-      <c r="M21" s="17" t="inlineStr">
+      <c r="N21" s="17" t="inlineStr">
         <is>
           <t>hogen</t>
         </is>
       </c>
-      <c r="N21" s="17" t="inlineStr">
+      <c r="O21" s="17" t="inlineStr">
         <is>
           <t>hogen</t>
-        </is>
-      </c>
-      <c r="O21" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P21" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="22" ht="84" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
+          <t>hyperfist</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
           <t>HYPERFIST</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>Chirality</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F22" s="17" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
         <is>
           <t>July 10, 2026</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="I22" s="17" t="inlineStr">
         <is>
           <t>Comic-styled first-person action focused on fast, fluid punching, grabbing, and mecha-fist combat.</t>
         </is>
       </c>
-      <c r="I22" s="17" t="inlineStr">
+      <c r="J22" s="17" t="inlineStr">
         <is>
           <t>A fast first-person melee action game presented with a comic-book style. Players control Heath, a local punk equipped with mechanical fists, and fight robotic enemies through a fluid combat system focused on punching, grabbing, and other close-range techniques.</t>
         </is>
       </c>
-      <c r="J22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K22" s="17" t="inlineStr">
+      <c r="L22" s="17" t="inlineStr">
         <is>
           <t>3689210</t>
         </is>
       </c>
-      <c r="L22" s="17" t="inlineStr">
+      <c r="M22" s="17" t="inlineStr">
         <is>
           <t>m-P1E2uCtbM</t>
         </is>
       </c>
-      <c r="M22" s="17" t="inlineStr">
+      <c r="N22" s="17" t="inlineStr">
         <is>
           <t>hyperfist</t>
         </is>
       </c>
-      <c r="N22" s="17" t="inlineStr">
+      <c r="O22" s="17" t="inlineStr">
         <is>
           <t>hyperfist</t>
-        </is>
-      </c>
-      <c r="O22" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P22" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="23" ht="84" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
+          <t>killing-baby-hitler</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
           <t>Killing Baby Hitler</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>The Coffee Industrial Complex</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="F23" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="H23" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and itch.io</t>
         </is>
       </c>
-      <c r="H23" s="17" t="inlineStr">
+      <c r="I23" s="17" t="inlineStr">
         <is>
           <t>A retro FPS through corrupted timelines using resistance art, grenades, dinosaurs, and a wicked guitar.</t>
         </is>
       </c>
-      <c r="I23" s="17" t="inlineStr">
+      <c r="J23" s="17" t="inlineStr">
         <is>
           <t>A retro-inspired first-person shooter about repairing timelines corrupted after a time-travel experiment goes wrong. Players fight fascism across altered versions of history, recover banned art to inspire resistance, throw grenades, ride dinosaurs, and use an extremely loud guitar against Nazi enemies.</t>
         </is>
       </c>
-      <c r="J23" s="17" t="inlineStr">
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K23" s="17" t="inlineStr">
+      <c r="L23" s="17" t="inlineStr">
         <is>
           <t>3317230</t>
         </is>
       </c>
-      <c r="L23" s="17" t="inlineStr">
+      <c r="M23" s="17" t="inlineStr">
         <is>
           <t>p2ENhCALff0</t>
         </is>
       </c>
-      <c r="M23" s="17" t="inlineStr">
+      <c r="N23" s="17" t="inlineStr">
         <is>
           <t>killingbabyhitler</t>
         </is>
       </c>
-      <c r="N23" s="17" t="inlineStr">
+      <c r="O23" s="17" t="inlineStr">
         <is>
           <t>killingbabyhitler</t>
-        </is>
-      </c>
-      <c r="O23" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P23" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="24" ht="84" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
+          <t>knockout-2-wrath-of-the-karen</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
           <t>Knockout 2: Wrath of the Karen</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>ExceptioNULL Games</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>PC, Steam, Mobile</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>Steam, Mobile</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>In development</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="I24" s="17" t="inlineStr">
         <is>
           <t>A comedic boxing adventure where the Federal Boxing Investigations settles every argument in the ring.</t>
         </is>
       </c>
-      <c r="I24" s="17" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
         <is>
           <t>A comedic boxing adventure set in a world where disputes and laws are settled in the ring. The player joins the Federal Boxing Investigations and faces a rising threat to national security, the world, and—perhaps most importantly—the bureau's quarterly performance bonus.</t>
         </is>
       </c>
-      <c r="J24" s="17" t="inlineStr">
+      <c r="K24" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K24" s="17" t="inlineStr">
+      <c r="L24" s="17" t="inlineStr">
         <is>
           <t>2349350</t>
         </is>
       </c>
-      <c r="L24" s="17" t="inlineStr">
+      <c r="M24" s="17" t="inlineStr">
         <is>
           <t>7qiAh0rK458</t>
         </is>
       </c>
-      <c r="M24" s="17" t="inlineStr">
+      <c r="N24" s="17" t="inlineStr">
         <is>
           <t>knockout2wrathofthekaren</t>
         </is>
       </c>
-      <c r="N24" s="17" t="inlineStr">
+      <c r="O24" s="17" t="inlineStr">
         <is>
           <t>knockout2wrathofthekaren</t>
-        </is>
-      </c>
-      <c r="O24" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P24" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="25" ht="84" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
+          <t>malice-in-wonderland</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
           <t>Malice In Wonderland</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>Slyglass Games</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="I25" s="17" t="inlineStr">
         <is>
           <t>A fast action roguelike based on the original Wonderland stories, where time itself is your health.</t>
         </is>
       </c>
-      <c r="I25" s="17" t="inlineStr">
+      <c r="J25" s="17" t="inlineStr">
         <is>
           <t>A fast action roguelike inspired by the original Wonderland stories. The player fights the Hatter while trapped in an endlessly repeating tea time, with remaining time replacing a conventional health bar. Taking damage shortens the clock, failure rewinds the run, and Decrees can combine with existing abilities to create destructive new builds.</t>
         </is>
       </c>
-      <c r="J25" s="17" t="inlineStr">
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K25" s="17" t="inlineStr">
+      <c r="L25" s="17" t="inlineStr">
         <is>
           <t>4552140</t>
         </is>
       </c>
-      <c r="L25" s="17" t="inlineStr">
+      <c r="M25" s="17" t="inlineStr">
         <is>
           <t>PYI_usmMim8</t>
         </is>
       </c>
-      <c r="M25" s="17" t="inlineStr">
+      <c r="N25" s="17" t="inlineStr">
         <is>
           <t>maliceinwonderland</t>
         </is>
       </c>
-      <c r="N25" s="17" t="inlineStr">
+      <c r="O25" s="17" t="inlineStr">
         <is>
           <t>maliceinwonderland</t>
-        </is>
-      </c>
-      <c r="O25" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P25" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="26" ht="84" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
+          <t>manafinder-ii</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
           <t>Manafinder II</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>Wolfsden LLC</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="F26" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="I26" s="17" t="inlineStr">
         <is>
           <t>A console-style turn-based RPG emphasizing party roles, weapon choices, and elemental affinities.</t>
         </is>
       </c>
-      <c r="I26" s="17" t="inlineStr">
+      <c r="J26" s="17" t="inlineStr">
         <is>
           <t>A console-style role-playing game with turn-based battles emphasizing party roles, weapon choices, and elemental relationships. Players travel through varied locations including fungal wilderness, the Luperci town of Alba, and the human ruins of Cuauhtla while confronting beasts, the Purged, and other dangers.</t>
         </is>
       </c>
-      <c r="J26" s="17" t="inlineStr">
+      <c r="K26" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K26" s="17" t="inlineStr">
+      <c r="L26" s="17" t="inlineStr">
         <is>
           <t>4568010</t>
         </is>
       </c>
-      <c r="L26" s="17" t="inlineStr">
+      <c r="M26" s="17" t="inlineStr">
         <is>
           <t>uR8CokKtDYw</t>
         </is>
       </c>
-      <c r="M26" s="17" t="inlineStr">
+      <c r="N26" s="17" t="inlineStr">
         <is>
           <t>manafinderii</t>
         </is>
       </c>
-      <c r="N26" s="17" t="inlineStr">
+      <c r="O26" s="17" t="inlineStr">
         <is>
           <t>manafinderii</t>
-        </is>
-      </c>
-      <c r="O26" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P26" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="27" ht="84" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
+          <t>myriorama</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
           <t>MYRIORAMA</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="C27" s="17" t="inlineStr">
         <is>
           <t>J&amp;K Games</t>
         </is>
       </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E27" s="17" t="inlineStr">
+      <c r="F27" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F27" s="17" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
         <is>
           <t>Coming soon</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H27" s="17" t="inlineStr">
+      <c r="I27" s="17" t="inlineStr">
         <is>
           <t>A stop-motion-styled top-down adventure where players rearrange dungeon rooms to solve puzzles.</t>
         </is>
       </c>
-      <c r="I27" s="17" t="inlineStr">
+      <c r="J27" s="17" t="inlineStr">
         <is>
           <t>A top-down adventure inspired by classic 2D Zelda games, with dungeons that can be rearranged room by room. Moving the dungeon itself becomes the key to solving puzzles and navigating its challenges. Low-frame-rate animation and handcrafted-looking environments give the world the appearance of a living stop-motion diorama.</t>
         </is>
       </c>
-      <c r="J27" s="17" t="inlineStr">
+      <c r="K27" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K27" s="17" t="inlineStr">
+      <c r="L27" s="17" t="inlineStr">
         <is>
           <t>4663150</t>
         </is>
       </c>
-      <c r="L27" s="17" t="inlineStr">
+      <c r="M27" s="17" t="inlineStr">
         <is>
           <t>ubZqNnt4tlo</t>
         </is>
       </c>
-      <c r="M27" s="17" t="inlineStr">
+      <c r="N27" s="17" t="inlineStr">
         <is>
           <t>myriorama</t>
         </is>
       </c>
-      <c r="N27" s="17" t="inlineStr">
+      <c r="O27" s="17" t="inlineStr">
         <is>
           <t>myriorama</t>
-        </is>
-      </c>
-      <c r="O27" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P27" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="28" ht="84" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
+          <t>nightmare-kitchen</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
           <t>Nightmare Kitchen</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>Byteback Studios</t>
         </is>
       </c>
-      <c r="C28" s="17" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F28" s="17" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="I28" s="17" t="inlineStr">
         <is>
           <t>A co-op FPS roguelite where chefs fight monstrous food with ridiculous culinary weapons.</t>
         </is>
       </c>
-      <c r="I28" s="17" t="inlineStr">
+      <c r="J28" s="17" t="inlineStr">
         <is>
           <t>A cooperative first-person roguelite where the food is trying to eat the chefs. Teams explore restaurant-themed dungeons, fight deranged culinary monsters, and wield absurd food-inspired weapons. Between runs, players improve their chefs and rebuild the food court at Tater Hills Mall in preparation for the Food-Pocalypse.</t>
         </is>
       </c>
-      <c r="J28" s="17" t="inlineStr">
+      <c r="K28" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K28" s="17" t="inlineStr">
+      <c r="L28" s="17" t="inlineStr">
         <is>
           <t>3077140</t>
         </is>
       </c>
-      <c r="L28" s="17" t="inlineStr">
+      <c r="M28" s="17" t="inlineStr">
         <is>
           <t>VVkEj57OxVc</t>
         </is>
       </c>
-      <c r="M28" s="17" t="inlineStr">
+      <c r="N28" s="17" t="inlineStr">
         <is>
           <t>nightmarekitchen</t>
         </is>
       </c>
-      <c r="N28" s="17" t="inlineStr">
+      <c r="O28" s="17" t="inlineStr">
         <is>
           <t>nightmarekitchen</t>
-        </is>
-      </c>
-      <c r="O28" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P28" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="29" ht="84" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
+          <t>nimbit-frontier</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
           <t>Nimbit Frontier</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>Megasploot</t>
         </is>
       </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="F29" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F29" s="17" t="inlineStr">
+      <c r="G29" s="17" t="inlineStr">
         <is>
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="H29" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="I29" s="17" t="inlineStr">
         <is>
           <t>A cozy creature-collecting life sim with detailed care, custom habitats, conservation, and roguelite expeditions.</t>
         </is>
       </c>
-      <c r="I29" s="17" t="inlineStr">
+      <c r="J29" s="17" t="inlineStr">
         <is>
           <t>A cozy creature-collecting life simulation with detailed creature care and roguelite exploration. Players raise Nimbits, design comfortable habitats, and venture into the changing Underwild to find rare species. Nurturing, discovery, atmosphere, and conservation are central to the experience.</t>
         </is>
       </c>
-      <c r="J29" s="17" t="inlineStr">
+      <c r="K29" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K29" s="17" t="inlineStr">
+      <c r="L29" s="17" t="inlineStr">
         <is>
           <t>2477710</t>
         </is>
       </c>
-      <c r="L29" s="17" t="inlineStr">
+      <c r="M29" s="17" t="inlineStr">
         <is>
           <t>YJxnDCrTqyM</t>
         </is>
       </c>
-      <c r="M29" s="17" t="inlineStr">
+      <c r="N29" s="17" t="inlineStr">
         <is>
           <t>nimbitfrontier</t>
         </is>
       </c>
-      <c r="N29" s="17" t="inlineStr">
+      <c r="O29" s="17" t="inlineStr">
         <is>
           <t>nimbitfrontier</t>
-        </is>
-      </c>
-      <c r="O29" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P29" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
+          <t>rune-gunner</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
           <t>RUNE GUNNER</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>False Summit</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="F30" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F30" s="17" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H30" s="17" t="inlineStr">
+      <c r="I30" s="17" t="inlineStr">
         <is>
           <t>A 1–4 player co-op roguelite shooter where guns and magic fuse into chaotic, build-breaking runs.</t>
         </is>
       </c>
-      <c r="I30" s="17" t="inlineStr">
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>A cooperative roguelite shooter for one to four players that combines firearms and magic. Classes can be mixed during a run, while stacking major upgrades creates increasingly powerful builds. Teams must survive chaotic encounters across a shattered world occupied by hostile Constructs.</t>
         </is>
       </c>
-      <c r="J30" s="17" t="inlineStr">
+      <c r="K30" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K30" s="17" t="inlineStr">
+      <c r="L30" s="17" t="inlineStr">
         <is>
           <t>3769870</t>
         </is>
       </c>
-      <c r="L30" s="17" t="inlineStr">
+      <c r="M30" s="17" t="inlineStr">
         <is>
           <t>AdDfigLpSjg</t>
         </is>
       </c>
-      <c r="M30" s="17" t="inlineStr">
+      <c r="N30" s="17" t="inlineStr">
         <is>
           <t>runegunner</t>
         </is>
       </c>
-      <c r="N30" s="17" t="inlineStr">
+      <c r="O30" s="17" t="inlineStr">
         <is>
           <t>runegunner</t>
-        </is>
-      </c>
-      <c r="O30" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P30" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="31" ht="84" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
+          <t>scp-antimemetics-division</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
           <t>SCP: Antimemetics Division</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>Quadrant Five</t>
         </is>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>In development</t>
         </is>
       </c>
-      <c r="G31" s="17" t="inlineStr">
+      <c r="H31" s="17" t="inlineStr">
         <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="H31" s="17" t="inlineStr">
+      <c r="I31" s="17" t="inlineStr">
         <is>
           <t>Tactile survival horror inside a locked-down SCP site where memory and reality are dangerous resources.</t>
         </is>
       </c>
-      <c r="I31" s="17" t="inlineStr">
+      <c r="J31" s="17" t="inlineStr">
         <is>
           <t>A tactile survival-horror game set after amnestics have taken effect and Site-48 has gone into lockdown. Players scavenge restricted equipment, earn access to forgotten areas, and manipulate reality while escaping lethal SCP anomalies. Memory itself is dangerous, because understanding too much can be fatal.</t>
         </is>
       </c>
-      <c r="J31" s="17" t="inlineStr">
+      <c r="K31" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K31" s="17" t="inlineStr">
+      <c r="L31" s="17" t="inlineStr">
         <is>
           <t>4385740</t>
         </is>
       </c>
-      <c r="L31" s="17" t="inlineStr">
+      <c r="M31" s="17" t="inlineStr">
         <is>
           <t>3ENXLCf6c2o</t>
         </is>
       </c>
-      <c r="M31" s="17" t="inlineStr">
+      <c r="N31" s="17" t="inlineStr">
         <is>
           <t>scpantimemeticsdivision</t>
         </is>
       </c>
-      <c r="N31" s="17" t="inlineStr">
+      <c r="O31" s="17" t="inlineStr">
         <is>
           <t>scpantimemeticsdivision</t>
-        </is>
-      </c>
-      <c r="O31" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P31" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="32" ht="84" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
+          <t>seedborne-soldiers</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
           <t>Seedborne Soldiers</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
         <is>
           <t>Hat Wobble Games</t>
         </is>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E32" s="17" t="inlineStr">
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F32" s="17" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>June 1, 2026</t>
         </is>
       </c>
-      <c r="G32" s="17" t="inlineStr">
+      <c r="H32" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H32" s="17" t="inlineStr">
+      <c r="I32" s="17" t="inlineStr">
         <is>
           <t>An auto-battler roguelike about growing heroes across time and space and assembling wild synergies.</t>
         </is>
       </c>
-      <c r="I32" s="17" t="inlineStr">
+      <c r="J32" s="17" t="inlineStr">
         <is>
           <t>An auto-battler roguelike about growing a team of heroes drawn from different points in time and space. Players level their recruits, equip new gear, and assemble powerful synergies while searching for an exit from a surreal dreamworld.</t>
         </is>
       </c>
-      <c r="J32" s="17" t="inlineStr">
+      <c r="K32" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K32" s="17" t="inlineStr">
+      <c r="L32" s="17" t="inlineStr">
         <is>
           <t>3039930</t>
         </is>
       </c>
-      <c r="L32" s="17" t="inlineStr">
+      <c r="M32" s="17" t="inlineStr">
         <is>
           <t>ejA_7I6fPTk</t>
         </is>
       </c>
-      <c r="M32" s="17" t="inlineStr">
+      <c r="N32" s="17" t="inlineStr">
         <is>
           <t>seedbornesoldiers</t>
         </is>
       </c>
-      <c r="N32" s="17" t="inlineStr">
+      <c r="O32" s="17" t="inlineStr">
         <is>
           <t>seedbornesoldiers</t>
-        </is>
-      </c>
-      <c r="O32" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P32" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="33" ht="84" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
+          <t>shroomwood</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
           <t>Shroomwood</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>Sporelite Games</t>
         </is>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>PC, Mac, Linux, Steam</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E33" s="17" t="inlineStr">
+      <c r="F33" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F33" s="17" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>Demo and playtest available on Steam</t>
         </is>
       </c>
-      <c r="H33" s="17" t="inlineStr">
+      <c r="I33" s="17" t="inlineStr">
         <is>
           <t>Play a tiny mushroom warrior in a transforming wilderness, mixing melee and ranged weapons.</t>
         </is>
       </c>
-      <c r="I33" s="17" t="inlineStr">
+      <c r="J33" s="17" t="inlineStr">
         <is>
           <t>A run-based action adventure set in a wilderness that changes and transforms. The player controls a small but determined mushroom warrior, combining melee and ranged weapons to battle the forest's peculiar creatures. The shifting environment is designed to make every run feel different.</t>
         </is>
       </c>
-      <c r="J33" s="17" t="inlineStr">
+      <c r="K33" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K33" s="17" t="inlineStr">
+      <c r="L33" s="17" t="inlineStr">
         <is>
           <t>3504020</t>
         </is>
       </c>
-      <c r="L33" s="17" t="inlineStr">
+      <c r="M33" s="17" t="inlineStr">
         <is>
           <t>qZtAtZZIl_w</t>
         </is>
       </c>
-      <c r="M33" s="17" t="inlineStr">
+      <c r="N33" s="17" t="inlineStr">
         <is>
           <t>Martin%20Hundrup</t>
         </is>
       </c>
-      <c r="N33" s="17" t="inlineStr">
+      <c r="O33" s="17" t="inlineStr">
         <is>
           <t>Martin%20Hundrup</t>
-        </is>
-      </c>
-      <c r="O33" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P33" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="34" ht="84" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
+          <t>steel-swarm-survivor</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
           <t>Steel Swarm: SURVIVOR</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>Clay Token Game Studio, Inc.</t>
         </is>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>PC, Linux, Steam</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F34" s="17" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
         <is>
           <t>Coming soon</t>
         </is>
       </c>
-      <c r="G34" s="17" t="inlineStr">
+      <c r="H34" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and itch.io</t>
         </is>
       </c>
-      <c r="H34" s="17" t="inlineStr">
+      <c r="I34" s="17" t="inlineStr">
         <is>
           <t>A fast survivors-like where customizable drone formations overwhelm metal hordes solo or in co-op.</t>
         </is>
       </c>
-      <c r="I34" s="17" t="inlineStr">
+      <c r="J34" s="17" t="inlineStr">
         <is>
           <t>A fast survivors-style roguelite centered on commanding drones against enormous mechanical hordes. Players arrange formations, upgrade individual drones, and refine their setup during each run. Enemy waves can be challenged alone or with other players in cooperative multiplayer.</t>
         </is>
       </c>
-      <c r="J34" s="17" t="inlineStr">
+      <c r="K34" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K34" s="17" t="inlineStr">
+      <c r="L34" s="17" t="inlineStr">
         <is>
           <t>4307100</t>
         </is>
       </c>
-      <c r="L34" s="17" t="inlineStr">
+      <c r="M34" s="17" t="inlineStr">
         <is>
           <t>poEK4BFvMYA</t>
         </is>
       </c>
-      <c r="M34" s="17" t="inlineStr">
+      <c r="N34" s="17" t="inlineStr">
         <is>
           <t>steelswarmsurvivor</t>
         </is>
       </c>
-      <c r="N34" s="17" t="inlineStr">
+      <c r="O34" s="17" t="inlineStr">
         <is>
           <t>steelswarmsurvivor</t>
-        </is>
-      </c>
-      <c r="O34" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P34" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="35" ht="84" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
+          <t>super-choppy</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
           <t>Super Choppy</t>
         </is>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>Sumoshell Bombfunk</t>
         </is>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>PC, Mac, Linux, Steam</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr">
+      <c r="F35" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F35" s="17" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="H35" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and itch.io</t>
         </is>
       </c>
-      <c r="H35" s="17" t="inlineStr">
+      <c r="I35" s="17" t="inlineStr">
         <is>
           <t>A pixel-art action platformer where Choppy uses an axe to throw, fly, climb, and chop.</t>
         </is>
       </c>
-      <c r="I35" s="17" t="inlineStr">
+      <c r="J35" s="17" t="inlineStr">
         <is>
           <t>A challenging action platformer with colorful retro pixel artwork and a deliberately silly revenge story. Choppy's axe is more than a weapon: it supports throwing, flying, climbing, chopping, and the advanced movement required to master each stage.</t>
         </is>
       </c>
-      <c r="J35" s="17" t="inlineStr">
+      <c r="K35" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K35" s="17" t="inlineStr">
+      <c r="L35" s="17" t="inlineStr">
         <is>
           <t>3616860</t>
         </is>
       </c>
-      <c r="L35" s="17" t="inlineStr">
+      <c r="M35" s="17" t="inlineStr">
         <is>
           <t>b6UtITtVuxk</t>
         </is>
       </c>
-      <c r="M35" s="17" t="inlineStr">
+      <c r="N35" s="17" t="inlineStr">
         <is>
           <t>superchoppy</t>
         </is>
       </c>
-      <c r="N35" s="17" t="inlineStr">
+      <c r="O35" s="17" t="inlineStr">
         <is>
           <t>superchoppy</t>
-        </is>
-      </c>
-      <c r="O35" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P35" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="36" ht="84" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
+          <t>telera</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
           <t>Telera</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>Entropico</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="D36" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F36" s="17" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G36" s="17" t="inlineStr">
+      <c r="H36" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="I36" s="17" t="inlineStr">
         <is>
           <t>A roguelike dice-builder about rolling, scoring, upgrading, combining magic items, and out-thinking luck.</t>
         </is>
       </c>
-      <c r="I36" s="17" t="inlineStr">
+      <c r="J36" s="17" t="inlineStr">
         <is>
           <t>A roguelike dice-building game for players who enjoy large scores and calculated risks. Each round involves rolling dice, earning points, and clearing levels; between rounds, players upgrade dice, acquire new ones, and combine magical items. Every run mixes luck, planning, and player choices on the path toward legendary bosses and a new high score.</t>
         </is>
       </c>
-      <c r="J36" s="17" t="inlineStr">
+      <c r="K36" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K36" s="17" t="inlineStr">
+      <c r="L36" s="17" t="inlineStr">
         <is>
           <t>4079370</t>
         </is>
       </c>
-      <c r="L36" s="17" t="inlineStr">
+      <c r="M36" s="17" t="inlineStr">
         <is>
           <t>Qv9GY_9RpGo</t>
         </is>
       </c>
-      <c r="M36" s="17" t="inlineStr">
+      <c r="N36" s="17" t="inlineStr">
         <is>
           <t>telera</t>
         </is>
       </c>
-      <c r="N36" s="17" t="inlineStr">
+      <c r="O36" s="17" t="inlineStr">
         <is>
           <t>telera</t>
-        </is>
-      </c>
-      <c r="O36" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P36" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="37" ht="84" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
+          <t>the-assessment</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
           <t>The Assessment</t>
         </is>
       </c>
-      <c r="B37" s="17" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>Miga Games</t>
         </is>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr">
+      <c r="F37" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F37" s="17" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
         <is>
           <t>Q4 2026</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="H37" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
         <is>
           <t>An archaeologist explores a forgotten castle, performs rituals, releases souls, and confronts corrupted memories.</t>
         </is>
       </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="J37" s="17" t="inlineStr">
         <is>
           <t>A narrative horror game about an archaeologist hired to examine a forgotten castle. The assignment reveals the truth behind human sacrifices sealed within its walls. Players perform rituals, free trapped souls, and experience Gabrielle's most painful memories as the castle's spirits distort them.</t>
         </is>
       </c>
-      <c r="J37" s="17" t="inlineStr">
+      <c r="K37" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K37" s="17" t="inlineStr">
+      <c r="L37" s="17" t="inlineStr">
         <is>
           <t>4081850</t>
         </is>
       </c>
-      <c r="L37" s="17" t="inlineStr">
+      <c r="M37" s="17" t="inlineStr">
         <is>
           <t>JR4hXyOlywQ</t>
         </is>
       </c>
-      <c r="M37" s="17" t="inlineStr">
+      <c r="N37" s="17" t="inlineStr">
         <is>
           <t>theassessment</t>
         </is>
       </c>
-      <c r="N37" s="17" t="inlineStr">
+      <c r="O37" s="17" t="inlineStr">
         <is>
           <t>theassessment</t>
-        </is>
-      </c>
-      <c r="O37" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P37" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="38" ht="84" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
+          <t>tileshire</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
           <t>TileShire</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="C38" s="17" t="inlineStr">
         <is>
           <t>Boss Blob</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>PC, Mac, Steam</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr">
+      <c r="F38" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F38" s="17" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G38" s="17" t="inlineStr">
+      <c r="H38" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H38" s="17" t="inlineStr">
+      <c r="I38" s="17" t="inlineStr">
         <is>
           <t>A minimalist townbuilder where placing and transforming tiles earns points, cards, and townsfolk.</t>
         </is>
       </c>
-      <c r="I38" s="17" t="inlineStr">
+      <c r="J38" s="17" t="inlineStr">
         <is>
           <t>A minimalist town-building game where placing and transforming tiles produces points and expands the settlement. As the shire develops, players draft new cards and recruit townsfolk whose abilities help turn a simple arrangement of tiles into a home filled with life.</t>
         </is>
       </c>
-      <c r="J38" s="17" t="inlineStr">
+      <c r="K38" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K38" s="17" t="inlineStr">
+      <c r="L38" s="17" t="inlineStr">
         <is>
           <t>4370780</t>
         </is>
       </c>
-      <c r="L38" s="17" t="inlineStr">
+      <c r="M38" s="17" t="inlineStr">
         <is>
           <t>C1afDQkrrLg</t>
         </is>
       </c>
-      <c r="M38" s="17" t="inlineStr">
+      <c r="N38" s="17" t="inlineStr">
         <is>
           <t>tileshire</t>
         </is>
       </c>
-      <c r="N38" s="17" t="inlineStr">
+      <c r="O38" s="17" t="inlineStr">
         <is>
           <t>tileshire</t>
-        </is>
-      </c>
-      <c r="O38" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P38" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="39" ht="84" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
+          <t>tower-lab</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
           <t>Tower Lab</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
         <is>
           <t>Play Tug Studio</t>
         </is>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E39" s="17" t="inlineStr">
+      <c r="F39" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F39" s="17" t="inlineStr">
+      <c r="G39" s="17" t="inlineStr">
         <is>
           <t>September 7, 2026</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr">
+      <c r="H39" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H39" s="17" t="inlineStr">
+      <c r="I39" s="17" t="inlineStr">
         <is>
           <t>A physics tower-defense roguelite: shrink, grow, split, and clone objects to push enemies away.</t>
         </is>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="J39" s="17" t="inlineStr">
         <is>
           <t>A physics-driven roguelite tower-defense game where enemies do not use traditional health. Projectiles and units are physical objects that can be enlarged, reduced, duplicated, or divided. Players combine towers into unusual contraptions designed to push entire enemy formations off the level.</t>
         </is>
       </c>
-      <c r="J39" s="17" t="inlineStr">
+      <c r="K39" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K39" s="17" t="inlineStr">
+      <c r="L39" s="17" t="inlineStr">
         <is>
           <t>3084810</t>
         </is>
       </c>
-      <c r="L39" s="17" t="inlineStr">
+      <c r="M39" s="17" t="inlineStr">
         <is>
           <t>FCEoowKglGA</t>
         </is>
       </c>
-      <c r="M39" s="17" t="inlineStr">
+      <c r="N39" s="17" t="inlineStr">
         <is>
           <t>towerlab</t>
         </is>
       </c>
-      <c r="N39" s="17" t="inlineStr">
+      <c r="O39" s="17" t="inlineStr">
         <is>
           <t>towerlab</t>
-        </is>
-      </c>
-      <c r="O39" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P39" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="40" ht="84" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
+          <t>tricky-and-the-dream-caster</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
           <t>Tricky and the Dream Caster</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="C40" s="17" t="inlineStr">
         <is>
           <t>PossQueen</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="D40" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E40" s="17" t="inlineStr">
+      <c r="F40" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F40" s="17" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
         <is>
           <t>Q4 2027</t>
         </is>
       </c>
-      <c r="G40" s="17" t="inlineStr">
+      <c r="H40" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam</t>
         </is>
       </c>
-      <c r="H40" s="17" t="inlineStr">
+      <c r="I40" s="17" t="inlineStr">
         <is>
           <t>A colorful platforming adventure starring Tricky O’Possum and Volt the Mouse on a wizard-punching mission.</t>
         </is>
       </c>
-      <c r="I40" s="17" t="inlineStr">
+      <c r="J40" s="17" t="inlineStr">
         <is>
           <t>A platforming adventure about breaking a curse of eternal sleep by invading the responsible wizard's castle and beating him up. Players control Tricky O'Possum and Volt the Mouse as they run, jump, collect keys, and battle through the Dream Caster's realm on the way to his stronghold.</t>
         </is>
       </c>
-      <c r="J40" s="17" t="inlineStr">
+      <c r="K40" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K40" s="17" t="inlineStr">
+      <c r="L40" s="17" t="inlineStr">
         <is>
           <t>3564580</t>
         </is>
       </c>
-      <c r="L40" s="17" t="inlineStr">
+      <c r="M40" s="17" t="inlineStr">
         <is>
           <t>nzQXQ_nIGFk</t>
         </is>
       </c>
-      <c r="M40" s="17" t="inlineStr">
+      <c r="N40" s="17" t="inlineStr">
         <is>
           <t>trickyandthedreamcaster</t>
         </is>
       </c>
-      <c r="N40" s="17" t="inlineStr">
+      <c r="O40" s="17" t="inlineStr">
         <is>
           <t>trickyandthedreamcaster</t>
-        </is>
-      </c>
-      <c r="O40" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P40" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="41" ht="84" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
+          <t>turning-manor</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
           <t>Turning Manor</t>
         </is>
       </c>
-      <c r="B41" s="17" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
         <is>
           <t>Sabbatical Games</t>
         </is>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E41" s="17" t="inlineStr">
+      <c r="F41" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F41" s="17" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G41" s="17" t="inlineStr">
+      <c r="H41" s="17" t="inlineStr">
         <is>
           <t>Demo available on Steam and itch.io</t>
         </is>
       </c>
-      <c r="H41" s="17" t="inlineStr">
+      <c r="I41" s="17" t="inlineStr">
         <is>
           <t>An anomaly-spotting horror game with no resets, more lore, and leaderboards inside a suspicious workplace.</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="J41" s="17" t="inlineStr">
         <is>
           <t>An anomaly-observation game that begins when unsettling events follow the signing of a new job contract. Players compare rooms and count differences while investigating the mystery of Turning Manor. The design expands the familiar anomaly format with persistent progress, additional story, and leaderboards rather than constant resets.</t>
         </is>
       </c>
-      <c r="J41" s="17" t="inlineStr">
+      <c r="K41" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K41" s="17" t="inlineStr">
+      <c r="L41" s="17" t="inlineStr">
         <is>
           <t>3855530</t>
         </is>
       </c>
-      <c r="L41" s="17" t="inlineStr">
+      <c r="M41" s="17" t="inlineStr">
         <is>
           <t>5JvE5PJ6-Bk</t>
         </is>
       </c>
-      <c r="M41" s="17" t="inlineStr">
+      <c r="N41" s="17" t="inlineStr">
         <is>
           <t>turningmanor</t>
         </is>
       </c>
-      <c r="N41" s="17" t="inlineStr">
+      <c r="O41" s="17" t="inlineStr">
         <is>
           <t>turningmanor</t>
-        </is>
-      </c>
-      <c r="O41" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P41" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="42" ht="84" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
+          <t>we-need-an-army</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
           <t>We Need An Army</t>
         </is>
       </c>
-      <c r="B42" s="17" t="inlineStr">
+      <c r="C42" s="17" t="inlineStr">
         <is>
           <t>Elder Bear Games</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="D42" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="E42" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E42" s="17" t="inlineStr">
+      <c r="F42" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F42" s="17" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>Q4 2026</t>
         </is>
       </c>
-      <c r="G42" s="17" t="inlineStr">
+      <c r="H42" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H42" s="17" t="inlineStr">
+      <c r="I42" s="17" t="inlineStr">
         <is>
           <t>A tactical slots-based roguelike battler about collecting units, finding relics, and shuffling an army.</t>
         </is>
       </c>
-      <c r="I42" s="17" t="inlineStr">
+      <c r="J42" s="17" t="inlineStr">
         <is>
           <t>A tactical, slots-based roguelike battler about constructing the strongest possible army. Players collect units, uncover relics, and complete minigames that affect their forces. Success comes from making good combinations and shuffling the available pieces into a winning formation.</t>
         </is>
       </c>
-      <c r="J42" s="17" t="inlineStr">
+      <c r="K42" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K42" s="17" t="inlineStr">
+      <c r="L42" s="17" t="inlineStr">
         <is>
           <t>3671320</t>
         </is>
       </c>
-      <c r="L42" s="17" t="inlineStr">
+      <c r="M42" s="17" t="inlineStr">
         <is>
           <t>qagBhjgCvs0</t>
         </is>
       </c>
-      <c r="M42" s="17" t="inlineStr">
+      <c r="N42" s="17" t="inlineStr">
         <is>
           <t>weneedanarmy</t>
         </is>
       </c>
-      <c r="N42" s="17" t="inlineStr">
+      <c r="O42" s="17" t="inlineStr">
         <is>
           <t>weneedanarmy</t>
-        </is>
-      </c>
-      <c r="O42" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P42" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="43" ht="84" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
+          <t>will-follow-the-light</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
           <t>WILL: Follow The Light</t>
         </is>
       </c>
-      <c r="B43" s="17" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>TomorrowHead Studio</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>PC, PlayStation, Steam</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>Steam, PlayStation</t>
         </is>
       </c>
-      <c r="E43" s="17" t="inlineStr">
+      <c r="F43" s="17" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F43" s="17" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
         <is>
           <t>May 7, 2026</t>
         </is>
       </c>
-      <c r="G43" s="17" t="inlineStr">
+      <c r="H43" s="17" t="inlineStr">
         <is>
           <t>No public demo currently available</t>
         </is>
       </c>
-      <c r="H43" s="17" t="inlineStr">
+      <c r="I43" s="17" t="inlineStr">
         <is>
           <t>A story-driven first-person adventure puzzle about sailing harsh northern waters to reunite with family.</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="J43" s="17" t="inlineStr">
         <is>
           <t>A story-driven first-person puzzle adventure about a dangerous personal journey through northern waters. Will sails across harsh, isolated landscapes while confronting environmental challenges and puzzles. His voyage is ultimately about finding peace, returning to his family, and understanding himself.</t>
         </is>
       </c>
-      <c r="J43" s="17" t="inlineStr">
+      <c r="K43" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K43" s="17" t="inlineStr">
+      <c r="L43" s="17" t="inlineStr">
         <is>
           <t>3144860</t>
         </is>
       </c>
-      <c r="L43" s="17" t="inlineStr">
+      <c r="M43" s="17" t="inlineStr">
         <is>
           <t>I7Scpm5vRIU</t>
         </is>
       </c>
-      <c r="M43" s="17" t="inlineStr">
+      <c r="N43" s="17" t="inlineStr">
         <is>
           <t>Roman%20Novikov</t>
         </is>
       </c>
-      <c r="N43" s="17" t="inlineStr">
+      <c r="O43" s="17" t="inlineStr">
         <is>
           <t>Roman%20Novikov</t>
-        </is>
-      </c>
-      <c r="O43" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P43" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
     <row r="44" ht="84" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
+          <t>wrestle-story</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
           <t>Wrestle Story</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>Tic Toc Games</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="D44" s="17" t="inlineStr">
         <is>
           <t>PC, Steam</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="E44" s="17" t="inlineStr">
         <is>
           <t>Steam</t>
         </is>
       </c>
-      <c r="E44" s="17" t="inlineStr">
+      <c r="F44" s="17" t="inlineStr">
         <is>
           <t>Not yet released</t>
         </is>
       </c>
-      <c r="F44" s="17" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr">
         <is>
           <t>To be announced</t>
         </is>
       </c>
-      <c r="G44" s="17" t="inlineStr">
+      <c r="H44" s="17" t="inlineStr">
         <is>
           <t>No public demo listed</t>
         </is>
       </c>
-      <c r="H44" s="17" t="inlineStr">
+      <c r="I44" s="17" t="inlineStr">
         <is>
           <t>A smack-talking 3D wrestling RPG about creating a wrestler, building a tag team, and living the story.</t>
         </is>
       </c>
-      <c r="I44" s="17" t="inlineStr">
+      <c r="J44" s="17" t="inlineStr">
         <is>
           <t>A wrestling role-playing adventure filled with hard hits and louder personalities. Players design their own wrestler, assemble a tag team, and explore a large 3D world built around the spectacle and culture of professional wrestling.</t>
         </is>
       </c>
-      <c r="J44" s="17" t="inlineStr">
+      <c r="K44" s="17" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="K44" s="17" t="inlineStr">
+      <c r="L44" s="17" t="inlineStr">
         <is>
           <t>2357610</t>
         </is>
       </c>
-      <c r="L44" s="17" t="inlineStr">
+      <c r="M44" s="17" t="inlineStr">
         <is>
           <t>Pbii7_HpooQ</t>
         </is>
       </c>
-      <c r="M44" s="17" t="inlineStr">
+      <c r="N44" s="17" t="inlineStr">
         <is>
           <t>wrestlestory</t>
         </is>
       </c>
-      <c r="N44" s="17" t="inlineStr">
+      <c r="O44" s="17" t="inlineStr">
         <is>
           <t>wrestlestory</t>
-        </is>
-      </c>
-      <c r="O44" s="17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P44" s="17" t="inlineStr">
-        <is>
-          <t>Verify status</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:P44"/>
+  <autoFilter ref="A3:O44"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update run of show generation
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run of Show" sheetId="1" r:id="Rb6be82ae8a694908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="descriptions" sheetId="2" r:id="R5e5ee9a5346d4199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run of Show" sheetId="1" r:id="R4e23978f9ebc43e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="descriptions" sheetId="2" r:id="Rde4e19047314433c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="10">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,8 +71,55 @@
       <x:color rgb="FFC2410C"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF202028"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFC2410C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF7445C7"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF66616E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5B2B82"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF245477"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF315D26"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -129,8 +176,53 @@
         <x:fgColor rgb="FFFCE4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B1B25"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF30203F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7445C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F2F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEADCF4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F6D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="15">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -178,11 +270,101 @@
         <x:color rgb="FFF4B183"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFDDD9E2"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="34">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -258,6 +440,121 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="16" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="17" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="17" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="18" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="18" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="19" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="20" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -529,1897 +826,2002 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8" customWidth="1"/>
-    <x:col min="2" max="2" width="31" customWidth="1"/>
-    <x:col min="3" max="3" width="28" customWidth="1"/>
-    <x:col min="4" max="4" width="12" customWidth="1"/>
-    <x:col min="5" max="5" width="12" customWidth="1"/>
-    <x:col min="6" max="6" width="11" customWidth="1"/>
-    <x:col min="7" max="7" width="62" customWidth="1"/>
+    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Seattle Indies Expo - SIX 2026 | Run of Show</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Run of Show - Rough Draft</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Host A = TBD | Host B = TBD | Host C = TBD | Host D = TBD | Host E = TBD | Host F = TBD</x:t>
-        </x:is>
-      </x:c>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="34" t="str">
+        <x:v>Seattle Indies Expo - SIX 2026 | Run of Show</x:v>
+      </x:c>
+      <x:c r="B1" s="34"/>
+      <x:c r="C1" s="34"/>
+      <x:c r="D1" s="34"/>
+      <x:c r="E1" s="34"/>
+      <x:c r="F1" s="34"/>
+      <x:c r="G1" s="34"/>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>Run of Show - Production Schedule</x:v>
+      </x:c>
+      <x:c r="B2" s="36"/>
+      <x:c r="C2" s="36"/>
+      <x:c r="D2" s="36"/>
+      <x:c r="E2" s="36"/>
+      <x:c r="F2" s="36"/>
+      <x:c r="G2" s="36"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="38" t="str">
+        <x:v>Host A = Stephazoid | Host B = AbdallahSmash | Host C = MacnCheesep1z | Host D = Rockagoth | Host E = AlchemistJoker</x:v>
+      </x:c>
+      <x:c r="B3" s="39"/>
+      <x:c r="C3" s="39"/>
+      <x:c r="D3" s="39"/>
+      <x:c r="E3" s="39"/>
+      <x:c r="F3" s="39"/>
+      <x:c r="G3" s="39"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SEG</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GAME / BREAK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEVELOPER / PUBLISHER</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">START</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">END</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" s="9" t="str">
+      <x:c r="A4" s="41" t="str">
+        <x:v>SEG</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>GAME / BREAK</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>DEVELOPER / PUBLISHER</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>START</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>END</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="str">
         <x:v>HOST</x:v>
       </x:c>
-      <x:c r="G4" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PRODUCTION NOTES</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="33" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B5" s="33" t="str">
+      <x:c r="G4" s="41" t="str">
+        <x:v>PRODUCTION NOTES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="20" customHeight="1">
+      <x:c r="A5" s="53" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B5" s="56" t="str">
         <x:v>SIX Hype Hour</x:v>
       </x:c>
-      <x:c r="C5" s="33" t="str">
+      <x:c r="C5" s="54" t="str">
         <x:v>Seattle Indies</x:v>
       </x:c>
-      <x:c r="D5" s="33" t="str">
+      <x:c r="D5" s="54" t="str">
         <x:v>10:00 AM</x:v>
       </x:c>
-      <x:c r="E5" s="33" t="str">
+      <x:c r="E5" s="54" t="str">
         <x:v>12:00 PM</x:v>
       </x:c>
-      <x:c r="F5" s="33" t="str">
+      <x:c r="F5" s="54" t="str">
         <x:v>Prerecorded</x:v>
       </x:c>
-      <x:c r="G5" s="33"/>
-    </x:row>
-    <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="21" t="str">
+      <x:c r="G5" s="55" t="str"/>
+    </x:row>
+    <x:row r="6" ht="20" customHeight="1">
+      <x:c r="A6" s="57" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="22" t="str">
-        <x:v>Opening / Welcome to SIX 2026</x:v>
-      </x:c>
-      <x:c r="C6" s="21" t="str">
+      <x:c r="B6" s="60" t="str">
+        <x:v>Tricky and the Dream Caster</x:v>
+      </x:c>
+      <x:c r="C6" s="58" t="str">
+        <x:v>PossQueen · Booth L27</x:v>
+      </x:c>
+      <x:c r="D6" s="58" t="str">
+        <x:v>12:00 PM</x:v>
+      </x:c>
+      <x:c r="E6" s="58" t="str">
+        <x:v>12:06 PM</x:v>
+      </x:c>
+      <x:c r="F6" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G6" s="59" t="str"/>
+    </x:row>
+    <x:row r="7" ht="20" customHeight="1">
+      <x:c r="A7" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B7" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C7" s="62" t="str">
+        <x:v>Block A</x:v>
+      </x:c>
+      <x:c r="D7" s="62" t="str">
+        <x:v>12:06 PM</x:v>
+      </x:c>
+      <x:c r="E7" s="62" t="str">
+        <x:v>12:07 PM</x:v>
+      </x:c>
+      <x:c r="F7" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G7" s="63" t="str"/>
+    </x:row>
+    <x:row r="8" ht="20" customHeight="1">
+      <x:c r="A8" s="57" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="60" t="str">
+        <x:v>TileShire</x:v>
+      </x:c>
+      <x:c r="C8" s="58" t="str">
+        <x:v>Boss Blob · Booth L28</x:v>
+      </x:c>
+      <x:c r="D8" s="58" t="str">
+        <x:v>12:07 PM</x:v>
+      </x:c>
+      <x:c r="E8" s="58" t="str">
+        <x:v>12:13 PM</x:v>
+      </x:c>
+      <x:c r="F8" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G8" s="59" t="str"/>
+    </x:row>
+    <x:row r="9" ht="20" customHeight="1">
+      <x:c r="A9" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B9" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C9" s="62" t="str">
+        <x:v>Block A</x:v>
+      </x:c>
+      <x:c r="D9" s="62" t="str">
+        <x:v>12:13 PM</x:v>
+      </x:c>
+      <x:c r="E9" s="62" t="str">
+        <x:v>12:14 PM</x:v>
+      </x:c>
+      <x:c r="F9" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G9" s="63" t="str"/>
+    </x:row>
+    <x:row r="10" ht="20" customHeight="1">
+      <x:c r="A10" s="57" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B10" s="60" t="str">
+        <x:v>Wrestle Story</x:v>
+      </x:c>
+      <x:c r="C10" s="58" t="str">
+        <x:v>Tic Toc Games · Booth L29</x:v>
+      </x:c>
+      <x:c r="D10" s="58" t="str">
+        <x:v>12:14 PM</x:v>
+      </x:c>
+      <x:c r="E10" s="58" t="str">
+        <x:v>12:20 PM</x:v>
+      </x:c>
+      <x:c r="F10" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G10" s="59" t="str"/>
+    </x:row>
+    <x:row r="11" ht="20" customHeight="1">
+      <x:c r="A11" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B11" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C11" s="62" t="str">
+        <x:v>Block A</x:v>
+      </x:c>
+      <x:c r="D11" s="62" t="str">
+        <x:v>12:20 PM</x:v>
+      </x:c>
+      <x:c r="E11" s="62" t="str">
+        <x:v>12:21 PM</x:v>
+      </x:c>
+      <x:c r="F11" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G11" s="63" t="str"/>
+    </x:row>
+    <x:row r="12" ht="20" customHeight="1">
+      <x:c r="A12" s="57" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B12" s="60" t="str">
+        <x:v>Breach Of Contract</x:v>
+      </x:c>
+      <x:c r="C12" s="58" t="str">
+        <x:v>Fern Sprout Studios · Booth L30</x:v>
+      </x:c>
+      <x:c r="D12" s="58" t="str">
+        <x:v>12:21 PM</x:v>
+      </x:c>
+      <x:c r="E12" s="58" t="str">
+        <x:v>12:27 PM</x:v>
+      </x:c>
+      <x:c r="F12" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G12" s="59" t="str"/>
+    </x:row>
+    <x:row r="13" ht="20" customHeight="1">
+      <x:c r="A13" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B13" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C13" s="62" t="str">
+        <x:v>Block A</x:v>
+      </x:c>
+      <x:c r="D13" s="62" t="str">
+        <x:v>12:27 PM</x:v>
+      </x:c>
+      <x:c r="E13" s="62" t="str">
+        <x:v>12:28 PM</x:v>
+      </x:c>
+      <x:c r="F13" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G13" s="63" t="str"/>
+    </x:row>
+    <x:row r="14" ht="20" customHeight="1">
+      <x:c r="A14" s="57" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B14" s="60" t="str">
+        <x:v>Dungeon Bodega Simulator</x:v>
+      </x:c>
+      <x:c r="C14" s="58" t="str">
+        <x:v>Alien Fruit Games · Booth L31</x:v>
+      </x:c>
+      <x:c r="D14" s="58" t="str">
+        <x:v>12:28 PM</x:v>
+      </x:c>
+      <x:c r="E14" s="58" t="str">
+        <x:v>12:34 PM</x:v>
+      </x:c>
+      <x:c r="F14" s="58" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G14" s="59" t="str"/>
+    </x:row>
+    <x:row r="15" ht="20" customHeight="1">
+      <x:c r="A15" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C15" s="62" t="str">
+        <x:v>Block A</x:v>
+      </x:c>
+      <x:c r="D15" s="62" t="str">
+        <x:v>12:34 PM</x:v>
+      </x:c>
+      <x:c r="E15" s="62" t="str">
+        <x:v>12:35 PM</x:v>
+      </x:c>
+      <x:c r="F15" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G15" s="63" t="str"/>
+    </x:row>
+    <x:row r="16" ht="20" customHeight="1">
+      <x:c r="A16" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B16" s="68" t="str">
+        <x:v>DigiPen Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C16" s="66" t="str">
+        <x:v>Sponsor segment · L01</x:v>
+      </x:c>
+      <x:c r="D16" s="66" t="str">
+        <x:v>12:35 PM</x:v>
+      </x:c>
+      <x:c r="E16" s="66" t="str">
+        <x:v>12:45 PM</x:v>
+      </x:c>
+      <x:c r="F16" s="66" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G16" s="67" t="str"/>
+    </x:row>
+    <x:row r="17" ht="20" customHeight="1">
+      <x:c r="A17" s="57" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B17" s="60" t="str">
+        <x:v>SCP: Antimemetics Division</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>Quadrant Five · Booth L22</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="str">
+        <x:v>12:45 PM</x:v>
+      </x:c>
+      <x:c r="E17" s="58" t="str">
+        <x:v>12:51 PM</x:v>
+      </x:c>
+      <x:c r="F17" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G17" s="59" t="str"/>
+    </x:row>
+    <x:row r="18" ht="20" customHeight="1">
+      <x:c r="A18" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B18" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C18" s="62" t="str">
+        <x:v>Block B</x:v>
+      </x:c>
+      <x:c r="D18" s="62" t="str">
+        <x:v>12:51 PM</x:v>
+      </x:c>
+      <x:c r="E18" s="62" t="str">
+        <x:v>12:52 PM</x:v>
+      </x:c>
+      <x:c r="F18" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G18" s="63" t="str"/>
+    </x:row>
+    <x:row r="19" ht="20" customHeight="1">
+      <x:c r="A19" s="57" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B19" s="60" t="str">
+        <x:v>Manafinder II</x:v>
+      </x:c>
+      <x:c r="C19" s="58" t="str">
+        <x:v>Wolfsden LLC · Booth L23</x:v>
+      </x:c>
+      <x:c r="D19" s="58" t="str">
+        <x:v>12:52 PM</x:v>
+      </x:c>
+      <x:c r="E19" s="58" t="str">
+        <x:v>12:58 PM</x:v>
+      </x:c>
+      <x:c r="F19" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G19" s="59" t="str"/>
+    </x:row>
+    <x:row r="20" ht="20" customHeight="1">
+      <x:c r="A20" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B20" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C20" s="62" t="str">
+        <x:v>Block B</x:v>
+      </x:c>
+      <x:c r="D20" s="62" t="str">
+        <x:v>12:58 PM</x:v>
+      </x:c>
+      <x:c r="E20" s="62" t="str">
+        <x:v>12:59 PM</x:v>
+      </x:c>
+      <x:c r="F20" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G20" s="63" t="str"/>
+    </x:row>
+    <x:row r="21" ht="20" customHeight="1">
+      <x:c r="A21" s="57" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B21" s="60" t="str">
+        <x:v>Malice In Wonderland</x:v>
+      </x:c>
+      <x:c r="C21" s="58" t="str">
+        <x:v>Slyglass Games · Booth L24</x:v>
+      </x:c>
+      <x:c r="D21" s="58" t="str">
+        <x:v>12:59 PM</x:v>
+      </x:c>
+      <x:c r="E21" s="58" t="str">
+        <x:v>1:05 PM</x:v>
+      </x:c>
+      <x:c r="F21" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G21" s="59" t="str"/>
+    </x:row>
+    <x:row r="22" ht="20" customHeight="1">
+      <x:c r="A22" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B22" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C22" s="62" t="str">
+        <x:v>Block B</x:v>
+      </x:c>
+      <x:c r="D22" s="62" t="str">
+        <x:v>1:05 PM</x:v>
+      </x:c>
+      <x:c r="E22" s="62" t="str">
+        <x:v>1:06 PM</x:v>
+      </x:c>
+      <x:c r="F22" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G22" s="63" t="str"/>
+    </x:row>
+    <x:row r="23" ht="20" customHeight="1">
+      <x:c r="A23" s="57" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B23" s="60" t="str">
+        <x:v>Project Cradle</x:v>
+      </x:c>
+      <x:c r="C23" s="58" t="str">
+        <x:v>ShazySoft · Booth L25</x:v>
+      </x:c>
+      <x:c r="D23" s="58" t="str">
+        <x:v>1:06 PM</x:v>
+      </x:c>
+      <x:c r="E23" s="58" t="str">
+        <x:v>1:12 PM</x:v>
+      </x:c>
+      <x:c r="F23" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G23" s="59" t="str"/>
+    </x:row>
+    <x:row r="24" ht="20" customHeight="1">
+      <x:c r="A24" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B24" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C24" s="62" t="str">
+        <x:v>Block B</x:v>
+      </x:c>
+      <x:c r="D24" s="62" t="str">
+        <x:v>1:12 PM</x:v>
+      </x:c>
+      <x:c r="E24" s="62" t="str">
+        <x:v>1:13 PM</x:v>
+      </x:c>
+      <x:c r="F24" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G24" s="63" t="str"/>
+    </x:row>
+    <x:row r="25" ht="20" customHeight="1">
+      <x:c r="A25" s="57" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B25" s="60" t="str">
+        <x:v>Diabolocracy</x:v>
+      </x:c>
+      <x:c r="C25" s="58" t="str">
+        <x:v>Chaos Gremlin Games · Booth L26</x:v>
+      </x:c>
+      <x:c r="D25" s="58" t="str">
+        <x:v>1:13 PM</x:v>
+      </x:c>
+      <x:c r="E25" s="58" t="str">
+        <x:v>1:19 PM</x:v>
+      </x:c>
+      <x:c r="F25" s="58" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G25" s="59" t="str"/>
+    </x:row>
+    <x:row r="26" ht="20" customHeight="1">
+      <x:c r="A26" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B26" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C26" s="62" t="str">
+        <x:v>Block B</x:v>
+      </x:c>
+      <x:c r="D26" s="62" t="str">
+        <x:v>1:19 PM</x:v>
+      </x:c>
+      <x:c r="E26" s="62" t="str">
+        <x:v>1:20 PM</x:v>
+      </x:c>
+      <x:c r="F26" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G26" s="63" t="str"/>
+    </x:row>
+    <x:row r="27" ht="20" customHeight="1">
+      <x:c r="A27" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B27" s="68" t="str">
+        <x:v>AIE Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C27" s="66" t="str">
+        <x:v>Sponsor segment · L02</x:v>
+      </x:c>
+      <x:c r="D27" s="66" t="str">
+        <x:v>1:20 PM</x:v>
+      </x:c>
+      <x:c r="E27" s="66" t="str">
+        <x:v>1:30 PM</x:v>
+      </x:c>
+      <x:c r="F27" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G27" s="67" t="str"/>
+    </x:row>
+    <x:row r="28" ht="20" customHeight="1">
+      <x:c r="A28" s="57" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B28" s="60" t="str">
+        <x:v>Seedborne Soldiers</x:v>
+      </x:c>
+      <x:c r="C28" s="58" t="str">
+        <x:v>Hat Wobble Games · Booth L17</x:v>
+      </x:c>
+      <x:c r="D28" s="58" t="str">
+        <x:v>1:30 PM</x:v>
+      </x:c>
+      <x:c r="E28" s="58" t="str">
+        <x:v>1:36 PM</x:v>
+      </x:c>
+      <x:c r="F28" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G28" s="59" t="str"/>
+    </x:row>
+    <x:row r="29" ht="20" customHeight="1">
+      <x:c r="A29" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B29" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C29" s="62" t="str">
+        <x:v>Block C</x:v>
+      </x:c>
+      <x:c r="D29" s="62" t="str">
+        <x:v>1:36 PM</x:v>
+      </x:c>
+      <x:c r="E29" s="62" t="str">
+        <x:v>1:37 PM</x:v>
+      </x:c>
+      <x:c r="F29" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G29" s="63" t="str"/>
+    </x:row>
+    <x:row r="30" ht="20" customHeight="1">
+      <x:c r="A30" s="57" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B30" s="60" t="str">
+        <x:v>Super Choppy</x:v>
+      </x:c>
+      <x:c r="C30" s="58" t="str">
+        <x:v>Sumoshell Bombfunk · Booth L18</x:v>
+      </x:c>
+      <x:c r="D30" s="58" t="str">
+        <x:v>1:37 PM</x:v>
+      </x:c>
+      <x:c r="E30" s="58" t="str">
+        <x:v>1:43 PM</x:v>
+      </x:c>
+      <x:c r="F30" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G30" s="59" t="str"/>
+    </x:row>
+    <x:row r="31" ht="20" customHeight="1">
+      <x:c r="A31" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B31" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C31" s="62" t="str">
+        <x:v>Block C</x:v>
+      </x:c>
+      <x:c r="D31" s="62" t="str">
+        <x:v>1:43 PM</x:v>
+      </x:c>
+      <x:c r="E31" s="62" t="str">
+        <x:v>1:44 PM</x:v>
+      </x:c>
+      <x:c r="F31" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G31" s="63" t="str"/>
+    </x:row>
+    <x:row r="32" ht="20" customHeight="1">
+      <x:c r="A32" s="57" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B32" s="60" t="str">
+        <x:v>Dig Too Deep</x:v>
+      </x:c>
+      <x:c r="C32" s="58" t="str">
+        <x:v>Punch Up Games · Booth L19</x:v>
+      </x:c>
+      <x:c r="D32" s="58" t="str">
+        <x:v>1:44 PM</x:v>
+      </x:c>
+      <x:c r="E32" s="58" t="str">
+        <x:v>1:50 PM</x:v>
+      </x:c>
+      <x:c r="F32" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G32" s="59" t="str"/>
+    </x:row>
+    <x:row r="33" ht="20" customHeight="1">
+      <x:c r="A33" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B33" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C33" s="62" t="str">
+        <x:v>Block C</x:v>
+      </x:c>
+      <x:c r="D33" s="62" t="str">
+        <x:v>1:50 PM</x:v>
+      </x:c>
+      <x:c r="E33" s="62" t="str">
+        <x:v>1:51 PM</x:v>
+      </x:c>
+      <x:c r="F33" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G33" s="63" t="str"/>
+    </x:row>
+    <x:row r="34" ht="20" customHeight="1">
+      <x:c r="A34" s="57" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B34" s="60" t="str">
+        <x:v>Nimbit Frontier</x:v>
+      </x:c>
+      <x:c r="C34" s="58" t="str">
+        <x:v>Megasploot · Booth L20</x:v>
+      </x:c>
+      <x:c r="D34" s="58" t="str">
+        <x:v>1:51 PM</x:v>
+      </x:c>
+      <x:c r="E34" s="58" t="str">
+        <x:v>1:57 PM</x:v>
+      </x:c>
+      <x:c r="F34" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G34" s="59" t="str"/>
+    </x:row>
+    <x:row r="35" ht="20" customHeight="1">
+      <x:c r="A35" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B35" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C35" s="62" t="str">
+        <x:v>Block C</x:v>
+      </x:c>
+      <x:c r="D35" s="62" t="str">
+        <x:v>1:57 PM</x:v>
+      </x:c>
+      <x:c r="E35" s="62" t="str">
+        <x:v>1:58 PM</x:v>
+      </x:c>
+      <x:c r="F35" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G35" s="63" t="str"/>
+    </x:row>
+    <x:row r="36" ht="20" customHeight="1">
+      <x:c r="A36" s="57" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B36" s="60" t="str">
+        <x:v>We Need An Army</x:v>
+      </x:c>
+      <x:c r="C36" s="58" t="str">
+        <x:v>Elder Bear Games · Booth L21</x:v>
+      </x:c>
+      <x:c r="D36" s="58" t="str">
+        <x:v>1:58 PM</x:v>
+      </x:c>
+      <x:c r="E36" s="58" t="str">
+        <x:v>2:04 PM</x:v>
+      </x:c>
+      <x:c r="F36" s="58" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G36" s="59" t="str"/>
+    </x:row>
+    <x:row r="37" ht="20" customHeight="1">
+      <x:c r="A37" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B37" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C37" s="62" t="str">
+        <x:v>Block C</x:v>
+      </x:c>
+      <x:c r="D37" s="62" t="str">
+        <x:v>2:04 PM</x:v>
+      </x:c>
+      <x:c r="E37" s="62" t="str">
+        <x:v>2:05 PM</x:v>
+      </x:c>
+      <x:c r="F37" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G37" s="63" t="str"/>
+    </x:row>
+    <x:row r="38" ht="20" customHeight="1">
+      <x:c r="A38" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B38" s="68" t="str">
+        <x:v>Unity Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C38" s="66" t="str">
+        <x:v>Sponsor segment · L03</x:v>
+      </x:c>
+      <x:c r="D38" s="66" t="str">
+        <x:v>2:05 PM</x:v>
+      </x:c>
+      <x:c r="E38" s="66" t="str">
+        <x:v>2:15 PM</x:v>
+      </x:c>
+      <x:c r="F38" s="66" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G38" s="67" t="str"/>
+    </x:row>
+    <x:row r="39" ht="20" customHeight="1">
+      <x:c r="A39" s="57" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B39" s="60" t="str">
+        <x:v>Feeding Gooble</x:v>
+      </x:c>
+      <x:c r="C39" s="58" t="str">
+        <x:v>Displacer Labs · Booth L12</x:v>
+      </x:c>
+      <x:c r="D39" s="58" t="str">
+        <x:v>2:15 PM</x:v>
+      </x:c>
+      <x:c r="E39" s="58" t="str">
+        <x:v>2:21 PM</x:v>
+      </x:c>
+      <x:c r="F39" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G39" s="59" t="str"/>
+    </x:row>
+    <x:row r="40" ht="20" customHeight="1">
+      <x:c r="A40" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B40" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C40" s="62" t="str">
+        <x:v>Block D</x:v>
+      </x:c>
+      <x:c r="D40" s="62" t="str">
+        <x:v>2:21 PM</x:v>
+      </x:c>
+      <x:c r="E40" s="62" t="str">
+        <x:v>2:22 PM</x:v>
+      </x:c>
+      <x:c r="F40" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G40" s="63" t="str"/>
+    </x:row>
+    <x:row r="41" ht="20" customHeight="1">
+      <x:c r="A41" s="57" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B41" s="60" t="str">
+        <x:v>BroomSweeper</x:v>
+      </x:c>
+      <x:c r="C41" s="58" t="str">
+        <x:v>BandWidth Games · Booth L13</x:v>
+      </x:c>
+      <x:c r="D41" s="58" t="str">
+        <x:v>2:22 PM</x:v>
+      </x:c>
+      <x:c r="E41" s="58" t="str">
+        <x:v>2:28 PM</x:v>
+      </x:c>
+      <x:c r="F41" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G41" s="59" t="str"/>
+    </x:row>
+    <x:row r="42" ht="20" customHeight="1">
+      <x:c r="A42" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B42" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C42" s="62" t="str">
+        <x:v>Block D</x:v>
+      </x:c>
+      <x:c r="D42" s="62" t="str">
+        <x:v>2:28 PM</x:v>
+      </x:c>
+      <x:c r="E42" s="62" t="str">
+        <x:v>2:29 PM</x:v>
+      </x:c>
+      <x:c r="F42" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G42" s="63" t="str"/>
+    </x:row>
+    <x:row r="43" ht="20" customHeight="1">
+      <x:c r="A43" s="57" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B43" s="60" t="str">
+        <x:v>Fairy Circle</x:v>
+      </x:c>
+      <x:c r="C43" s="58" t="str">
+        <x:v>Play Hooky · Booth L14</x:v>
+      </x:c>
+      <x:c r="D43" s="58" t="str">
+        <x:v>2:29 PM</x:v>
+      </x:c>
+      <x:c r="E43" s="58" t="str">
+        <x:v>2:35 PM</x:v>
+      </x:c>
+      <x:c r="F43" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G43" s="59" t="str"/>
+    </x:row>
+    <x:row r="44" ht="20" customHeight="1">
+      <x:c r="A44" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B44" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C44" s="62" t="str">
+        <x:v>Block D</x:v>
+      </x:c>
+      <x:c r="D44" s="62" t="str">
+        <x:v>2:35 PM</x:v>
+      </x:c>
+      <x:c r="E44" s="62" t="str">
+        <x:v>2:36 PM</x:v>
+      </x:c>
+      <x:c r="F44" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G44" s="63" t="str"/>
+    </x:row>
+    <x:row r="45" ht="20" customHeight="1">
+      <x:c r="A45" s="57" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B45" s="60" t="str">
+        <x:v>MYRIORAMA</x:v>
+      </x:c>
+      <x:c r="C45" s="58" t="str">
+        <x:v>J&amp;K Games · Booth L15</x:v>
+      </x:c>
+      <x:c r="D45" s="58" t="str">
+        <x:v>2:36 PM</x:v>
+      </x:c>
+      <x:c r="E45" s="58" t="str">
+        <x:v>2:42 PM</x:v>
+      </x:c>
+      <x:c r="F45" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G45" s="59" t="str"/>
+    </x:row>
+    <x:row r="46" ht="20" customHeight="1">
+      <x:c r="A46" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B46" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C46" s="62" t="str">
+        <x:v>Block D</x:v>
+      </x:c>
+      <x:c r="D46" s="62" t="str">
+        <x:v>2:42 PM</x:v>
+      </x:c>
+      <x:c r="E46" s="62" t="str">
+        <x:v>2:43 PM</x:v>
+      </x:c>
+      <x:c r="F46" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G46" s="63" t="str"/>
+    </x:row>
+    <x:row r="47" ht="20" customHeight="1">
+      <x:c r="A47" s="57" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B47" s="60" t="str">
+        <x:v>Dittori</x:v>
+      </x:c>
+      <x:c r="C47" s="58" t="str">
+        <x:v>Blookerstein · Booth L16</x:v>
+      </x:c>
+      <x:c r="D47" s="58" t="str">
+        <x:v>2:43 PM</x:v>
+      </x:c>
+      <x:c r="E47" s="58" t="str">
+        <x:v>2:49 PM</x:v>
+      </x:c>
+      <x:c r="F47" s="58" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G47" s="59" t="str"/>
+    </x:row>
+    <x:row r="48" ht="20" customHeight="1">
+      <x:c r="A48" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B48" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C48" s="62" t="str">
+        <x:v>Block D</x:v>
+      </x:c>
+      <x:c r="D48" s="62" t="str">
+        <x:v>2:49 PM</x:v>
+      </x:c>
+      <x:c r="E48" s="62" t="str">
+        <x:v>2:50 PM</x:v>
+      </x:c>
+      <x:c r="F48" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G48" s="63" t="str"/>
+    </x:row>
+    <x:row r="49" ht="20" customHeight="1">
+      <x:c r="A49" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B49" s="68" t="str">
+        <x:v>Forge Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C49" s="66" t="str">
+        <x:v>Sponsor segment · L05</x:v>
+      </x:c>
+      <x:c r="D49" s="66" t="str">
+        <x:v>2:50 PM</x:v>
+      </x:c>
+      <x:c r="E49" s="66" t="str">
+        <x:v>3:00 PM</x:v>
+      </x:c>
+      <x:c r="F49" s="66" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G49" s="67" t="str"/>
+    </x:row>
+    <x:row r="50" ht="20" customHeight="1">
+      <x:c r="A50" s="57" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B50" s="60" t="str">
+        <x:v>End of Garbage</x:v>
+      </x:c>
+      <x:c r="C50" s="58" t="str">
+        <x:v>Joshua Rosen (Rakelock LLC) · Booth L35</x:v>
+      </x:c>
+      <x:c r="D50" s="58" t="str">
+        <x:v>3:00 PM</x:v>
+      </x:c>
+      <x:c r="E50" s="58" t="str">
+        <x:v>3:06 PM</x:v>
+      </x:c>
+      <x:c r="F50" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G50" s="59" t="str"/>
+    </x:row>
+    <x:row r="51" ht="20" customHeight="1">
+      <x:c r="A51" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B51" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C51" s="62" t="str">
+        <x:v>Block E</x:v>
+      </x:c>
+      <x:c r="D51" s="62" t="str">
+        <x:v>3:06 PM</x:v>
+      </x:c>
+      <x:c r="E51" s="62" t="str">
+        <x:v>3:07 PM</x:v>
+      </x:c>
+      <x:c r="F51" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G51" s="63" t="str"/>
+    </x:row>
+    <x:row r="52" ht="20" customHeight="1">
+      <x:c r="A52" s="57" t="str">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B52" s="60" t="str">
+        <x:v>Gravity Goblins</x:v>
+      </x:c>
+      <x:c r="C52" s="58" t="str">
+        <x:v>The Rat Zone · Booth L34</x:v>
+      </x:c>
+      <x:c r="D52" s="58" t="str">
+        <x:v>3:07 PM</x:v>
+      </x:c>
+      <x:c r="E52" s="58" t="str">
+        <x:v>3:13 PM</x:v>
+      </x:c>
+      <x:c r="F52" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G52" s="59" t="str"/>
+    </x:row>
+    <x:row r="53" ht="20" customHeight="1">
+      <x:c r="A53" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B53" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C53" s="62" t="str">
+        <x:v>Block E</x:v>
+      </x:c>
+      <x:c r="D53" s="62" t="str">
+        <x:v>3:13 PM</x:v>
+      </x:c>
+      <x:c r="E53" s="62" t="str">
+        <x:v>3:14 PM</x:v>
+      </x:c>
+      <x:c r="F53" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G53" s="63" t="str"/>
+    </x:row>
+    <x:row r="54" ht="20" customHeight="1">
+      <x:c r="A54" s="57" t="str">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B54" s="60" t="str">
+        <x:v>Creature Kitchen</x:v>
+      </x:c>
+      <x:c r="C54" s="58" t="str">
+        <x:v>The Rat Zone · Booth L33</x:v>
+      </x:c>
+      <x:c r="D54" s="58" t="str">
+        <x:v>3:14 PM</x:v>
+      </x:c>
+      <x:c r="E54" s="58" t="str">
+        <x:v>3:20 PM</x:v>
+      </x:c>
+      <x:c r="F54" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G54" s="59" t="str"/>
+    </x:row>
+    <x:row r="55" ht="20" customHeight="1">
+      <x:c r="A55" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B55" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C55" s="62" t="str">
+        <x:v>Block E</x:v>
+      </x:c>
+      <x:c r="D55" s="62" t="str">
+        <x:v>3:20 PM</x:v>
+      </x:c>
+      <x:c r="E55" s="62" t="str">
+        <x:v>3:21 PM</x:v>
+      </x:c>
+      <x:c r="F55" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G55" s="63" t="str"/>
+    </x:row>
+    <x:row r="56" ht="20" customHeight="1">
+      <x:c r="A56" s="57" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B56" s="60" t="str">
+        <x:v>Desolus</x:v>
+      </x:c>
+      <x:c r="C56" s="58" t="str">
+        <x:v>Mark J. Mayers · Booth L32</x:v>
+      </x:c>
+      <x:c r="D56" s="58" t="str">
+        <x:v>3:21 PM</x:v>
+      </x:c>
+      <x:c r="E56" s="58" t="str">
+        <x:v>3:27 PM</x:v>
+      </x:c>
+      <x:c r="F56" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G56" s="59" t="str"/>
+    </x:row>
+    <x:row r="57" ht="20" customHeight="1">
+      <x:c r="A57" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B57" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C57" s="62" t="str">
+        <x:v>Block E</x:v>
+      </x:c>
+      <x:c r="D57" s="62" t="str">
+        <x:v>3:27 PM</x:v>
+      </x:c>
+      <x:c r="E57" s="62" t="str">
+        <x:v>3:28 PM</x:v>
+      </x:c>
+      <x:c r="F57" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G57" s="63" t="str"/>
+    </x:row>
+    <x:row r="58" ht="20" customHeight="1">
+      <x:c r="A58" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B58" s="68" t="str">
+        <x:v>GeekGirlCon Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C58" s="66" t="str">
+        <x:v>Sponsor segment · L04</x:v>
+      </x:c>
+      <x:c r="D58" s="66" t="str">
+        <x:v>3:28 PM</x:v>
+      </x:c>
+      <x:c r="E58" s="66" t="str">
+        <x:v>3:35 PM</x:v>
+      </x:c>
+      <x:c r="F58" s="66" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G58" s="67" t="str"/>
+    </x:row>
+    <x:row r="59" ht="20" customHeight="1">
+      <x:c r="A59" s="57" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B59" s="60" t="str">
+        <x:v>Ascent Rivals</x:v>
+      </x:c>
+      <x:c r="C59" s="58" t="str">
+        <x:v>GENUN Games · Booth L11</x:v>
+      </x:c>
+      <x:c r="D59" s="58" t="str">
+        <x:v>3:35 PM</x:v>
+      </x:c>
+      <x:c r="E59" s="58" t="str">
+        <x:v>3:41 PM</x:v>
+      </x:c>
+      <x:c r="F59" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G59" s="59" t="str"/>
+    </x:row>
+    <x:row r="60" ht="20" customHeight="1">
+      <x:c r="A60" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B60" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C60" s="62" t="str">
+        <x:v>Block F</x:v>
+      </x:c>
+      <x:c r="D60" s="62" t="str">
+        <x:v>3:41 PM</x:v>
+      </x:c>
+      <x:c r="E60" s="62" t="str">
+        <x:v>3:42 PM</x:v>
+      </x:c>
+      <x:c r="F60" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G60" s="63" t="str"/>
+    </x:row>
+    <x:row r="61" ht="20" customHeight="1">
+      <x:c r="A61" s="57" t="str">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B61" s="60" t="str">
+        <x:v>Hamsteria</x:v>
+      </x:c>
+      <x:c r="C61" s="58" t="str">
+        <x:v>2WheelerDev · Booth L10</x:v>
+      </x:c>
+      <x:c r="D61" s="58" t="str">
+        <x:v>3:42 PM</x:v>
+      </x:c>
+      <x:c r="E61" s="58" t="str">
+        <x:v>3:48 PM</x:v>
+      </x:c>
+      <x:c r="F61" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G61" s="59" t="str"/>
+    </x:row>
+    <x:row r="62" ht="20" customHeight="1">
+      <x:c r="A62" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B62" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C62" s="62" t="str">
+        <x:v>Block F</x:v>
+      </x:c>
+      <x:c r="D62" s="62" t="str">
+        <x:v>3:48 PM</x:v>
+      </x:c>
+      <x:c r="E62" s="62" t="str">
+        <x:v>3:49 PM</x:v>
+      </x:c>
+      <x:c r="F62" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G62" s="63" t="str"/>
+    </x:row>
+    <x:row r="63" ht="20" customHeight="1">
+      <x:c r="A63" s="57" t="str">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B63" s="60" t="str">
+        <x:v>Haunted Heist</x:v>
+      </x:c>
+      <x:c r="C63" s="58" t="str">
+        <x:v>autotroph games · Booth L09</x:v>
+      </x:c>
+      <x:c r="D63" s="58" t="str">
+        <x:v>3:49 PM</x:v>
+      </x:c>
+      <x:c r="E63" s="58" t="str">
+        <x:v>3:55 PM</x:v>
+      </x:c>
+      <x:c r="F63" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G63" s="59" t="str"/>
+    </x:row>
+    <x:row r="64" ht="20" customHeight="1">
+      <x:c r="A64" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B64" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C64" s="62" t="str">
+        <x:v>Block F</x:v>
+      </x:c>
+      <x:c r="D64" s="62" t="str">
+        <x:v>3:55 PM</x:v>
+      </x:c>
+      <x:c r="E64" s="62" t="str">
+        <x:v>3:56 PM</x:v>
+      </x:c>
+      <x:c r="F64" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G64" s="63" t="str"/>
+    </x:row>
+    <x:row r="65" ht="20" customHeight="1">
+      <x:c r="A65" s="57" t="str">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B65" s="60" t="str">
+        <x:v>RUNE GUNNER</x:v>
+      </x:c>
+      <x:c r="C65" s="58" t="str">
+        <x:v>False Summit · Booth L08</x:v>
+      </x:c>
+      <x:c r="D65" s="58" t="str">
+        <x:v>3:56 PM</x:v>
+      </x:c>
+      <x:c r="E65" s="58" t="str">
+        <x:v>4:02 PM</x:v>
+      </x:c>
+      <x:c r="F65" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G65" s="59" t="str"/>
+    </x:row>
+    <x:row r="66" ht="20" customHeight="1">
+      <x:c r="A66" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B66" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C66" s="62" t="str">
+        <x:v>Block F</x:v>
+      </x:c>
+      <x:c r="D66" s="62" t="str">
+        <x:v>4:02 PM</x:v>
+      </x:c>
+      <x:c r="E66" s="62" t="str">
+        <x:v>4:03 PM</x:v>
+      </x:c>
+      <x:c r="F66" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G66" s="63" t="str"/>
+    </x:row>
+    <x:row r="67" ht="20" customHeight="1">
+      <x:c r="A67" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B67" s="68" t="str">
+        <x:v>11 Bit Studios Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C67" s="66" t="str">
+        <x:v>Sponsor segment · L06</x:v>
+      </x:c>
+      <x:c r="D67" s="66" t="str">
+        <x:v>4:03 PM</x:v>
+      </x:c>
+      <x:c r="E67" s="66" t="str">
+        <x:v>4:10 PM</x:v>
+      </x:c>
+      <x:c r="F67" s="66" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G67" s="67" t="str"/>
+    </x:row>
+    <x:row r="68" ht="20" customHeight="1">
+      <x:c r="A68" s="57" t="str">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B68" s="60" t="str">
+        <x:v>Telera</x:v>
+      </x:c>
+      <x:c r="C68" s="58" t="str">
+        <x:v>Entropico · Booth U21</x:v>
+      </x:c>
+      <x:c r="D68" s="58" t="str">
+        <x:v>4:10 PM</x:v>
+      </x:c>
+      <x:c r="E68" s="58" t="str">
+        <x:v>4:16 PM</x:v>
+      </x:c>
+      <x:c r="F68" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G68" s="59" t="str"/>
+    </x:row>
+    <x:row r="69" ht="20" customHeight="1">
+      <x:c r="A69" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B69" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C69" s="62" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D69" s="62" t="str">
+        <x:v>4:16 PM</x:v>
+      </x:c>
+      <x:c r="E69" s="62" t="str">
+        <x:v>4:17 PM</x:v>
+      </x:c>
+      <x:c r="F69" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G69" s="63" t="str"/>
+    </x:row>
+    <x:row r="70" ht="20" customHeight="1">
+      <x:c r="A70" s="57" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B70" s="60" t="str">
+        <x:v>Hogen</x:v>
+      </x:c>
+      <x:c r="C70" s="58" t="str">
+        <x:v>Scrappyard Games · Booth U22</x:v>
+      </x:c>
+      <x:c r="D70" s="58" t="str">
+        <x:v>4:17 PM</x:v>
+      </x:c>
+      <x:c r="E70" s="58" t="str">
+        <x:v>4:23 PM</x:v>
+      </x:c>
+      <x:c r="F70" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G70" s="59" t="str"/>
+    </x:row>
+    <x:row r="71" ht="20" customHeight="1">
+      <x:c r="A71" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B71" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C71" s="62" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D71" s="62" t="str">
+        <x:v>4:23 PM</x:v>
+      </x:c>
+      <x:c r="E71" s="62" t="str">
+        <x:v>4:24 PM</x:v>
+      </x:c>
+      <x:c r="F71" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G71" s="63" t="str"/>
+    </x:row>
+    <x:row r="72" ht="20" customHeight="1">
+      <x:c r="A72" s="57" t="str">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B72" s="60" t="str">
+        <x:v>WILL: Follow The Light</x:v>
+      </x:c>
+      <x:c r="C72" s="58" t="str">
+        <x:v>TomorrowHead Studio · Booth U23</x:v>
+      </x:c>
+      <x:c r="D72" s="58" t="str">
+        <x:v>4:24 PM</x:v>
+      </x:c>
+      <x:c r="E72" s="58" t="str">
+        <x:v>4:30 PM</x:v>
+      </x:c>
+      <x:c r="F72" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G72" s="59" t="str"/>
+    </x:row>
+    <x:row r="73" ht="20" customHeight="1">
+      <x:c r="A73" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B73" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C73" s="62" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D73" s="62" t="str">
+        <x:v>4:30 PM</x:v>
+      </x:c>
+      <x:c r="E73" s="62" t="str">
+        <x:v>4:31 PM</x:v>
+      </x:c>
+      <x:c r="F73" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G73" s="63" t="str"/>
+    </x:row>
+    <x:row r="74" ht="20" customHeight="1">
+      <x:c r="A74" s="57" t="str">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B74" s="60" t="str">
+        <x:v>Turning Manor</x:v>
+      </x:c>
+      <x:c r="C74" s="58" t="str">
+        <x:v>Sabbatical Games · Booth U24</x:v>
+      </x:c>
+      <x:c r="D74" s="58" t="str">
+        <x:v>4:31 PM</x:v>
+      </x:c>
+      <x:c r="E74" s="58" t="str">
+        <x:v>4:37 PM</x:v>
+      </x:c>
+      <x:c r="F74" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G74" s="59" t="str"/>
+    </x:row>
+    <x:row r="75" ht="20" customHeight="1">
+      <x:c r="A75" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B75" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C75" s="62" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D75" s="62" t="str">
+        <x:v>4:37 PM</x:v>
+      </x:c>
+      <x:c r="E75" s="62" t="str">
+        <x:v>4:38 PM</x:v>
+      </x:c>
+      <x:c r="F75" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G75" s="63" t="str"/>
+    </x:row>
+    <x:row r="76" ht="20" customHeight="1">
+      <x:c r="A76" s="57" t="str">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B76" s="60" t="str">
+        <x:v>Steel Swarm: SURVIVOR</x:v>
+      </x:c>
+      <x:c r="C76" s="58" t="str">
+        <x:v>Clay Token Game Studio, Inc. · Booth U25</x:v>
+      </x:c>
+      <x:c r="D76" s="58" t="str">
+        <x:v>4:38 PM</x:v>
+      </x:c>
+      <x:c r="E76" s="58" t="str">
+        <x:v>4:44 PM</x:v>
+      </x:c>
+      <x:c r="F76" s="58" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G76" s="59" t="str"/>
+    </x:row>
+    <x:row r="77" ht="20" customHeight="1">
+      <x:c r="A77" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B77" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C77" s="62" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D77" s="62" t="str">
+        <x:v>4:44 PM</x:v>
+      </x:c>
+      <x:c r="E77" s="62" t="str">
+        <x:v>4:45 PM</x:v>
+      </x:c>
+      <x:c r="F77" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G77" s="63" t="str"/>
+    </x:row>
+    <x:row r="78" ht="20" customHeight="1">
+      <x:c r="A78" s="65" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B78" s="68" t="str">
+        <x:v>NDVisibility Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C78" s="66" t="str">
+        <x:v>Sponsor segment · 000</x:v>
+      </x:c>
+      <x:c r="D78" s="66" t="str">
+        <x:v>4:45 PM</x:v>
+      </x:c>
+      <x:c r="E78" s="66" t="str">
+        <x:v>4:55 PM</x:v>
+      </x:c>
+      <x:c r="F78" s="66" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G78" s="67" t="str"/>
+    </x:row>
+    <x:row r="79" ht="20" customHeight="1">
+      <x:c r="A79" s="57" t="str">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B79" s="60" t="str">
+        <x:v>HYPERFIST</x:v>
+      </x:c>
+      <x:c r="C79" s="58" t="str">
+        <x:v>Chirality · Booth U15</x:v>
+      </x:c>
+      <x:c r="D79" s="58" t="str">
+        <x:v>4:55 PM</x:v>
+      </x:c>
+      <x:c r="E79" s="58" t="str">
+        <x:v>5:01 PM</x:v>
+      </x:c>
+      <x:c r="F79" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G79" s="59" t="str"/>
+    </x:row>
+    <x:row r="80" ht="20" customHeight="1">
+      <x:c r="A80" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B80" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C80" s="62" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D80" s="62" t="str">
+        <x:v>5:01 PM</x:v>
+      </x:c>
+      <x:c r="E80" s="62" t="str">
+        <x:v>5:02 PM</x:v>
+      </x:c>
+      <x:c r="F80" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G80" s="63" t="str"/>
+    </x:row>
+    <x:row r="81" ht="20" customHeight="1">
+      <x:c r="A81" s="57" t="str">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B81" s="60" t="str">
+        <x:v>Nightmare Kitchen</x:v>
+      </x:c>
+      <x:c r="C81" s="58" t="str">
+        <x:v>Byteback Studios · Booth U16</x:v>
+      </x:c>
+      <x:c r="D81" s="58" t="str">
+        <x:v>5:02 PM</x:v>
+      </x:c>
+      <x:c r="E81" s="58" t="str">
+        <x:v>5:08 PM</x:v>
+      </x:c>
+      <x:c r="F81" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G81" s="59" t="str"/>
+    </x:row>
+    <x:row r="82" ht="20" customHeight="1">
+      <x:c r="A82" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B82" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C82" s="62" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D82" s="62" t="str">
+        <x:v>5:08 PM</x:v>
+      </x:c>
+      <x:c r="E82" s="62" t="str">
+        <x:v>5:09 PM</x:v>
+      </x:c>
+      <x:c r="F82" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G82" s="63" t="str"/>
+    </x:row>
+    <x:row r="83" ht="20" customHeight="1">
+      <x:c r="A83" s="57" t="str">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B83" s="60" t="str">
+        <x:v>Shroomwood</x:v>
+      </x:c>
+      <x:c r="C83" s="58" t="str">
+        <x:v>Sporelite Games · Booth U17</x:v>
+      </x:c>
+      <x:c r="D83" s="58" t="str">
+        <x:v>5:09 PM</x:v>
+      </x:c>
+      <x:c r="E83" s="58" t="str">
+        <x:v>5:15 PM</x:v>
+      </x:c>
+      <x:c r="F83" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G83" s="59" t="str"/>
+    </x:row>
+    <x:row r="84" ht="20" customHeight="1">
+      <x:c r="A84" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B84" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C84" s="62" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D84" s="62" t="str">
+        <x:v>5:15 PM</x:v>
+      </x:c>
+      <x:c r="E84" s="62" t="str">
+        <x:v>5:16 PM</x:v>
+      </x:c>
+      <x:c r="F84" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G84" s="63" t="str"/>
+    </x:row>
+    <x:row r="85" ht="20" customHeight="1">
+      <x:c r="A85" s="57" t="str">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B85" s="60" t="str">
+        <x:v>Knockout 2: Wrath of the Karen</x:v>
+      </x:c>
+      <x:c r="C85" s="58" t="str">
+        <x:v>ExceptioNULL Games · Booth U18</x:v>
+      </x:c>
+      <x:c r="D85" s="58" t="str">
+        <x:v>5:16 PM</x:v>
+      </x:c>
+      <x:c r="E85" s="58" t="str">
+        <x:v>5:22 PM</x:v>
+      </x:c>
+      <x:c r="F85" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G85" s="59" t="str"/>
+    </x:row>
+    <x:row r="86" ht="20" customHeight="1">
+      <x:c r="A86" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B86" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C86" s="62" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D86" s="62" t="str">
+        <x:v>5:22 PM</x:v>
+      </x:c>
+      <x:c r="E86" s="62" t="str">
+        <x:v>5:23 PM</x:v>
+      </x:c>
+      <x:c r="F86" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G86" s="63" t="str"/>
+    </x:row>
+    <x:row r="87" ht="20" customHeight="1">
+      <x:c r="A87" s="57" t="str">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B87" s="60" t="str">
+        <x:v>Cooking Fist</x:v>
+      </x:c>
+      <x:c r="C87" s="58" t="str">
+        <x:v>Spaghetti Code LLC · Booth U19</x:v>
+      </x:c>
+      <x:c r="D87" s="58" t="str">
+        <x:v>5:23 PM</x:v>
+      </x:c>
+      <x:c r="E87" s="58" t="str">
+        <x:v>5:29 PM</x:v>
+      </x:c>
+      <x:c r="F87" s="58" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G87" s="59" t="str"/>
+    </x:row>
+    <x:row r="88" ht="20" customHeight="1">
+      <x:c r="A88" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B88" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C88" s="62" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D88" s="62" t="str">
+        <x:v>5:29 PM</x:v>
+      </x:c>
+      <x:c r="E88" s="62" t="str">
+        <x:v>5:30 PM</x:v>
+      </x:c>
+      <x:c r="F88" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G88" s="63" t="str"/>
+    </x:row>
+    <x:row r="89" ht="20" customHeight="1">
+      <x:c r="A89" s="69" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B89" s="72" t="str">
+        <x:v>Ukrainian Games Videos</x:v>
+      </x:c>
+      <x:c r="C89" s="70" t="str">
+        <x:v>International showcase · 000</x:v>
+      </x:c>
+      <x:c r="D89" s="70" t="str">
+        <x:v>5:30 PM</x:v>
+      </x:c>
+      <x:c r="E89" s="70" t="str">
+        <x:v>5:35 PM</x:v>
+      </x:c>
+      <x:c r="F89" s="70" t="str">
+        <x:v>Prerecorded</x:v>
+      </x:c>
+      <x:c r="G89" s="71" t="str"/>
+    </x:row>
+    <x:row r="90" ht="20" customHeight="1">
+      <x:c r="A90" s="57" t="str">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B90" s="60" t="str">
+        <x:v>Killing Baby Hitler</x:v>
+      </x:c>
+      <x:c r="C90" s="58" t="str">
+        <x:v>The Coffee Industrial Complex · Booth U14</x:v>
+      </x:c>
+      <x:c r="D90" s="58" t="str">
+        <x:v>5:35 PM</x:v>
+      </x:c>
+      <x:c r="E90" s="58" t="str">
+        <x:v>5:41 PM</x:v>
+      </x:c>
+      <x:c r="F90" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G90" s="59" t="str"/>
+    </x:row>
+    <x:row r="91" ht="20" customHeight="1">
+      <x:c r="A91" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B91" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C91" s="62" t="str">
+        <x:v>Block I</x:v>
+      </x:c>
+      <x:c r="D91" s="62" t="str">
+        <x:v>5:41 PM</x:v>
+      </x:c>
+      <x:c r="E91" s="62" t="str">
+        <x:v>5:42 PM</x:v>
+      </x:c>
+      <x:c r="F91" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G91" s="63" t="str"/>
+    </x:row>
+    <x:row r="92" ht="20" customHeight="1">
+      <x:c r="A92" s="57" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B92" s="60" t="str">
+        <x:v>The Assessment</x:v>
+      </x:c>
+      <x:c r="C92" s="58" t="str">
+        <x:v>Miga Games · Booth U11</x:v>
+      </x:c>
+      <x:c r="D92" s="58" t="str">
+        <x:v>5:42 PM</x:v>
+      </x:c>
+      <x:c r="E92" s="58" t="str">
+        <x:v>5:48 PM</x:v>
+      </x:c>
+      <x:c r="F92" s="58" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G92" s="59" t="str"/>
+    </x:row>
+    <x:row r="93" ht="20" customHeight="1">
+      <x:c r="A93" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B93" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C93" s="62" t="str">
+        <x:v>Block I</x:v>
+      </x:c>
+      <x:c r="D93" s="62" t="str">
+        <x:v>5:48 PM</x:v>
+      </x:c>
+      <x:c r="E93" s="62" t="str">
+        <x:v>5:49 PM</x:v>
+      </x:c>
+      <x:c r="F93" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G93" s="63" t="str"/>
+    </x:row>
+    <x:row r="94" ht="20" customHeight="1">
+      <x:c r="A94" s="69" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B94" s="72" t="str">
+        <x:v>Chile Games Showcase Video</x:v>
+      </x:c>
+      <x:c r="C94" s="70" t="str">
+        <x:v>International showcase · 000</x:v>
+      </x:c>
+      <x:c r="D94" s="70" t="str">
+        <x:v>5:49 PM</x:v>
+      </x:c>
+      <x:c r="E94" s="70" t="str">
+        <x:v>5:54 PM</x:v>
+      </x:c>
+      <x:c r="F94" s="70" t="str">
+        <x:v>Prerecorded</x:v>
+      </x:c>
+      <x:c r="G94" s="71" t="str"/>
+    </x:row>
+    <x:row r="95" ht="20" customHeight="1">
+      <x:c r="A95" s="61" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B95" s="64" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C95" s="62" t="str">
+        <x:v>Block I</x:v>
+      </x:c>
+      <x:c r="D95" s="62" t="str">
+        <x:v>5:54 PM</x:v>
+      </x:c>
+      <x:c r="E95" s="62" t="str">
+        <x:v>5:55 PM</x:v>
+      </x:c>
+      <x:c r="F95" s="62" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G95" s="63" t="str"/>
+    </x:row>
+    <x:row r="96" ht="20" customHeight="1">
+      <x:c r="A96" s="73" t="str">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B96" s="76" t="str">
+        <x:v>Closing / Thank You</x:v>
+      </x:c>
+      <x:c r="C96" s="74" t="str">
         <x:v>Seattle Indies</x:v>
       </x:c>
-      <x:c r="D6" s="21" t="str">
-        <x:v>12:00 PM</x:v>
-      </x:c>
-      <x:c r="E6" s="21" t="str">
-        <x:v>12:05 PM</x:v>
-      </x:c>
-      <x:c r="F6" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G6" s="21"/>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B7" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C7" s="18"/>
-      <x:c r="D7" s="18" t="str">
-        <x:v>12:05 PM</x:v>
-      </x:c>
-      <x:c r="E7" s="18" t="str">
-        <x:v>12:07 PM</x:v>
-      </x:c>
-      <x:c r="F7" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G7" s="18"/>
-    </x:row>
-    <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="21" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B8" s="22" t="str">
-        <x:v>Ascent Rivals</x:v>
-      </x:c>
-      <x:c r="C8" s="21" t="str">
-        <x:v>GENUN Games</x:v>
-      </x:c>
-      <x:c r="D8" s="21" t="str">
-        <x:v>12:07 PM</x:v>
-      </x:c>
-      <x:c r="E8" s="21" t="str">
-        <x:v>12:13 PM</x:v>
-      </x:c>
-      <x:c r="F8" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G8" s="21"/>
-    </x:row>
-    <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B9" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C9" s="18"/>
-      <x:c r="D9" s="18" t="str">
-        <x:v>12:13 PM</x:v>
-      </x:c>
-      <x:c r="E9" s="18" t="str">
-        <x:v>12:15 PM</x:v>
-      </x:c>
-      <x:c r="F9" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G9" s="18"/>
-    </x:row>
-    <x:row r="10" ht="25" customHeight="1">
-      <x:c r="A10" s="21" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B10" s="22" t="str">
-        <x:v>Breach Of Contract</x:v>
-      </x:c>
-      <x:c r="C10" s="21" t="str">
-        <x:v>Fern Sprout Studios</x:v>
-      </x:c>
-      <x:c r="D10" s="21" t="str">
-        <x:v>12:15 PM</x:v>
-      </x:c>
-      <x:c r="E10" s="21" t="str">
-        <x:v>12:21 PM</x:v>
-      </x:c>
-      <x:c r="F10" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="21"/>
-    </x:row>
-    <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B11" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C11" s="18"/>
-      <x:c r="D11" s="18" t="str">
-        <x:v>12:21 PM</x:v>
-      </x:c>
-      <x:c r="E11" s="18" t="str">
-        <x:v>12:23 PM</x:v>
-      </x:c>
-      <x:c r="F11" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G11" s="18"/>
-    </x:row>
-    <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="21" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B12" s="22" t="str">
-        <x:v>BroomSweeper</x:v>
-      </x:c>
-      <x:c r="C12" s="21" t="str">
-        <x:v>BandWidth Games</x:v>
-      </x:c>
-      <x:c r="D12" s="21" t="str">
-        <x:v>12:23 PM</x:v>
-      </x:c>
-      <x:c r="E12" s="21" t="str">
-        <x:v>12:29 PM</x:v>
-      </x:c>
-      <x:c r="F12" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G12" s="21"/>
-    </x:row>
-    <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B13" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C13" s="18"/>
-      <x:c r="D13" s="18" t="str">
-        <x:v>12:29 PM</x:v>
-      </x:c>
-      <x:c r="E13" s="18" t="str">
-        <x:v>12:31 PM</x:v>
-      </x:c>
-      <x:c r="F13" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G13" s="18"/>
-    </x:row>
-    <x:row r="14" ht="25" customHeight="1">
-      <x:c r="A14" s="21" t="str">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B14" s="22" t="str">
-        <x:v>Cooking Fist</x:v>
-      </x:c>
-      <x:c r="C14" s="21" t="str">
-        <x:v>Spaghetti Code LLC</x:v>
-      </x:c>
-      <x:c r="D14" s="21" t="str">
-        <x:v>12:31 PM</x:v>
-      </x:c>
-      <x:c r="E14" s="21" t="str">
-        <x:v>12:37 PM</x:v>
-      </x:c>
-      <x:c r="F14" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G14" s="21"/>
-    </x:row>
-    <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B15" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C15" s="18"/>
-      <x:c r="D15" s="18" t="str">
-        <x:v>12:37 PM</x:v>
-      </x:c>
-      <x:c r="E15" s="18" t="str">
-        <x:v>12:39 PM</x:v>
-      </x:c>
-      <x:c r="F15" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G15" s="18"/>
-    </x:row>
-    <x:row r="16" ht="25" customHeight="1">
-      <x:c r="A16" s="21" t="str">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B16" s="22" t="str">
-        <x:v>Creature Kitchen</x:v>
-      </x:c>
-      <x:c r="C16" s="21" t="str">
-        <x:v>The Rat Zone</x:v>
-      </x:c>
-      <x:c r="D16" s="21" t="str">
-        <x:v>12:39 PM</x:v>
-      </x:c>
-      <x:c r="E16" s="21" t="str">
-        <x:v>12:45 PM</x:v>
-      </x:c>
-      <x:c r="F16" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G16" s="21"/>
-    </x:row>
-    <x:row r="17" ht="25" customHeight="1">
-      <x:c r="A17" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B17" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C17" s="18"/>
-      <x:c r="D17" s="18" t="str">
-        <x:v>12:45 PM</x:v>
-      </x:c>
-      <x:c r="E17" s="18" t="str">
-        <x:v>12:47 PM</x:v>
-      </x:c>
-      <x:c r="F17" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G17" s="18"/>
-    </x:row>
-    <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="21" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B18" s="22" t="str">
-        <x:v>Desolus</x:v>
-      </x:c>
-      <x:c r="C18" s="21" t="str">
-        <x:v>Mark J. Mayers</x:v>
-      </x:c>
-      <x:c r="D18" s="21" t="str">
-        <x:v>12:47 PM</x:v>
-      </x:c>
-      <x:c r="E18" s="21" t="str">
-        <x:v>12:53 PM</x:v>
-      </x:c>
-      <x:c r="F18" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G18" s="21"/>
-    </x:row>
-    <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B19" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C19" s="18"/>
-      <x:c r="D19" s="18" t="str">
-        <x:v>12:53 PM</x:v>
-      </x:c>
-      <x:c r="E19" s="18" t="str">
-        <x:v>12:55 PM</x:v>
-      </x:c>
-      <x:c r="F19" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G19" s="18"/>
-    </x:row>
-    <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="24" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B20" s="24" t="str">
-        <x:v>Diabolocracy</x:v>
-      </x:c>
-      <x:c r="C20" s="24" t="str">
-        <x:v>Chaos Gremlin Games</x:v>
-      </x:c>
-      <x:c r="D20" s="24" t="str">
-        <x:v>12:55 PM</x:v>
-      </x:c>
-      <x:c r="E20" s="24" t="str">
-        <x:v>1:01 PM</x:v>
-      </x:c>
-      <x:c r="F20" s="24" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G20" s="24"/>
-    </x:row>
-    <x:row r="21" ht="25" customHeight="1">
-      <x:c r="A21" s="21" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B21" s="22" t="str">
-        <x:v>Seattle Indies / Sponsor Ad Read</x:v>
-      </x:c>
-      <x:c r="C21" s="21" t="str">
-        <x:v>Sponsor copy pending</x:v>
-      </x:c>
-      <x:c r="D21" s="21" t="str">
-        <x:v>1:01 PM</x:v>
-      </x:c>
-      <x:c r="E21" s="21" t="str">
-        <x:v>1:03 PM</x:v>
-      </x:c>
-      <x:c r="F21" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G21" s="21"/>
-    </x:row>
-    <x:row r="22" ht="25" customHeight="1">
-      <x:c r="A22" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B22" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C22" s="18"/>
-      <x:c r="D22" s="18" t="str">
-        <x:v>1:03 PM</x:v>
-      </x:c>
-      <x:c r="E22" s="18" t="str">
-        <x:v>1:05 PM</x:v>
-      </x:c>
-      <x:c r="F22" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G22" s="18"/>
-    </x:row>
-    <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="21" t="str">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B23" s="22" t="str">
-        <x:v>Dig Too Deep</x:v>
-      </x:c>
-      <x:c r="C23" s="21" t="str">
-        <x:v>Punch Up Games</x:v>
-      </x:c>
-      <x:c r="D23" s="21" t="str">
-        <x:v>1:05 PM</x:v>
-      </x:c>
-      <x:c r="E23" s="21" t="str">
-        <x:v>1:11 PM</x:v>
-      </x:c>
-      <x:c r="F23" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G23" s="21"/>
-    </x:row>
-    <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B24" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C24" s="18"/>
-      <x:c r="D24" s="18" t="str">
-        <x:v>1:11 PM</x:v>
-      </x:c>
-      <x:c r="E24" s="18" t="str">
-        <x:v>1:13 PM</x:v>
-      </x:c>
-      <x:c r="F24" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G24" s="18"/>
-    </x:row>
-    <x:row r="25" ht="25" customHeight="1">
-      <x:c r="A25" s="21" t="str">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B25" s="22" t="str">
-        <x:v>Dittori</x:v>
-      </x:c>
-      <x:c r="C25" s="21" t="str">
-        <x:v>Blookerstein</x:v>
-      </x:c>
-      <x:c r="D25" s="21" t="str">
-        <x:v>1:13 PM</x:v>
-      </x:c>
-      <x:c r="E25" s="21" t="str">
-        <x:v>1:19 PM</x:v>
-      </x:c>
-      <x:c r="F25" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G25" s="21"/>
-    </x:row>
-    <x:row r="26" ht="25" customHeight="1">
-      <x:c r="A26" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B26" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C26" s="18"/>
-      <x:c r="D26" s="18" t="str">
-        <x:v>1:19 PM</x:v>
-      </x:c>
-      <x:c r="E26" s="18" t="str">
-        <x:v>1:21 PM</x:v>
-      </x:c>
-      <x:c r="F26" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G26" s="18"/>
-    </x:row>
-    <x:row r="27" ht="25" customHeight="1">
-      <x:c r="A27" s="21" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B27" s="22" t="str">
-        <x:v>Dungeon Bodega Simulator</x:v>
-      </x:c>
-      <x:c r="C27" s="21" t="str">
-        <x:v>Alien Fruit Games</x:v>
-      </x:c>
-      <x:c r="D27" s="21" t="str">
-        <x:v>1:21 PM</x:v>
-      </x:c>
-      <x:c r="E27" s="21" t="str">
-        <x:v>1:27 PM</x:v>
-      </x:c>
-      <x:c r="F27" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G27" s="21"/>
-    </x:row>
-    <x:row r="28" ht="25" customHeight="1">
-      <x:c r="A28" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B28" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C28" s="18"/>
-      <x:c r="D28" s="18" t="str">
-        <x:v>1:27 PM</x:v>
-      </x:c>
-      <x:c r="E28" s="18" t="str">
-        <x:v>1:29 PM</x:v>
-      </x:c>
-      <x:c r="F28" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G28" s="18"/>
-    </x:row>
-    <x:row r="29" ht="25" customHeight="1">
-      <x:c r="A29" s="21" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B29" s="22" t="str">
-        <x:v>End of Garbage</x:v>
-      </x:c>
-      <x:c r="C29" s="21" t="str">
-        <x:v>Joshua Rosen (Rakelock LLC)</x:v>
-      </x:c>
-      <x:c r="D29" s="21" t="str">
-        <x:v>1:29 PM</x:v>
-      </x:c>
-      <x:c r="E29" s="21" t="str">
-        <x:v>1:35 PM</x:v>
-      </x:c>
-      <x:c r="F29" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G29" s="21"/>
-    </x:row>
-    <x:row r="30" ht="25" customHeight="1">
-      <x:c r="A30" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B30" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C30" s="18"/>
-      <x:c r="D30" s="18" t="str">
-        <x:v>1:35 PM</x:v>
-      </x:c>
-      <x:c r="E30" s="18" t="str">
-        <x:v>1:37 PM</x:v>
-      </x:c>
-      <x:c r="F30" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G30" s="18"/>
-    </x:row>
-    <x:row r="31" ht="25" customHeight="1">
-      <x:c r="A31" s="21" t="str">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B31" s="22" t="str">
-        <x:v>Fairy Circle</x:v>
-      </x:c>
-      <x:c r="C31" s="21" t="str">
-        <x:v>Play Hooky</x:v>
-      </x:c>
-      <x:c r="D31" s="21" t="str">
-        <x:v>1:37 PM</x:v>
-      </x:c>
-      <x:c r="E31" s="21" t="str">
-        <x:v>1:43 PM</x:v>
-      </x:c>
-      <x:c r="F31" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G31" s="21"/>
-    </x:row>
-    <x:row r="32" ht="25" customHeight="1">
-      <x:c r="A32" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B32" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C32" s="18"/>
-      <x:c r="D32" s="18" t="str">
-        <x:v>1:43 PM</x:v>
-      </x:c>
-      <x:c r="E32" s="18" t="str">
-        <x:v>1:45 PM</x:v>
-      </x:c>
-      <x:c r="F32" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G32" s="18"/>
-    </x:row>
-    <x:row r="33" ht="25" customHeight="1">
-      <x:c r="A33" s="21" t="str">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B33" s="22" t="str">
-        <x:v>Feeding Gooble</x:v>
-      </x:c>
-      <x:c r="C33" s="21" t="str">
-        <x:v>Displacer Labs</x:v>
-      </x:c>
-      <x:c r="D33" s="21" t="str">
-        <x:v>1:45 PM</x:v>
-      </x:c>
-      <x:c r="E33" s="21" t="str">
-        <x:v>1:51 PM</x:v>
-      </x:c>
-      <x:c r="F33" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G33" s="21"/>
-    </x:row>
-    <x:row r="34" ht="25" customHeight="1">
-      <x:c r="A34" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B34" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C34" s="18"/>
-      <x:c r="D34" s="18" t="str">
-        <x:v>1:51 PM</x:v>
-      </x:c>
-      <x:c r="E34" s="18" t="str">
-        <x:v>1:53 PM</x:v>
-      </x:c>
-      <x:c r="F34" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G34" s="18"/>
-    </x:row>
-    <x:row r="35" ht="25" customHeight="1">
-      <x:c r="A35" s="21" t="str">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B35" s="22" t="str">
-        <x:v>Gravity Goblins</x:v>
-      </x:c>
-      <x:c r="C35" s="21" t="str">
-        <x:v>The Rat Zone</x:v>
-      </x:c>
-      <x:c r="D35" s="21" t="str">
-        <x:v>1:53 PM</x:v>
-      </x:c>
-      <x:c r="E35" s="21" t="str">
-        <x:v>1:59 PM</x:v>
-      </x:c>
-      <x:c r="F35" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G35" s="21"/>
-    </x:row>
-    <x:row r="36" ht="25" customHeight="1">
-      <x:c r="A36" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B36" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C36" s="18"/>
-      <x:c r="D36" s="18" t="str">
-        <x:v>1:59 PM</x:v>
-      </x:c>
-      <x:c r="E36" s="18" t="str">
-        <x:v>2:01 PM</x:v>
-      </x:c>
-      <x:c r="F36" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G36" s="18"/>
-    </x:row>
-    <x:row r="37" ht="25" customHeight="1">
-      <x:c r="A37" s="24" t="str">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B37" s="24" t="str">
-        <x:v>Hamsteria</x:v>
-      </x:c>
-      <x:c r="C37" s="24" t="str">
-        <x:v>2WheelerDev</x:v>
-      </x:c>
-      <x:c r="D37" s="24" t="str">
-        <x:v>2:01 PM</x:v>
-      </x:c>
-      <x:c r="E37" s="24" t="str">
-        <x:v>2:07 PM</x:v>
-      </x:c>
-      <x:c r="F37" s="24" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G37" s="24"/>
-    </x:row>
-    <x:row r="38" ht="25" customHeight="1">
-      <x:c r="A38" s="21" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B38" s="22" t="str">
-        <x:v>Seattle Indies / Sponsor Ad Read</x:v>
-      </x:c>
-      <x:c r="C38" s="21" t="str">
-        <x:v>Sponsor copy pending</x:v>
-      </x:c>
-      <x:c r="D38" s="21" t="str">
-        <x:v>2:07 PM</x:v>
-      </x:c>
-      <x:c r="E38" s="21" t="str">
-        <x:v>2:09 PM</x:v>
-      </x:c>
-      <x:c r="F38" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G38" s="21"/>
-    </x:row>
-    <x:row r="39" ht="25" customHeight="1">
-      <x:c r="A39" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B39" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C39" s="18"/>
-      <x:c r="D39" s="18" t="str">
-        <x:v>2:09 PM</x:v>
-      </x:c>
-      <x:c r="E39" s="18" t="str">
-        <x:v>2:11 PM</x:v>
-      </x:c>
-      <x:c r="F39" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G39" s="18"/>
-    </x:row>
-    <x:row r="40" ht="25" customHeight="1">
-      <x:c r="A40" s="21" t="str">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B40" s="22" t="str">
-        <x:v>Haunted Heist</x:v>
-      </x:c>
-      <x:c r="C40" s="21" t="str">
-        <x:v>autotroph games</x:v>
-      </x:c>
-      <x:c r="D40" s="21" t="str">
-        <x:v>2:11 PM</x:v>
-      </x:c>
-      <x:c r="E40" s="21" t="str">
-        <x:v>2:17 PM</x:v>
-      </x:c>
-      <x:c r="F40" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G40" s="21"/>
-    </x:row>
-    <x:row r="41" ht="25" customHeight="1">
-      <x:c r="A41" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B41" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C41" s="18"/>
-      <x:c r="D41" s="18" t="str">
-        <x:v>2:17 PM</x:v>
-      </x:c>
-      <x:c r="E41" s="18" t="str">
-        <x:v>2:19 PM</x:v>
-      </x:c>
-      <x:c r="F41" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G41" s="18"/>
-    </x:row>
-    <x:row r="42" ht="25" customHeight="1">
-      <x:c r="A42" s="21" t="str">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B42" s="22" t="str">
-        <x:v>Hogen</x:v>
-      </x:c>
-      <x:c r="C42" s="21" t="str">
-        <x:v>Scrappyard Games</x:v>
-      </x:c>
-      <x:c r="D42" s="21" t="str">
-        <x:v>2:19 PM</x:v>
-      </x:c>
-      <x:c r="E42" s="21" t="str">
-        <x:v>2:25 PM</x:v>
-      </x:c>
-      <x:c r="F42" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G42" s="21"/>
-    </x:row>
-    <x:row r="43" ht="25" customHeight="1">
-      <x:c r="A43" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B43" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C43" s="18"/>
-      <x:c r="D43" s="18" t="str">
-        <x:v>2:25 PM</x:v>
-      </x:c>
-      <x:c r="E43" s="18" t="str">
-        <x:v>2:27 PM</x:v>
-      </x:c>
-      <x:c r="F43" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G43" s="18"/>
-    </x:row>
-    <x:row r="44" ht="25" customHeight="1">
-      <x:c r="A44" s="21" t="str">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B44" s="22" t="str">
-        <x:v>HYPERFIST</x:v>
-      </x:c>
-      <x:c r="C44" s="21" t="str">
-        <x:v>Chirality</x:v>
-      </x:c>
-      <x:c r="D44" s="21" t="str">
-        <x:v>2:27 PM</x:v>
-      </x:c>
-      <x:c r="E44" s="21" t="str">
-        <x:v>2:33 PM</x:v>
-      </x:c>
-      <x:c r="F44" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G44" s="21"/>
-    </x:row>
-    <x:row r="45" ht="25" customHeight="1">
-      <x:c r="A45" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B45" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C45" s="18"/>
-      <x:c r="D45" s="18" t="str">
-        <x:v>2:33 PM</x:v>
-      </x:c>
-      <x:c r="E45" s="18" t="str">
-        <x:v>2:35 PM</x:v>
-      </x:c>
-      <x:c r="F45" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G45" s="18"/>
-    </x:row>
-    <x:row r="46" ht="25" customHeight="1">
-      <x:c r="A46" s="21" t="str">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B46" s="22" t="str">
-        <x:v>Killing Baby Hitler</x:v>
-      </x:c>
-      <x:c r="C46" s="21" t="str">
-        <x:v>The Coffee Industrial Complex</x:v>
-      </x:c>
-      <x:c r="D46" s="21" t="str">
-        <x:v>2:35 PM</x:v>
-      </x:c>
-      <x:c r="E46" s="21" t="str">
-        <x:v>2:41 PM</x:v>
-      </x:c>
-      <x:c r="F46" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G46" s="21"/>
-    </x:row>
-    <x:row r="47" ht="25" customHeight="1">
-      <x:c r="A47" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B47" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C47" s="18"/>
-      <x:c r="D47" s="18" t="str">
-        <x:v>2:41 PM</x:v>
-      </x:c>
-      <x:c r="E47" s="18" t="str">
-        <x:v>2:43 PM</x:v>
-      </x:c>
-      <x:c r="F47" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G47" s="18"/>
-    </x:row>
-    <x:row r="48" ht="25" customHeight="1">
-      <x:c r="A48" s="21" t="str">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B48" s="22" t="str">
-        <x:v>Knockout 2: Wrath of the Karen</x:v>
-      </x:c>
-      <x:c r="C48" s="21" t="str">
-        <x:v>ExceptioNULL Games</x:v>
-      </x:c>
-      <x:c r="D48" s="21" t="str">
-        <x:v>2:43 PM</x:v>
-      </x:c>
-      <x:c r="E48" s="21" t="str">
-        <x:v>2:49 PM</x:v>
-      </x:c>
-      <x:c r="F48" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G48" s="21"/>
-    </x:row>
-    <x:row r="49" ht="25" customHeight="1">
-      <x:c r="A49" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B49" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C49" s="18"/>
-      <x:c r="D49" s="18" t="str">
-        <x:v>2:49 PM</x:v>
-      </x:c>
-      <x:c r="E49" s="18" t="str">
-        <x:v>2:51 PM</x:v>
-      </x:c>
-      <x:c r="F49" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G49" s="18"/>
-    </x:row>
-    <x:row r="50" ht="25" customHeight="1">
-      <x:c r="A50" s="21" t="str">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B50" s="22" t="str">
-        <x:v>Malice In Wonderland</x:v>
-      </x:c>
-      <x:c r="C50" s="21" t="str">
-        <x:v>Slyglass Games</x:v>
-      </x:c>
-      <x:c r="D50" s="21" t="str">
-        <x:v>2:51 PM</x:v>
-      </x:c>
-      <x:c r="E50" s="21" t="str">
-        <x:v>2:57 PM</x:v>
-      </x:c>
-      <x:c r="F50" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G50" s="21"/>
-    </x:row>
-    <x:row r="51" ht="25" customHeight="1">
-      <x:c r="A51" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B51" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C51" s="18"/>
-      <x:c r="D51" s="18" t="str">
-        <x:v>2:57 PM</x:v>
-      </x:c>
-      <x:c r="E51" s="18" t="str">
-        <x:v>2:59 PM</x:v>
-      </x:c>
-      <x:c r="F51" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G51" s="18"/>
-    </x:row>
-    <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="24" t="str">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B52" s="24" t="str">
-        <x:v>Manafinder II</x:v>
-      </x:c>
-      <x:c r="C52" s="24" t="str">
-        <x:v>Wolfsden LLC</x:v>
-      </x:c>
-      <x:c r="D52" s="24" t="str">
-        <x:v>2:59 PM</x:v>
-      </x:c>
-      <x:c r="E52" s="24" t="str">
-        <x:v>3:05 PM</x:v>
-      </x:c>
-      <x:c r="F52" s="24" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G52" s="24"/>
-    </x:row>
-    <x:row r="53" ht="25" customHeight="1">
-      <x:c r="A53" s="21" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B53" s="22" t="str">
-        <x:v>Seattle Indies / Sponsor Ad Read</x:v>
-      </x:c>
-      <x:c r="C53" s="21" t="str">
-        <x:v>Sponsor copy pending</x:v>
-      </x:c>
-      <x:c r="D53" s="21" t="str">
-        <x:v>3:05 PM</x:v>
-      </x:c>
-      <x:c r="E53" s="21" t="str">
-        <x:v>3:07 PM</x:v>
-      </x:c>
-      <x:c r="F53" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G53" s="21"/>
-    </x:row>
-    <x:row r="54" ht="25" customHeight="1">
-      <x:c r="A54" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B54" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C54" s="18"/>
-      <x:c r="D54" s="18" t="str">
-        <x:v>3:07 PM</x:v>
-      </x:c>
-      <x:c r="E54" s="18" t="str">
-        <x:v>3:09 PM</x:v>
-      </x:c>
-      <x:c r="F54" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G54" s="18"/>
-    </x:row>
-    <x:row r="55" ht="25" customHeight="1">
-      <x:c r="A55" s="21" t="str">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B55" s="22" t="str">
-        <x:v>MYRIORAMA</x:v>
-      </x:c>
-      <x:c r="C55" s="21" t="str">
-        <x:v>J&amp;K Games</x:v>
-      </x:c>
-      <x:c r="D55" s="21" t="str">
-        <x:v>3:09 PM</x:v>
-      </x:c>
-      <x:c r="E55" s="21" t="str">
-        <x:v>3:15 PM</x:v>
-      </x:c>
-      <x:c r="F55" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G55" s="21"/>
-    </x:row>
-    <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B56" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C56" s="18"/>
-      <x:c r="D56" s="18" t="str">
-        <x:v>3:15 PM</x:v>
-      </x:c>
-      <x:c r="E56" s="18" t="str">
-        <x:v>3:17 PM</x:v>
-      </x:c>
-      <x:c r="F56" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G56" s="18"/>
-    </x:row>
-    <x:row r="57" ht="25" customHeight="1">
-      <x:c r="A57" s="21" t="str">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B57" s="22" t="str">
-        <x:v>Nightmare Kitchen</x:v>
-      </x:c>
-      <x:c r="C57" s="21" t="str">
-        <x:v>Byteback Studios</x:v>
-      </x:c>
-      <x:c r="D57" s="21" t="str">
-        <x:v>3:17 PM</x:v>
-      </x:c>
-      <x:c r="E57" s="21" t="str">
-        <x:v>3:23 PM</x:v>
-      </x:c>
-      <x:c r="F57" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G57" s="21"/>
-    </x:row>
-    <x:row r="58" ht="25" customHeight="1">
-      <x:c r="A58" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B58" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C58" s="18"/>
-      <x:c r="D58" s="18" t="str">
-        <x:v>3:23 PM</x:v>
-      </x:c>
-      <x:c r="E58" s="18" t="str">
-        <x:v>3:25 PM</x:v>
-      </x:c>
-      <x:c r="F58" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G58" s="18"/>
-    </x:row>
-    <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="21" t="str">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B59" s="22" t="str">
-        <x:v>Nimbit Frontier</x:v>
-      </x:c>
-      <x:c r="C59" s="21" t="str">
-        <x:v>Megasploot</x:v>
-      </x:c>
-      <x:c r="D59" s="21" t="str">
-        <x:v>3:25 PM</x:v>
-      </x:c>
-      <x:c r="E59" s="21" t="str">
-        <x:v>3:31 PM</x:v>
-      </x:c>
-      <x:c r="F59" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G59" s="21"/>
-    </x:row>
-    <x:row r="60" ht="25" customHeight="1">
-      <x:c r="A60" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B60" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C60" s="18"/>
-      <x:c r="D60" s="18" t="str">
-        <x:v>3:31 PM</x:v>
-      </x:c>
-      <x:c r="E60" s="18" t="str">
-        <x:v>3:33 PM</x:v>
-      </x:c>
-      <x:c r="F60" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G60" s="18"/>
-    </x:row>
-    <x:row r="61" ht="25" customHeight="1">
-      <x:c r="A61" s="21" t="str">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B61" s="22" t="str">
-        <x:v>RUNE GUNNER</x:v>
-      </x:c>
-      <x:c r="C61" s="21" t="str">
-        <x:v>False Summit</x:v>
-      </x:c>
-      <x:c r="D61" s="21" t="str">
-        <x:v>3:33 PM</x:v>
-      </x:c>
-      <x:c r="E61" s="21" t="str">
-        <x:v>3:39 PM</x:v>
-      </x:c>
-      <x:c r="F61" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G61" s="21"/>
-    </x:row>
-    <x:row r="62" ht="25" customHeight="1">
-      <x:c r="A62" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B62" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C62" s="18"/>
-      <x:c r="D62" s="18" t="str">
-        <x:v>3:39 PM</x:v>
-      </x:c>
-      <x:c r="E62" s="18" t="str">
-        <x:v>3:41 PM</x:v>
-      </x:c>
-      <x:c r="F62" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G62" s="18"/>
-    </x:row>
-    <x:row r="63" ht="25" customHeight="1">
-      <x:c r="A63" s="21" t="str">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B63" s="22" t="str">
-        <x:v>SCP: Antimemetics Division</x:v>
-      </x:c>
-      <x:c r="C63" s="21" t="str">
-        <x:v>Quadrant Five</x:v>
-      </x:c>
-      <x:c r="D63" s="21" t="str">
-        <x:v>3:41 PM</x:v>
-      </x:c>
-      <x:c r="E63" s="21" t="str">
-        <x:v>3:47 PM</x:v>
-      </x:c>
-      <x:c r="F63" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G63" s="21"/>
-    </x:row>
-    <x:row r="64" ht="25" customHeight="1">
-      <x:c r="A64" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B64" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C64" s="18"/>
-      <x:c r="D64" s="18" t="str">
-        <x:v>3:47 PM</x:v>
-      </x:c>
-      <x:c r="E64" s="18" t="str">
-        <x:v>3:49 PM</x:v>
-      </x:c>
-      <x:c r="F64" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G64" s="18"/>
-    </x:row>
-    <x:row r="65" ht="25" customHeight="1">
-      <x:c r="A65" s="21" t="str">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B65" s="22" t="str">
-        <x:v>Seedborne Soldiers</x:v>
-      </x:c>
-      <x:c r="C65" s="21" t="str">
-        <x:v>Hat Wobble Games</x:v>
-      </x:c>
-      <x:c r="D65" s="21" t="str">
-        <x:v>3:49 PM</x:v>
-      </x:c>
-      <x:c r="E65" s="21" t="str">
-        <x:v>3:55 PM</x:v>
-      </x:c>
-      <x:c r="F65" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G65" s="21"/>
-    </x:row>
-    <x:row r="66" ht="25" customHeight="1">
-      <x:c r="A66" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B66" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C66" s="18"/>
-      <x:c r="D66" s="18" t="str">
-        <x:v>3:55 PM</x:v>
-      </x:c>
-      <x:c r="E66" s="18" t="str">
-        <x:v>3:57 PM</x:v>
-      </x:c>
-      <x:c r="F66" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G66" s="18"/>
-    </x:row>
-    <x:row r="67" ht="25" customHeight="1">
-      <x:c r="A67" s="24" t="str">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B67" s="24" t="str">
-        <x:v>Shroomwood</x:v>
-      </x:c>
-      <x:c r="C67" s="24" t="str">
-        <x:v>Sporelite Games</x:v>
-      </x:c>
-      <x:c r="D67" s="24" t="str">
-        <x:v>3:57 PM</x:v>
-      </x:c>
-      <x:c r="E67" s="24" t="str">
-        <x:v>4:03 PM</x:v>
-      </x:c>
-      <x:c r="F67" s="24" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G67" s="24"/>
-    </x:row>
-    <x:row r="68" ht="25" customHeight="1">
-      <x:c r="A68" s="21" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B68" s="22" t="str">
-        <x:v>Seattle Indies / Sponsor Ad Read</x:v>
-      </x:c>
-      <x:c r="C68" s="21" t="str">
-        <x:v>Sponsor copy pending</x:v>
-      </x:c>
-      <x:c r="D68" s="21" t="str">
-        <x:v>4:03 PM</x:v>
-      </x:c>
-      <x:c r="E68" s="21" t="str">
-        <x:v>4:05 PM</x:v>
-      </x:c>
-      <x:c r="F68" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G68" s="21"/>
-    </x:row>
-    <x:row r="69" ht="25" customHeight="1">
-      <x:c r="A69" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B69" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C69" s="18"/>
-      <x:c r="D69" s="18" t="str">
-        <x:v>4:05 PM</x:v>
-      </x:c>
-      <x:c r="E69" s="18" t="str">
-        <x:v>4:07 PM</x:v>
-      </x:c>
-      <x:c r="F69" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G69" s="18"/>
-    </x:row>
-    <x:row r="70" ht="25" customHeight="1">
-      <x:c r="A70" s="21" t="str">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B70" s="22" t="str">
-        <x:v>Steel Swarm: SURVIVOR</x:v>
-      </x:c>
-      <x:c r="C70" s="21" t="str">
-        <x:v>Clay Token Game Studio, Inc.</x:v>
-      </x:c>
-      <x:c r="D70" s="21" t="str">
-        <x:v>4:07 PM</x:v>
-      </x:c>
-      <x:c r="E70" s="21" t="str">
-        <x:v>4:13 PM</x:v>
-      </x:c>
-      <x:c r="F70" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G70" s="21"/>
-    </x:row>
-    <x:row r="71" ht="25" customHeight="1">
-      <x:c r="A71" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B71" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C71" s="18"/>
-      <x:c r="D71" s="18" t="str">
-        <x:v>4:13 PM</x:v>
-      </x:c>
-      <x:c r="E71" s="18" t="str">
-        <x:v>4:15 PM</x:v>
-      </x:c>
-      <x:c r="F71" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G71" s="18"/>
-    </x:row>
-    <x:row r="72" ht="25" customHeight="1">
-      <x:c r="A72" s="21" t="str">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B72" s="22" t="str">
-        <x:v>Super Choppy</x:v>
-      </x:c>
-      <x:c r="C72" s="21" t="str">
-        <x:v>Sumoshell Bombfunk</x:v>
-      </x:c>
-      <x:c r="D72" s="21" t="str">
-        <x:v>4:15 PM</x:v>
-      </x:c>
-      <x:c r="E72" s="21" t="str">
-        <x:v>4:21 PM</x:v>
-      </x:c>
-      <x:c r="F72" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G72" s="21"/>
-    </x:row>
-    <x:row r="73" ht="25" customHeight="1">
-      <x:c r="A73" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B73" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C73" s="18"/>
-      <x:c r="D73" s="18" t="str">
-        <x:v>4:21 PM</x:v>
-      </x:c>
-      <x:c r="E73" s="18" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="F73" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G73" s="18"/>
-    </x:row>
-    <x:row r="74" ht="25" customHeight="1">
-      <x:c r="A74" s="21" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B74" s="22" t="str">
-        <x:v>Telera</x:v>
-      </x:c>
-      <x:c r="C74" s="21" t="str">
-        <x:v>Entropico</x:v>
-      </x:c>
-      <x:c r="D74" s="21" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="E74" s="21" t="str">
-        <x:v>4:29 PM</x:v>
-      </x:c>
-      <x:c r="F74" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G74" s="21"/>
-    </x:row>
-    <x:row r="75" ht="25" customHeight="1">
-      <x:c r="A75" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B75" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C75" s="18"/>
-      <x:c r="D75" s="18" t="str">
-        <x:v>4:29 PM</x:v>
-      </x:c>
-      <x:c r="E75" s="18" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="F75" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G75" s="18"/>
-    </x:row>
-    <x:row r="76" ht="25" customHeight="1">
-      <x:c r="A76" s="21" t="str">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B76" s="22" t="str">
-        <x:v>The Assessment</x:v>
-      </x:c>
-      <x:c r="C76" s="21" t="str">
-        <x:v>Miga Games</x:v>
-      </x:c>
-      <x:c r="D76" s="21" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="E76" s="21" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="F76" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G76" s="21"/>
-    </x:row>
-    <x:row r="77" ht="25" customHeight="1">
-      <x:c r="A77" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B77" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C77" s="18"/>
-      <x:c r="D77" s="18" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="E77" s="18" t="str">
-        <x:v>4:39 PM</x:v>
-      </x:c>
-      <x:c r="F77" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G77" s="18"/>
-    </x:row>
-    <x:row r="78" ht="25" customHeight="1">
-      <x:c r="A78" s="21" t="str">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B78" s="22" t="str">
-        <x:v>TileShire</x:v>
-      </x:c>
-      <x:c r="C78" s="21" t="str">
-        <x:v>Boss Blob</x:v>
-      </x:c>
-      <x:c r="D78" s="21" t="str">
-        <x:v>4:39 PM</x:v>
-      </x:c>
-      <x:c r="E78" s="21" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="F78" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G78" s="21"/>
-    </x:row>
-    <x:row r="79" ht="25" customHeight="1">
-      <x:c r="A79" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B79" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C79" s="18"/>
-      <x:c r="D79" s="18" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="E79" s="18" t="str">
-        <x:v>4:47 PM</x:v>
-      </x:c>
-      <x:c r="F79" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G79" s="18"/>
-    </x:row>
-    <x:row r="80" ht="25" customHeight="1">
-      <x:c r="A80" s="21" t="str">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B80" s="22" t="str">
-        <x:v>Tower Lab</x:v>
-      </x:c>
-      <x:c r="C80" s="21" t="str">
-        <x:v>Play Tug Studio</x:v>
-      </x:c>
-      <x:c r="D80" s="21" t="str">
-        <x:v>4:47 PM</x:v>
-      </x:c>
-      <x:c r="E80" s="21" t="str">
-        <x:v>4:53 PM</x:v>
-      </x:c>
-      <x:c r="F80" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G80" s="21"/>
-    </x:row>
-    <x:row r="81" ht="25" customHeight="1">
-      <x:c r="A81" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B81" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C81" s="18"/>
-      <x:c r="D81" s="18" t="str">
-        <x:v>4:53 PM</x:v>
-      </x:c>
-      <x:c r="E81" s="18" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="F81" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G81" s="18"/>
-    </x:row>
-    <x:row r="82" ht="25" customHeight="1">
-      <x:c r="A82" s="24" t="str">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B82" s="24" t="str">
-        <x:v>Tricky and the Dream Caster</x:v>
-      </x:c>
-      <x:c r="C82" s="24" t="str">
-        <x:v>PossQueen</x:v>
-      </x:c>
-      <x:c r="D82" s="24" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="E82" s="24" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="F82" s="24" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G82" s="24"/>
-    </x:row>
-    <x:row r="83" ht="25" customHeight="1">
-      <x:c r="A83" s="21" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B83" s="22" t="str">
-        <x:v>Seattle Indies / Sponsor Ad Read</x:v>
-      </x:c>
-      <x:c r="C83" s="21" t="str">
-        <x:v>Sponsor copy pending</x:v>
-      </x:c>
-      <x:c r="D83" s="21" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="E83" s="21" t="str">
-        <x:v>5:03 PM</x:v>
-      </x:c>
-      <x:c r="F83" s="21" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G83" s="21"/>
-    </x:row>
-    <x:row r="84" ht="25" customHeight="1">
-      <x:c r="A84" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B84" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C84" s="18"/>
-      <x:c r="D84" s="18" t="str">
-        <x:v>5:03 PM</x:v>
-      </x:c>
-      <x:c r="E84" s="18" t="str">
-        <x:v>5:05 PM</x:v>
-      </x:c>
-      <x:c r="F84" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G84" s="18"/>
-    </x:row>
-    <x:row r="85" ht="25" customHeight="1">
-      <x:c r="A85" s="21" t="str">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B85" s="22" t="str">
-        <x:v>Turning Manor</x:v>
-      </x:c>
-      <x:c r="C85" s="21" t="str">
-        <x:v>Sabbatical Games</x:v>
-      </x:c>
-      <x:c r="D85" s="21" t="str">
-        <x:v>5:05 PM</x:v>
-      </x:c>
-      <x:c r="E85" s="21" t="str">
-        <x:v>5:11 PM</x:v>
-      </x:c>
-      <x:c r="F85" s="21" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G85" s="21"/>
-    </x:row>
-    <x:row r="86" ht="25" customHeight="1">
-      <x:c r="A86" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B86" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C86" s="18"/>
-      <x:c r="D86" s="18" t="str">
-        <x:v>5:11 PM</x:v>
-      </x:c>
-      <x:c r="E86" s="18" t="str">
-        <x:v>5:13 PM</x:v>
-      </x:c>
-      <x:c r="F86" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G86" s="18"/>
-    </x:row>
-    <x:row r="87" ht="25" customHeight="1">
-      <x:c r="A87" s="21" t="str">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B87" s="22" t="str">
-        <x:v>We Need An Army</x:v>
-      </x:c>
-      <x:c r="C87" s="21" t="str">
-        <x:v>Elder Bear Games</x:v>
-      </x:c>
-      <x:c r="D87" s="21" t="str">
-        <x:v>5:13 PM</x:v>
-      </x:c>
-      <x:c r="E87" s="21" t="str">
-        <x:v>5:19 PM</x:v>
-      </x:c>
-      <x:c r="F87" s="21" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G87" s="21"/>
-    </x:row>
-    <x:row r="88" ht="25" customHeight="1">
-      <x:c r="A88" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B88" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C88" s="18"/>
-      <x:c r="D88" s="18" t="str">
-        <x:v>5:19 PM</x:v>
-      </x:c>
-      <x:c r="E88" s="18" t="str">
-        <x:v>5:21 PM</x:v>
-      </x:c>
-      <x:c r="F88" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G88" s="18"/>
-    </x:row>
-    <x:row r="89" ht="25" customHeight="1">
-      <x:c r="A89" s="21" t="str">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B89" s="22" t="str">
-        <x:v>WILL: Follow The Light</x:v>
-      </x:c>
-      <x:c r="C89" s="21" t="str">
-        <x:v>TomorrowHead Studio</x:v>
-      </x:c>
-      <x:c r="D89" s="21" t="str">
-        <x:v>5:21 PM</x:v>
-      </x:c>
-      <x:c r="E89" s="21" t="str">
-        <x:v>5:27 PM</x:v>
-      </x:c>
-      <x:c r="F89" s="21" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G89" s="21"/>
-    </x:row>
-    <x:row r="90" ht="25" customHeight="1">
-      <x:c r="A90" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B90" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C90" s="18"/>
-      <x:c r="D90" s="18" t="str">
-        <x:v>5:27 PM</x:v>
-      </x:c>
-      <x:c r="E90" s="18" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="F90" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G90" s="18"/>
-    </x:row>
-    <x:row r="91" ht="25" customHeight="1">
-      <x:c r="A91" s="21" t="str">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B91" s="22" t="str">
-        <x:v>Wrestle Story</x:v>
-      </x:c>
-      <x:c r="C91" s="21" t="str">
-        <x:v>Tic Toc Games</x:v>
-      </x:c>
-      <x:c r="D91" s="21" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="E91" s="21" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="F91" s="21" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G91" s="21"/>
-    </x:row>
-    <x:row r="92" ht="25" customHeight="1">
-      <x:c r="A92" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B92" s="23" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C92" s="18"/>
-      <x:c r="D92" s="18" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="E92" s="18" t="str">
-        <x:v>5:37 PM</x:v>
-      </x:c>
-      <x:c r="F92" s="18" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G92" s="18"/>
-    </x:row>
-    <x:row r="93" ht="25" customHeight="1">
-      <x:c r="A93" s="21" t="str">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B93" s="22" t="str">
-        <x:v>Hit &amp; Haunted</x:v>
-      </x:c>
-      <x:c r="C93" s="21" t="str">
-        <x:v>Amnesiac Ghost</x:v>
-      </x:c>
-      <x:c r="D93" s="21" t="str">
-        <x:v>5:37 PM</x:v>
-      </x:c>
-      <x:c r="E93" s="21" t="str">
-        <x:v>5:43 PM</x:v>
-      </x:c>
-      <x:c r="F93" s="21" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G93" s="21"/>
-    </x:row>
-    <x:row r="94" ht="25" customHeight="1">
-      <x:c r="A94" s="25" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B94" s="25" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C94" s="25"/>
-      <x:c r="D94" s="25" t="str">
-        <x:v>5:43 PM</x:v>
-      </x:c>
-      <x:c r="E94" s="25" t="str">
-        <x:v>5:45 PM</x:v>
-      </x:c>
-      <x:c r="F94" s="25" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G94" s="25"/>
-    </x:row>
-    <x:row r="95">
-      <x:c r="A95" t="str">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B95" t="str">
-        <x:v>Closing / Thank You</x:v>
-      </x:c>
-      <x:c r="C95" t="str">
-        <x:v>Seattle Indies</x:v>
-      </x:c>
-      <x:c r="D95" t="str">
-        <x:v>5:45 PM</x:v>
-      </x:c>
-      <x:c r="E95" t="str">
-        <x:v>5:50 PM</x:v>
-      </x:c>
-      <x:c r="F95" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G95"/>
+      <x:c r="D96" s="74" t="str">
+        <x:v>5:55 PM</x:v>
+      </x:c>
+      <x:c r="E96" s="74" t="str">
+        <x:v>6:05 PM</x:v>
+      </x:c>
+      <x:c r="F96" s="74" t="str">
+        <x:v>All Hosts</x:v>
+      </x:c>
+      <x:c r="G96" s="75" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2466,72 +2868,72 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="9" t="inlineStr">
+      <x:c r="A3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Name</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="9" t="inlineStr">
+      <x:c r="B3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer / Publisher</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="9" t="inlineStr">
+      <x:c r="C3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Platforms</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="9" t="inlineStr">
+      <x:c r="D3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Display Platforms</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" s="9" t="inlineStr">
+      <x:c r="E3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Availability</x:t>
         </x:is>
       </x:c>
-      <x:c r="F3" s="9" t="inlineStr">
+      <x:c r="F3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Release</x:t>
         </x:is>
       </x:c>
-      <x:c r="G3" s="9" t="inlineStr">
+      <x:c r="G3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Demo / Build</x:t>
         </x:is>
       </x:c>
-      <x:c r="H3" s="9" t="inlineStr">
+      <x:c r="H3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Quick Overview</x:t>
         </x:is>
       </x:c>
-      <x:c r="I3" s="9" t="inlineStr">
+      <x:c r="I3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Full Description</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" s="9" t="inlineStr">
+      <x:c r="J3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Official URL</x:t>
         </x:is>
       </x:c>
-      <x:c r="K3" s="9" t="inlineStr">
+      <x:c r="K3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Steam App ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="L3" s="9" t="inlineStr">
+      <x:c r="L3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">YouTube Video ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="M3" s="9" t="inlineStr">
+      <x:c r="M3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Media Slug</x:t>
         </x:is>
       </x:c>
-      <x:c r="N3" s="9" t="inlineStr">
+      <x:c r="N3" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Media Folder</x:t>
         </x:is>
@@ -5487,6 +5889,50 @@
         <x:is>
           <x:t xml:space="preserve">wrestlestory</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>Project Cradle</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>ShazySoft</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>PC, Steam, itch.io</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>Steam, itch.io</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Not yet released</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>Demo available on Steam and itch.io</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>A fast momentum platformer starring a nimble robotic kangaroo built for speed, aerial tricks, and exploration.</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>A momentum-based action platformer from ShazySoft. Players control HelperBody, a robotic kangaroo search-and-rescue unit, and build speed by riding slopes, wall-jumping, grinding, bursting, and redirecting momentum through mysterious underground facilities while searching for humanity.</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>https://store.steampowered.com/app/2757950/Project_Cradle/</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>2757950</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>0_2wcoYW8gA</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>projectcradle</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>projectcradle</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update run of show host assignments
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run of Show" sheetId="1" r:id="R4e23978f9ebc43e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="descriptions" sheetId="2" r:id="Rde4e19047314433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run of Show" sheetId="1" r:id="R0dee3d8391f54f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="descriptions" sheetId="2" r:id="R1e484a3aa35040f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="18">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -118,8 +118,44 @@
       <x:color rgb="FF315D26"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFC2410C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF7445C7"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF66616E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5B2B82"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF245477"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF315D26"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -174,6 +210,51 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B1B25"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF30203F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7445C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F2F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEADCF4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F6D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -364,7 +445,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="77">
+  <x:cellXfs count="104">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -554,6 +635,83 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="17" fillId="20" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="24" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="24" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="24" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="26" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="26" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="26" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="26" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="28" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="29" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="29" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -836,30 +994,30 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="34" t="str">
+      <x:c r="A1" s="77" t="str">
         <x:v>Seattle Indies Expo - SIX 2026 | Run of Show</x:v>
       </x:c>
-      <x:c r="B1" s="34"/>
-      <x:c r="C1" s="34"/>
-      <x:c r="D1" s="34"/>
-      <x:c r="E1" s="34"/>
-      <x:c r="F1" s="34"/>
-      <x:c r="G1" s="34"/>
+      <x:c r="B1" s="77"/>
+      <x:c r="C1" s="77"/>
+      <x:c r="D1" s="77"/>
+      <x:c r="E1" s="77"/>
+      <x:c r="F1" s="77"/>
+      <x:c r="G1" s="77"/>
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
-      <x:c r="A2" s="36" t="str">
+      <x:c r="A2" s="78" t="str">
         <x:v>Run of Show - Production Schedule</x:v>
       </x:c>
-      <x:c r="B2" s="36"/>
-      <x:c r="C2" s="36"/>
-      <x:c r="D2" s="36"/>
-      <x:c r="E2" s="36"/>
-      <x:c r="F2" s="36"/>
-      <x:c r="G2" s="36"/>
+      <x:c r="B2" s="78"/>
+      <x:c r="C2" s="78"/>
+      <x:c r="D2" s="78"/>
+      <x:c r="E2" s="78"/>
+      <x:c r="F2" s="78"/>
+      <x:c r="G2" s="78"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="38" t="str">
-        <x:v>Host A = Stephazoid | Host B = AbdallahSmash | Host C = MacnCheesep1z | Host D = Rockagoth | Host E = AlchemistJoker</x:v>
+        <x:v>Host A = Unavailable | Host B = AbdallahSmash | Host C = MacnCheesep1z | Host D = Rockagoth | Host E = AlchemistJoker</x:v>
       </x:c>
       <x:c r="B3" s="39"/>
       <x:c r="C3" s="39"/>
@@ -869,1959 +1027,1959 @@
       <x:c r="G3" s="39"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="41" t="str">
+      <x:c r="A4" s="79" t="str">
         <x:v>SEG</x:v>
       </x:c>
-      <x:c r="B4" s="41" t="str">
+      <x:c r="B4" s="79" t="str">
         <x:v>GAME / BREAK</x:v>
       </x:c>
-      <x:c r="C4" s="41" t="str">
+      <x:c r="C4" s="79" t="str">
         <x:v>DEVELOPER / PUBLISHER</x:v>
       </x:c>
-      <x:c r="D4" s="41" t="str">
+      <x:c r="D4" s="79" t="str">
         <x:v>START</x:v>
       </x:c>
-      <x:c r="E4" s="41" t="str">
+      <x:c r="E4" s="79" t="str">
         <x:v>END</x:v>
       </x:c>
-      <x:c r="F4" s="41" t="str">
+      <x:c r="F4" s="79" t="str">
         <x:v>HOST</x:v>
       </x:c>
-      <x:c r="G4" s="41" t="str">
+      <x:c r="G4" s="79" t="str">
         <x:v>PRODUCTION NOTES</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="53" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B5" s="56" t="str">
+      <x:c r="A5" s="80" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B5" s="83" t="str">
         <x:v>SIX Hype Hour</x:v>
       </x:c>
-      <x:c r="C5" s="54" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Seattle Indies</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>10:00 AM</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>12:00 PM</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Prerecorded</x:v>
       </x:c>
-      <x:c r="G5" s="55" t="str"/>
+      <x:c r="G5" s="82" t="str"/>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
-      <x:c r="A6" s="57" t="str">
+      <x:c r="A6" s="84" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="60" t="str">
+      <x:c r="B6" s="87" t="str">
         <x:v>Tricky and the Dream Caster</x:v>
       </x:c>
-      <x:c r="C6" s="58" t="str">
+      <x:c r="C6" s="85" t="str">
         <x:v>PossQueen · Booth L27</x:v>
       </x:c>
-      <x:c r="D6" s="58" t="str">
+      <x:c r="D6" s="85" t="str">
         <x:v>12:00 PM</x:v>
       </x:c>
-      <x:c r="E6" s="58" t="str">
+      <x:c r="E6" s="85" t="str">
         <x:v>12:06 PM</x:v>
       </x:c>
-      <x:c r="F6" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G6" s="59" t="str"/>
+      <x:c r="F6" s="85" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G6" s="86" t="str"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B7" s="64" t="str">
+      <x:c r="A7" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B7" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C7" s="62" t="str">
+      <x:c r="C7" s="89" t="str">
         <x:v>Block A</x:v>
       </x:c>
-      <x:c r="D7" s="62" t="str">
+      <x:c r="D7" s="89" t="str">
         <x:v>12:06 PM</x:v>
       </x:c>
-      <x:c r="E7" s="62" t="str">
+      <x:c r="E7" s="89" t="str">
         <x:v>12:07 PM</x:v>
       </x:c>
-      <x:c r="F7" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G7" s="63" t="str"/>
+      <x:c r="F7" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G7" s="90" t="str"/>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
-      <x:c r="A8" s="57" t="str">
+      <x:c r="A8" s="84" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B8" s="60" t="str">
+      <x:c r="B8" s="87" t="str">
         <x:v>TileShire</x:v>
       </x:c>
-      <x:c r="C8" s="58" t="str">
+      <x:c r="C8" s="85" t="str">
         <x:v>Boss Blob · Booth L28</x:v>
       </x:c>
-      <x:c r="D8" s="58" t="str">
+      <x:c r="D8" s="85" t="str">
         <x:v>12:07 PM</x:v>
       </x:c>
-      <x:c r="E8" s="58" t="str">
+      <x:c r="E8" s="85" t="str">
         <x:v>12:13 PM</x:v>
       </x:c>
-      <x:c r="F8" s="58" t="str">
+      <x:c r="F8" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G8" s="59" t="str"/>
+      <x:c r="G8" s="86" t="str"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
-      <x:c r="A9" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B9" s="64" t="str">
+      <x:c r="A9" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B9" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C9" s="62" t="str">
+      <x:c r="C9" s="89" t="str">
         <x:v>Block A</x:v>
       </x:c>
-      <x:c r="D9" s="62" t="str">
+      <x:c r="D9" s="89" t="str">
         <x:v>12:13 PM</x:v>
       </x:c>
-      <x:c r="E9" s="62" t="str">
+      <x:c r="E9" s="89" t="str">
         <x:v>12:14 PM</x:v>
       </x:c>
-      <x:c r="F9" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G9" s="63" t="str"/>
+      <x:c r="F9" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G9" s="90" t="str"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="57" t="str">
+      <x:c r="A10" s="84" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B10" s="60" t="str">
+      <x:c r="B10" s="87" t="str">
         <x:v>Wrestle Story</x:v>
       </x:c>
-      <x:c r="C10" s="58" t="str">
+      <x:c r="C10" s="85" t="str">
         <x:v>Tic Toc Games · Booth L29</x:v>
       </x:c>
-      <x:c r="D10" s="58" t="str">
+      <x:c r="D10" s="85" t="str">
         <x:v>12:14 PM</x:v>
       </x:c>
-      <x:c r="E10" s="58" t="str">
+      <x:c r="E10" s="85" t="str">
         <x:v>12:20 PM</x:v>
       </x:c>
-      <x:c r="F10" s="58" t="str">
+      <x:c r="F10" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G10" s="59" t="str"/>
+      <x:c r="G10" s="86" t="str"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B11" s="64" t="str">
+      <x:c r="A11" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B11" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C11" s="62" t="str">
+      <x:c r="C11" s="89" t="str">
         <x:v>Block A</x:v>
       </x:c>
-      <x:c r="D11" s="62" t="str">
+      <x:c r="D11" s="89" t="str">
         <x:v>12:20 PM</x:v>
       </x:c>
-      <x:c r="E11" s="62" t="str">
+      <x:c r="E11" s="89" t="str">
         <x:v>12:21 PM</x:v>
       </x:c>
-      <x:c r="F11" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G11" s="63" t="str"/>
+      <x:c r="F11" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G11" s="90" t="str"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="57" t="str">
+      <x:c r="A12" s="84" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B12" s="60" t="str">
+      <x:c r="B12" s="87" t="str">
         <x:v>Breach Of Contract</x:v>
       </x:c>
-      <x:c r="C12" s="58" t="str">
+      <x:c r="C12" s="85" t="str">
         <x:v>Fern Sprout Studios · Booth L30</x:v>
       </x:c>
-      <x:c r="D12" s="58" t="str">
+      <x:c r="D12" s="85" t="str">
         <x:v>12:21 PM</x:v>
       </x:c>
-      <x:c r="E12" s="58" t="str">
+      <x:c r="E12" s="85" t="str">
         <x:v>12:27 PM</x:v>
       </x:c>
-      <x:c r="F12" s="58" t="str">
+      <x:c r="F12" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G12" s="59" t="str"/>
+      <x:c r="G12" s="86" t="str"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B13" s="64" t="str">
+      <x:c r="A13" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B13" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C13" s="62" t="str">
+      <x:c r="C13" s="89" t="str">
         <x:v>Block A</x:v>
       </x:c>
-      <x:c r="D13" s="62" t="str">
+      <x:c r="D13" s="89" t="str">
         <x:v>12:27 PM</x:v>
       </x:c>
-      <x:c r="E13" s="62" t="str">
+      <x:c r="E13" s="89" t="str">
         <x:v>12:28 PM</x:v>
       </x:c>
-      <x:c r="F13" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G13" s="63" t="str"/>
+      <x:c r="F13" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G13" s="90" t="str"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
-      <x:c r="A14" s="57" t="str">
+      <x:c r="A14" s="84" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B14" s="60" t="str">
+      <x:c r="B14" s="87" t="str">
         <x:v>Dungeon Bodega Simulator</x:v>
       </x:c>
-      <x:c r="C14" s="58" t="str">
+      <x:c r="C14" s="85" t="str">
         <x:v>Alien Fruit Games · Booth L31</x:v>
       </x:c>
-      <x:c r="D14" s="58" t="str">
+      <x:c r="D14" s="85" t="str">
         <x:v>12:28 PM</x:v>
       </x:c>
-      <x:c r="E14" s="58" t="str">
+      <x:c r="E14" s="85" t="str">
         <x:v>12:34 PM</x:v>
       </x:c>
-      <x:c r="F14" s="58" t="str">
+      <x:c r="F14" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G14" s="59" t="str"/>
+      <x:c r="G14" s="86" t="str"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B15" s="64" t="str">
+      <x:c r="A15" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B15" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C15" s="62" t="str">
+      <x:c r="C15" s="89" t="str">
         <x:v>Block A</x:v>
       </x:c>
-      <x:c r="D15" s="62" t="str">
+      <x:c r="D15" s="89" t="str">
         <x:v>12:34 PM</x:v>
       </x:c>
-      <x:c r="E15" s="62" t="str">
+      <x:c r="E15" s="89" t="str">
         <x:v>12:35 PM</x:v>
       </x:c>
-      <x:c r="F15" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G15" s="63" t="str"/>
+      <x:c r="F15" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G15" s="90" t="str"/>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B16" s="68" t="str">
+      <x:c r="A16" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B16" s="95" t="str">
         <x:v>DigiPen Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C16" s="66" t="str">
+      <x:c r="C16" s="93" t="str">
         <x:v>Sponsor segment · L01</x:v>
       </x:c>
-      <x:c r="D16" s="66" t="str">
+      <x:c r="D16" s="93" t="str">
         <x:v>12:35 PM</x:v>
       </x:c>
-      <x:c r="E16" s="66" t="str">
+      <x:c r="E16" s="93" t="str">
         <x:v>12:45 PM</x:v>
       </x:c>
-      <x:c r="F16" s="66" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G16" s="67" t="str"/>
+      <x:c r="F16" s="93" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G16" s="94" t="str"/>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="57" t="str">
+      <x:c r="A17" s="84" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B17" s="60" t="str">
+      <x:c r="B17" s="87" t="str">
         <x:v>SCP: Antimemetics Division</x:v>
       </x:c>
-      <x:c r="C17" s="58" t="str">
+      <x:c r="C17" s="85" t="str">
         <x:v>Quadrant Five · Booth L22</x:v>
       </x:c>
-      <x:c r="D17" s="58" t="str">
+      <x:c r="D17" s="85" t="str">
         <x:v>12:45 PM</x:v>
       </x:c>
-      <x:c r="E17" s="58" t="str">
+      <x:c r="E17" s="85" t="str">
         <x:v>12:51 PM</x:v>
       </x:c>
-      <x:c r="F17" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str"/>
+      <x:c r="F17" s="85" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G17" s="86" t="str"/>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B18" s="64" t="str">
+      <x:c r="A18" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B18" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C18" s="62" t="str">
+      <x:c r="C18" s="89" t="str">
         <x:v>Block B</x:v>
       </x:c>
-      <x:c r="D18" s="62" t="str">
+      <x:c r="D18" s="89" t="str">
         <x:v>12:51 PM</x:v>
       </x:c>
-      <x:c r="E18" s="62" t="str">
+      <x:c r="E18" s="89" t="str">
         <x:v>12:52 PM</x:v>
       </x:c>
-      <x:c r="F18" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G18" s="63" t="str"/>
+      <x:c r="F18" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G18" s="90" t="str"/>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="57" t="str">
+      <x:c r="A19" s="84" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B19" s="60" t="str">
+      <x:c r="B19" s="87" t="str">
         <x:v>Manafinder II</x:v>
       </x:c>
-      <x:c r="C19" s="58" t="str">
+      <x:c r="C19" s="85" t="str">
         <x:v>Wolfsden LLC · Booth L23</x:v>
       </x:c>
-      <x:c r="D19" s="58" t="str">
+      <x:c r="D19" s="85" t="str">
         <x:v>12:52 PM</x:v>
       </x:c>
-      <x:c r="E19" s="58" t="str">
+      <x:c r="E19" s="85" t="str">
         <x:v>12:58 PM</x:v>
       </x:c>
-      <x:c r="F19" s="58" t="str">
+      <x:c r="F19" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G19" s="59" t="str"/>
+      <x:c r="G19" s="86" t="str"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B20" s="64" t="str">
+      <x:c r="A20" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B20" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C20" s="62" t="str">
+      <x:c r="C20" s="89" t="str">
         <x:v>Block B</x:v>
       </x:c>
-      <x:c r="D20" s="62" t="str">
+      <x:c r="D20" s="89" t="str">
         <x:v>12:58 PM</x:v>
       </x:c>
-      <x:c r="E20" s="62" t="str">
+      <x:c r="E20" s="89" t="str">
         <x:v>12:59 PM</x:v>
       </x:c>
-      <x:c r="F20" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G20" s="63" t="str"/>
+      <x:c r="F20" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G20" s="90" t="str"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="57" t="str">
+      <x:c r="A21" s="84" t="str">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B21" s="60" t="str">
+      <x:c r="B21" s="87" t="str">
         <x:v>Malice In Wonderland</x:v>
       </x:c>
-      <x:c r="C21" s="58" t="str">
+      <x:c r="C21" s="85" t="str">
         <x:v>Slyglass Games · Booth L24</x:v>
       </x:c>
-      <x:c r="D21" s="58" t="str">
+      <x:c r="D21" s="85" t="str">
         <x:v>12:59 PM</x:v>
       </x:c>
-      <x:c r="E21" s="58" t="str">
+      <x:c r="E21" s="85" t="str">
         <x:v>1:05 PM</x:v>
       </x:c>
-      <x:c r="F21" s="58" t="str">
+      <x:c r="F21" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G21" s="59" t="str"/>
+      <x:c r="G21" s="86" t="str"/>
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B22" s="64" t="str">
+      <x:c r="A22" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B22" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C22" s="62" t="str">
+      <x:c r="C22" s="89" t="str">
         <x:v>Block B</x:v>
       </x:c>
-      <x:c r="D22" s="62" t="str">
+      <x:c r="D22" s="89" t="str">
         <x:v>1:05 PM</x:v>
       </x:c>
-      <x:c r="E22" s="62" t="str">
+      <x:c r="E22" s="89" t="str">
         <x:v>1:06 PM</x:v>
       </x:c>
-      <x:c r="F22" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G22" s="63" t="str"/>
+      <x:c r="F22" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G22" s="90" t="str"/>
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="57" t="str">
+      <x:c r="A23" s="84" t="str">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B23" s="60" t="str">
+      <x:c r="B23" s="87" t="str">
         <x:v>Project Cradle</x:v>
       </x:c>
-      <x:c r="C23" s="58" t="str">
+      <x:c r="C23" s="85" t="str">
         <x:v>ShazySoft · Booth L25</x:v>
       </x:c>
-      <x:c r="D23" s="58" t="str">
+      <x:c r="D23" s="85" t="str">
         <x:v>1:06 PM</x:v>
       </x:c>
-      <x:c r="E23" s="58" t="str">
+      <x:c r="E23" s="85" t="str">
         <x:v>1:12 PM</x:v>
       </x:c>
-      <x:c r="F23" s="58" t="str">
+      <x:c r="F23" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G23" s="59" t="str"/>
+      <x:c r="G23" s="86" t="str"/>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B24" s="64" t="str">
+      <x:c r="A24" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B24" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C24" s="62" t="str">
+      <x:c r="C24" s="89" t="str">
         <x:v>Block B</x:v>
       </x:c>
-      <x:c r="D24" s="62" t="str">
+      <x:c r="D24" s="89" t="str">
         <x:v>1:12 PM</x:v>
       </x:c>
-      <x:c r="E24" s="62" t="str">
+      <x:c r="E24" s="89" t="str">
         <x:v>1:13 PM</x:v>
       </x:c>
-      <x:c r="F24" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G24" s="63" t="str"/>
+      <x:c r="F24" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G24" s="90" t="str"/>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
-      <x:c r="A25" s="57" t="str">
+      <x:c r="A25" s="84" t="str">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B25" s="60" t="str">
+      <x:c r="B25" s="87" t="str">
         <x:v>Diabolocracy</x:v>
       </x:c>
-      <x:c r="C25" s="58" t="str">
+      <x:c r="C25" s="85" t="str">
         <x:v>Chaos Gremlin Games · Booth L26</x:v>
       </x:c>
-      <x:c r="D25" s="58" t="str">
+      <x:c r="D25" s="85" t="str">
         <x:v>1:13 PM</x:v>
       </x:c>
-      <x:c r="E25" s="58" t="str">
+      <x:c r="E25" s="85" t="str">
         <x:v>1:19 PM</x:v>
       </x:c>
-      <x:c r="F25" s="58" t="str">
+      <x:c r="F25" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G25" s="59" t="str"/>
+      <x:c r="G25" s="86" t="str"/>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
-      <x:c r="A26" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B26" s="64" t="str">
+      <x:c r="A26" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B26" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C26" s="62" t="str">
+      <x:c r="C26" s="89" t="str">
         <x:v>Block B</x:v>
       </x:c>
-      <x:c r="D26" s="62" t="str">
+      <x:c r="D26" s="89" t="str">
         <x:v>1:19 PM</x:v>
       </x:c>
-      <x:c r="E26" s="62" t="str">
+      <x:c r="E26" s="89" t="str">
         <x:v>1:20 PM</x:v>
       </x:c>
-      <x:c r="F26" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G26" s="63" t="str"/>
+      <x:c r="F26" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G26" s="90" t="str"/>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
-      <x:c r="A27" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B27" s="68" t="str">
+      <x:c r="A27" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B27" s="95" t="str">
         <x:v>AIE Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C27" s="66" t="str">
+      <x:c r="C27" s="93" t="str">
         <x:v>Sponsor segment · L02</x:v>
       </x:c>
-      <x:c r="D27" s="66" t="str">
+      <x:c r="D27" s="93" t="str">
         <x:v>1:20 PM</x:v>
       </x:c>
-      <x:c r="E27" s="66" t="str">
+      <x:c r="E27" s="93" t="str">
         <x:v>1:30 PM</x:v>
       </x:c>
-      <x:c r="F27" s="66" t="str">
+      <x:c r="F27" s="93" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G27" s="67" t="str"/>
+      <x:c r="G27" s="94" t="str"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="57" t="str">
+      <x:c r="A28" s="84" t="str">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B28" s="60" t="str">
+      <x:c r="B28" s="87" t="str">
         <x:v>Seedborne Soldiers</x:v>
       </x:c>
-      <x:c r="C28" s="58" t="str">
+      <x:c r="C28" s="85" t="str">
         <x:v>Hat Wobble Games · Booth L17</x:v>
       </x:c>
-      <x:c r="D28" s="58" t="str">
+      <x:c r="D28" s="85" t="str">
         <x:v>1:30 PM</x:v>
       </x:c>
-      <x:c r="E28" s="58" t="str">
+      <x:c r="E28" s="85" t="str">
         <x:v>1:36 PM</x:v>
       </x:c>
-      <x:c r="F28" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G28" s="59" t="str"/>
+      <x:c r="F28" s="85" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G28" s="86" t="str"/>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
-      <x:c r="A29" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B29" s="64" t="str">
+      <x:c r="A29" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B29" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C29" s="62" t="str">
+      <x:c r="C29" s="89" t="str">
         <x:v>Block C</x:v>
       </x:c>
-      <x:c r="D29" s="62" t="str">
+      <x:c r="D29" s="89" t="str">
         <x:v>1:36 PM</x:v>
       </x:c>
-      <x:c r="E29" s="62" t="str">
+      <x:c r="E29" s="89" t="str">
         <x:v>1:37 PM</x:v>
       </x:c>
-      <x:c r="F29" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G29" s="63" t="str"/>
+      <x:c r="F29" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G29" s="90" t="str"/>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
-      <x:c r="A30" s="57" t="str">
+      <x:c r="A30" s="84" t="str">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B30" s="60" t="str">
+      <x:c r="B30" s="87" t="str">
         <x:v>Super Choppy</x:v>
       </x:c>
-      <x:c r="C30" s="58" t="str">
+      <x:c r="C30" s="85" t="str">
         <x:v>Sumoshell Bombfunk · Booth L18</x:v>
       </x:c>
-      <x:c r="D30" s="58" t="str">
+      <x:c r="D30" s="85" t="str">
         <x:v>1:37 PM</x:v>
       </x:c>
-      <x:c r="E30" s="58" t="str">
+      <x:c r="E30" s="85" t="str">
         <x:v>1:43 PM</x:v>
       </x:c>
-      <x:c r="F30" s="58" t="str">
+      <x:c r="F30" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G30" s="59" t="str"/>
+      <x:c r="G30" s="86" t="str"/>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
-      <x:c r="A31" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B31" s="64" t="str">
+      <x:c r="A31" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B31" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C31" s="62" t="str">
+      <x:c r="C31" s="89" t="str">
         <x:v>Block C</x:v>
       </x:c>
-      <x:c r="D31" s="62" t="str">
+      <x:c r="D31" s="89" t="str">
         <x:v>1:43 PM</x:v>
       </x:c>
-      <x:c r="E31" s="62" t="str">
+      <x:c r="E31" s="89" t="str">
         <x:v>1:44 PM</x:v>
       </x:c>
-      <x:c r="F31" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G31" s="63" t="str"/>
+      <x:c r="F31" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G31" s="90" t="str"/>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
-      <x:c r="A32" s="57" t="str">
+      <x:c r="A32" s="84" t="str">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B32" s="60" t="str">
+      <x:c r="B32" s="87" t="str">
         <x:v>Dig Too Deep</x:v>
       </x:c>
-      <x:c r="C32" s="58" t="str">
+      <x:c r="C32" s="85" t="str">
         <x:v>Punch Up Games · Booth L19</x:v>
       </x:c>
-      <x:c r="D32" s="58" t="str">
+      <x:c r="D32" s="85" t="str">
         <x:v>1:44 PM</x:v>
       </x:c>
-      <x:c r="E32" s="58" t="str">
+      <x:c r="E32" s="85" t="str">
         <x:v>1:50 PM</x:v>
       </x:c>
-      <x:c r="F32" s="58" t="str">
+      <x:c r="F32" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G32" s="59" t="str"/>
+      <x:c r="G32" s="86" t="str"/>
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
-      <x:c r="A33" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B33" s="64" t="str">
+      <x:c r="A33" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B33" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C33" s="62" t="str">
+      <x:c r="C33" s="89" t="str">
         <x:v>Block C</x:v>
       </x:c>
-      <x:c r="D33" s="62" t="str">
+      <x:c r="D33" s="89" t="str">
         <x:v>1:50 PM</x:v>
       </x:c>
-      <x:c r="E33" s="62" t="str">
+      <x:c r="E33" s="89" t="str">
         <x:v>1:51 PM</x:v>
       </x:c>
-      <x:c r="F33" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G33" s="63" t="str"/>
+      <x:c r="F33" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G33" s="90" t="str"/>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
-      <x:c r="A34" s="57" t="str">
+      <x:c r="A34" s="84" t="str">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B34" s="60" t="str">
+      <x:c r="B34" s="87" t="str">
         <x:v>Nimbit Frontier</x:v>
       </x:c>
-      <x:c r="C34" s="58" t="str">
+      <x:c r="C34" s="85" t="str">
         <x:v>Megasploot · Booth L20</x:v>
       </x:c>
-      <x:c r="D34" s="58" t="str">
+      <x:c r="D34" s="85" t="str">
         <x:v>1:51 PM</x:v>
       </x:c>
-      <x:c r="E34" s="58" t="str">
+      <x:c r="E34" s="85" t="str">
         <x:v>1:57 PM</x:v>
       </x:c>
-      <x:c r="F34" s="58" t="str">
+      <x:c r="F34" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G34" s="59" t="str"/>
+      <x:c r="G34" s="86" t="str"/>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
-      <x:c r="A35" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B35" s="64" t="str">
+      <x:c r="A35" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B35" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C35" s="62" t="str">
+      <x:c r="C35" s="89" t="str">
         <x:v>Block C</x:v>
       </x:c>
-      <x:c r="D35" s="62" t="str">
+      <x:c r="D35" s="89" t="str">
         <x:v>1:57 PM</x:v>
       </x:c>
-      <x:c r="E35" s="62" t="str">
+      <x:c r="E35" s="89" t="str">
         <x:v>1:58 PM</x:v>
       </x:c>
-      <x:c r="F35" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G35" s="63" t="str"/>
+      <x:c r="F35" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G35" s="90" t="str"/>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
-      <x:c r="A36" s="57" t="str">
+      <x:c r="A36" s="84" t="str">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B36" s="60" t="str">
+      <x:c r="B36" s="87" t="str">
         <x:v>We Need An Army</x:v>
       </x:c>
-      <x:c r="C36" s="58" t="str">
+      <x:c r="C36" s="85" t="str">
         <x:v>Elder Bear Games · Booth L21</x:v>
       </x:c>
-      <x:c r="D36" s="58" t="str">
+      <x:c r="D36" s="85" t="str">
         <x:v>1:58 PM</x:v>
       </x:c>
-      <x:c r="E36" s="58" t="str">
+      <x:c r="E36" s="85" t="str">
         <x:v>2:04 PM</x:v>
       </x:c>
-      <x:c r="F36" s="58" t="str">
+      <x:c r="F36" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G36" s="59" t="str"/>
+      <x:c r="G36" s="86" t="str"/>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
-      <x:c r="A37" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B37" s="64" t="str">
+      <x:c r="A37" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B37" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C37" s="62" t="str">
+      <x:c r="C37" s="89" t="str">
         <x:v>Block C</x:v>
       </x:c>
-      <x:c r="D37" s="62" t="str">
+      <x:c r="D37" s="89" t="str">
         <x:v>2:04 PM</x:v>
       </x:c>
-      <x:c r="E37" s="62" t="str">
+      <x:c r="E37" s="89" t="str">
         <x:v>2:05 PM</x:v>
       </x:c>
-      <x:c r="F37" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G37" s="63" t="str"/>
+      <x:c r="F37" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G37" s="90" t="str"/>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
-      <x:c r="A38" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B38" s="68" t="str">
+      <x:c r="A38" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B38" s="95" t="str">
         <x:v>Unity Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C38" s="66" t="str">
+      <x:c r="C38" s="93" t="str">
         <x:v>Sponsor segment · L03</x:v>
       </x:c>
-      <x:c r="D38" s="66" t="str">
+      <x:c r="D38" s="93" t="str">
         <x:v>2:05 PM</x:v>
       </x:c>
-      <x:c r="E38" s="66" t="str">
+      <x:c r="E38" s="93" t="str">
         <x:v>2:15 PM</x:v>
       </x:c>
-      <x:c r="F38" s="66" t="str">
+      <x:c r="F38" s="93" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G38" s="67" t="str"/>
+      <x:c r="G38" s="94" t="str"/>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
-      <x:c r="A39" s="57" t="str">
+      <x:c r="A39" s="84" t="str">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B39" s="60" t="str">
+      <x:c r="B39" s="87" t="str">
         <x:v>Feeding Gooble</x:v>
       </x:c>
-      <x:c r="C39" s="58" t="str">
+      <x:c r="C39" s="85" t="str">
         <x:v>Displacer Labs · Booth L12</x:v>
       </x:c>
-      <x:c r="D39" s="58" t="str">
+      <x:c r="D39" s="85" t="str">
         <x:v>2:15 PM</x:v>
       </x:c>
-      <x:c r="E39" s="58" t="str">
+      <x:c r="E39" s="85" t="str">
         <x:v>2:21 PM</x:v>
       </x:c>
-      <x:c r="F39" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G39" s="59" t="str"/>
+      <x:c r="F39" s="85" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G39" s="86" t="str"/>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
-      <x:c r="A40" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B40" s="64" t="str">
+      <x:c r="A40" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B40" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C40" s="62" t="str">
+      <x:c r="C40" s="89" t="str">
         <x:v>Block D</x:v>
       </x:c>
-      <x:c r="D40" s="62" t="str">
+      <x:c r="D40" s="89" t="str">
         <x:v>2:21 PM</x:v>
       </x:c>
-      <x:c r="E40" s="62" t="str">
+      <x:c r="E40" s="89" t="str">
         <x:v>2:22 PM</x:v>
       </x:c>
-      <x:c r="F40" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G40" s="63" t="str"/>
+      <x:c r="F40" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G40" s="90" t="str"/>
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
-      <x:c r="A41" s="57" t="str">
+      <x:c r="A41" s="84" t="str">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B41" s="60" t="str">
+      <x:c r="B41" s="87" t="str">
         <x:v>BroomSweeper</x:v>
       </x:c>
-      <x:c r="C41" s="58" t="str">
+      <x:c r="C41" s="85" t="str">
         <x:v>BandWidth Games · Booth L13</x:v>
       </x:c>
-      <x:c r="D41" s="58" t="str">
+      <x:c r="D41" s="85" t="str">
         <x:v>2:22 PM</x:v>
       </x:c>
-      <x:c r="E41" s="58" t="str">
+      <x:c r="E41" s="85" t="str">
         <x:v>2:28 PM</x:v>
       </x:c>
-      <x:c r="F41" s="58" t="str">
+      <x:c r="F41" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G41" s="59" t="str"/>
+      <x:c r="G41" s="86" t="str"/>
     </x:row>
     <x:row r="42" ht="20" customHeight="1">
-      <x:c r="A42" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B42" s="64" t="str">
+      <x:c r="A42" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B42" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C42" s="62" t="str">
+      <x:c r="C42" s="89" t="str">
         <x:v>Block D</x:v>
       </x:c>
-      <x:c r="D42" s="62" t="str">
+      <x:c r="D42" s="89" t="str">
         <x:v>2:28 PM</x:v>
       </x:c>
-      <x:c r="E42" s="62" t="str">
+      <x:c r="E42" s="89" t="str">
         <x:v>2:29 PM</x:v>
       </x:c>
-      <x:c r="F42" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G42" s="63" t="str"/>
+      <x:c r="F42" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G42" s="90" t="str"/>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
-      <x:c r="A43" s="57" t="str">
+      <x:c r="A43" s="84" t="str">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B43" s="60" t="str">
+      <x:c r="B43" s="87" t="str">
         <x:v>Fairy Circle</x:v>
       </x:c>
-      <x:c r="C43" s="58" t="str">
+      <x:c r="C43" s="85" t="str">
         <x:v>Play Hooky · Booth L14</x:v>
       </x:c>
-      <x:c r="D43" s="58" t="str">
+      <x:c r="D43" s="85" t="str">
         <x:v>2:29 PM</x:v>
       </x:c>
-      <x:c r="E43" s="58" t="str">
+      <x:c r="E43" s="85" t="str">
         <x:v>2:35 PM</x:v>
       </x:c>
-      <x:c r="F43" s="58" t="str">
+      <x:c r="F43" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G43" s="59" t="str"/>
+      <x:c r="G43" s="86" t="str"/>
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
-      <x:c r="A44" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B44" s="64" t="str">
+      <x:c r="A44" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B44" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C44" s="62" t="str">
+      <x:c r="C44" s="89" t="str">
         <x:v>Block D</x:v>
       </x:c>
-      <x:c r="D44" s="62" t="str">
+      <x:c r="D44" s="89" t="str">
         <x:v>2:35 PM</x:v>
       </x:c>
-      <x:c r="E44" s="62" t="str">
+      <x:c r="E44" s="89" t="str">
         <x:v>2:36 PM</x:v>
       </x:c>
-      <x:c r="F44" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G44" s="63" t="str"/>
+      <x:c r="F44" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G44" s="90" t="str"/>
     </x:row>
     <x:row r="45" ht="20" customHeight="1">
-      <x:c r="A45" s="57" t="str">
+      <x:c r="A45" s="84" t="str">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B45" s="60" t="str">
+      <x:c r="B45" s="87" t="str">
         <x:v>MYRIORAMA</x:v>
       </x:c>
-      <x:c r="C45" s="58" t="str">
+      <x:c r="C45" s="85" t="str">
         <x:v>J&amp;K Games · Booth L15</x:v>
       </x:c>
-      <x:c r="D45" s="58" t="str">
+      <x:c r="D45" s="85" t="str">
         <x:v>2:36 PM</x:v>
       </x:c>
-      <x:c r="E45" s="58" t="str">
+      <x:c r="E45" s="85" t="str">
         <x:v>2:42 PM</x:v>
       </x:c>
-      <x:c r="F45" s="58" t="str">
+      <x:c r="F45" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G45" s="59" t="str"/>
+      <x:c r="G45" s="86" t="str"/>
     </x:row>
     <x:row r="46" ht="20" customHeight="1">
-      <x:c r="A46" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B46" s="64" t="str">
+      <x:c r="A46" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B46" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C46" s="62" t="str">
+      <x:c r="C46" s="89" t="str">
         <x:v>Block D</x:v>
       </x:c>
-      <x:c r="D46" s="62" t="str">
+      <x:c r="D46" s="89" t="str">
         <x:v>2:42 PM</x:v>
       </x:c>
-      <x:c r="E46" s="62" t="str">
+      <x:c r="E46" s="89" t="str">
         <x:v>2:43 PM</x:v>
       </x:c>
-      <x:c r="F46" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G46" s="63" t="str"/>
+      <x:c r="F46" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G46" s="90" t="str"/>
     </x:row>
     <x:row r="47" ht="20" customHeight="1">
-      <x:c r="A47" s="57" t="str">
+      <x:c r="A47" s="84" t="str">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B47" s="60" t="str">
+      <x:c r="B47" s="87" t="str">
         <x:v>Dittori</x:v>
       </x:c>
-      <x:c r="C47" s="58" t="str">
+      <x:c r="C47" s="85" t="str">
         <x:v>Blookerstein · Booth L16</x:v>
       </x:c>
-      <x:c r="D47" s="58" t="str">
+      <x:c r="D47" s="85" t="str">
         <x:v>2:43 PM</x:v>
       </x:c>
-      <x:c r="E47" s="58" t="str">
+      <x:c r="E47" s="85" t="str">
         <x:v>2:49 PM</x:v>
       </x:c>
-      <x:c r="F47" s="58" t="str">
+      <x:c r="F47" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G47" s="59" t="str"/>
+      <x:c r="G47" s="86" t="str"/>
     </x:row>
     <x:row r="48" ht="20" customHeight="1">
-      <x:c r="A48" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B48" s="64" t="str">
+      <x:c r="A48" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B48" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C48" s="62" t="str">
+      <x:c r="C48" s="89" t="str">
         <x:v>Block D</x:v>
       </x:c>
-      <x:c r="D48" s="62" t="str">
+      <x:c r="D48" s="89" t="str">
         <x:v>2:49 PM</x:v>
       </x:c>
-      <x:c r="E48" s="62" t="str">
+      <x:c r="E48" s="89" t="str">
         <x:v>2:50 PM</x:v>
       </x:c>
-      <x:c r="F48" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G48" s="63" t="str"/>
+      <x:c r="F48" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G48" s="90" t="str"/>
     </x:row>
     <x:row r="49" ht="20" customHeight="1">
-      <x:c r="A49" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B49" s="68" t="str">
+      <x:c r="A49" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B49" s="95" t="str">
         <x:v>Forge Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C49" s="66" t="str">
+      <x:c r="C49" s="93" t="str">
         <x:v>Sponsor segment · L05</x:v>
       </x:c>
-      <x:c r="D49" s="66" t="str">
+      <x:c r="D49" s="93" t="str">
         <x:v>2:50 PM</x:v>
       </x:c>
-      <x:c r="E49" s="66" t="str">
+      <x:c r="E49" s="93" t="str">
         <x:v>3:00 PM</x:v>
       </x:c>
-      <x:c r="F49" s="66" t="str">
+      <x:c r="F49" s="93" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G49" s="67" t="str"/>
+      <x:c r="G49" s="94" t="str"/>
     </x:row>
     <x:row r="50" ht="20" customHeight="1">
-      <x:c r="A50" s="57" t="str">
+      <x:c r="A50" s="84" t="str">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B50" s="60" t="str">
+      <x:c r="B50" s="87" t="str">
         <x:v>End of Garbage</x:v>
       </x:c>
-      <x:c r="C50" s="58" t="str">
+      <x:c r="C50" s="85" t="str">
         <x:v>Joshua Rosen (Rakelock LLC) · Booth L35</x:v>
       </x:c>
-      <x:c r="D50" s="58" t="str">
+      <x:c r="D50" s="85" t="str">
         <x:v>3:00 PM</x:v>
       </x:c>
-      <x:c r="E50" s="58" t="str">
+      <x:c r="E50" s="85" t="str">
         <x:v>3:06 PM</x:v>
       </x:c>
-      <x:c r="F50" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G50" s="59" t="str"/>
+      <x:c r="F50" s="85" t="str">
+        <x:v>E</x:v>
+      </x:c>
+      <x:c r="G50" s="86" t="str"/>
     </x:row>
     <x:row r="51" ht="20" customHeight="1">
-      <x:c r="A51" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B51" s="64" t="str">
+      <x:c r="A51" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B51" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C51" s="62" t="str">
+      <x:c r="C51" s="89" t="str">
         <x:v>Block E</x:v>
       </x:c>
-      <x:c r="D51" s="62" t="str">
+      <x:c r="D51" s="89" t="str">
         <x:v>3:06 PM</x:v>
       </x:c>
-      <x:c r="E51" s="62" t="str">
+      <x:c r="E51" s="89" t="str">
         <x:v>3:07 PM</x:v>
       </x:c>
-      <x:c r="F51" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G51" s="63" t="str"/>
+      <x:c r="F51" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G51" s="90" t="str"/>
     </x:row>
     <x:row r="52" ht="20" customHeight="1">
-      <x:c r="A52" s="57" t="str">
+      <x:c r="A52" s="84" t="str">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B52" s="60" t="str">
+      <x:c r="B52" s="87" t="str">
         <x:v>Gravity Goblins</x:v>
       </x:c>
-      <x:c r="C52" s="58" t="str">
+      <x:c r="C52" s="85" t="str">
         <x:v>The Rat Zone · Booth L34</x:v>
       </x:c>
-      <x:c r="D52" s="58" t="str">
+      <x:c r="D52" s="85" t="str">
         <x:v>3:07 PM</x:v>
       </x:c>
-      <x:c r="E52" s="58" t="str">
+      <x:c r="E52" s="85" t="str">
         <x:v>3:13 PM</x:v>
       </x:c>
-      <x:c r="F52" s="58" t="str">
+      <x:c r="F52" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G52" s="59" t="str"/>
+      <x:c r="G52" s="86" t="str"/>
     </x:row>
     <x:row r="53" ht="20" customHeight="1">
-      <x:c r="A53" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B53" s="64" t="str">
+      <x:c r="A53" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B53" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C53" s="62" t="str">
+      <x:c r="C53" s="89" t="str">
         <x:v>Block E</x:v>
       </x:c>
-      <x:c r="D53" s="62" t="str">
+      <x:c r="D53" s="89" t="str">
         <x:v>3:13 PM</x:v>
       </x:c>
-      <x:c r="E53" s="62" t="str">
+      <x:c r="E53" s="89" t="str">
         <x:v>3:14 PM</x:v>
       </x:c>
-      <x:c r="F53" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G53" s="63" t="str"/>
+      <x:c r="F53" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G53" s="90" t="str"/>
     </x:row>
     <x:row r="54" ht="20" customHeight="1">
-      <x:c r="A54" s="57" t="str">
+      <x:c r="A54" s="84" t="str">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B54" s="60" t="str">
+      <x:c r="B54" s="87" t="str">
         <x:v>Creature Kitchen</x:v>
       </x:c>
-      <x:c r="C54" s="58" t="str">
+      <x:c r="C54" s="85" t="str">
         <x:v>The Rat Zone · Booth L33</x:v>
       </x:c>
-      <x:c r="D54" s="58" t="str">
+      <x:c r="D54" s="85" t="str">
         <x:v>3:14 PM</x:v>
       </x:c>
-      <x:c r="E54" s="58" t="str">
+      <x:c r="E54" s="85" t="str">
         <x:v>3:20 PM</x:v>
       </x:c>
-      <x:c r="F54" s="58" t="str">
+      <x:c r="F54" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G54" s="59" t="str"/>
+      <x:c r="G54" s="86" t="str"/>
     </x:row>
     <x:row r="55" ht="20" customHeight="1">
-      <x:c r="A55" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B55" s="64" t="str">
+      <x:c r="A55" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B55" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C55" s="62" t="str">
+      <x:c r="C55" s="89" t="str">
         <x:v>Block E</x:v>
       </x:c>
-      <x:c r="D55" s="62" t="str">
+      <x:c r="D55" s="89" t="str">
         <x:v>3:20 PM</x:v>
       </x:c>
-      <x:c r="E55" s="62" t="str">
+      <x:c r="E55" s="89" t="str">
         <x:v>3:21 PM</x:v>
       </x:c>
-      <x:c r="F55" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G55" s="63" t="str"/>
+      <x:c r="F55" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G55" s="90" t="str"/>
     </x:row>
     <x:row r="56" ht="20" customHeight="1">
-      <x:c r="A56" s="57" t="str">
+      <x:c r="A56" s="84" t="str">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B56" s="60" t="str">
+      <x:c r="B56" s="87" t="str">
         <x:v>Desolus</x:v>
       </x:c>
-      <x:c r="C56" s="58" t="str">
+      <x:c r="C56" s="85" t="str">
         <x:v>Mark J. Mayers · Booth L32</x:v>
       </x:c>
-      <x:c r="D56" s="58" t="str">
+      <x:c r="D56" s="85" t="str">
         <x:v>3:21 PM</x:v>
       </x:c>
-      <x:c r="E56" s="58" t="str">
+      <x:c r="E56" s="85" t="str">
         <x:v>3:27 PM</x:v>
       </x:c>
-      <x:c r="F56" s="58" t="str">
+      <x:c r="F56" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G56" s="59" t="str"/>
+      <x:c r="G56" s="86" t="str"/>
     </x:row>
     <x:row r="57" ht="20" customHeight="1">
-      <x:c r="A57" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B57" s="64" t="str">
+      <x:c r="A57" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B57" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C57" s="62" t="str">
+      <x:c r="C57" s="89" t="str">
         <x:v>Block E</x:v>
       </x:c>
-      <x:c r="D57" s="62" t="str">
+      <x:c r="D57" s="89" t="str">
         <x:v>3:27 PM</x:v>
       </x:c>
-      <x:c r="E57" s="62" t="str">
+      <x:c r="E57" s="89" t="str">
         <x:v>3:28 PM</x:v>
       </x:c>
-      <x:c r="F57" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G57" s="63" t="str"/>
+      <x:c r="F57" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G57" s="90" t="str"/>
     </x:row>
     <x:row r="58" ht="20" customHeight="1">
-      <x:c r="A58" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B58" s="68" t="str">
+      <x:c r="A58" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B58" s="95" t="str">
         <x:v>GeekGirlCon Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C58" s="66" t="str">
+      <x:c r="C58" s="93" t="str">
         <x:v>Sponsor segment · L04</x:v>
       </x:c>
-      <x:c r="D58" s="66" t="str">
+      <x:c r="D58" s="93" t="str">
         <x:v>3:28 PM</x:v>
       </x:c>
-      <x:c r="E58" s="66" t="str">
+      <x:c r="E58" s="93" t="str">
         <x:v>3:35 PM</x:v>
       </x:c>
-      <x:c r="F58" s="66" t="str">
+      <x:c r="F58" s="93" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G58" s="67" t="str"/>
+      <x:c r="G58" s="94" t="str"/>
     </x:row>
     <x:row r="59" ht="20" customHeight="1">
-      <x:c r="A59" s="57" t="str">
+      <x:c r="A59" s="84" t="str">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B59" s="60" t="str">
+      <x:c r="B59" s="87" t="str">
         <x:v>Ascent Rivals</x:v>
       </x:c>
-      <x:c r="C59" s="58" t="str">
+      <x:c r="C59" s="85" t="str">
         <x:v>GENUN Games · Booth L11</x:v>
       </x:c>
-      <x:c r="D59" s="58" t="str">
+      <x:c r="D59" s="85" t="str">
         <x:v>3:35 PM</x:v>
       </x:c>
-      <x:c r="E59" s="58" t="str">
+      <x:c r="E59" s="85" t="str">
         <x:v>3:41 PM</x:v>
       </x:c>
-      <x:c r="F59" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G59" s="59" t="str"/>
+      <x:c r="F59" s="85" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G59" s="86" t="str"/>
     </x:row>
     <x:row r="60" ht="20" customHeight="1">
-      <x:c r="A60" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B60" s="64" t="str">
+      <x:c r="A60" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B60" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C60" s="62" t="str">
+      <x:c r="C60" s="89" t="str">
         <x:v>Block F</x:v>
       </x:c>
-      <x:c r="D60" s="62" t="str">
+      <x:c r="D60" s="89" t="str">
         <x:v>3:41 PM</x:v>
       </x:c>
-      <x:c r="E60" s="62" t="str">
+      <x:c r="E60" s="89" t="str">
         <x:v>3:42 PM</x:v>
       </x:c>
-      <x:c r="F60" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G60" s="63" t="str"/>
+      <x:c r="F60" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G60" s="90" t="str"/>
     </x:row>
     <x:row r="61" ht="20" customHeight="1">
-      <x:c r="A61" s="57" t="str">
+      <x:c r="A61" s="84" t="str">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B61" s="60" t="str">
+      <x:c r="B61" s="87" t="str">
         <x:v>Hamsteria</x:v>
       </x:c>
-      <x:c r="C61" s="58" t="str">
+      <x:c r="C61" s="85" t="str">
         <x:v>2WheelerDev · Booth L10</x:v>
       </x:c>
-      <x:c r="D61" s="58" t="str">
+      <x:c r="D61" s="85" t="str">
         <x:v>3:42 PM</x:v>
       </x:c>
-      <x:c r="E61" s="58" t="str">
+      <x:c r="E61" s="85" t="str">
         <x:v>3:48 PM</x:v>
       </x:c>
-      <x:c r="F61" s="58" t="str">
+      <x:c r="F61" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G61" s="59" t="str"/>
+      <x:c r="G61" s="86" t="str"/>
     </x:row>
     <x:row r="62" ht="20" customHeight="1">
-      <x:c r="A62" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B62" s="64" t="str">
+      <x:c r="A62" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B62" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C62" s="62" t="str">
+      <x:c r="C62" s="89" t="str">
         <x:v>Block F</x:v>
       </x:c>
-      <x:c r="D62" s="62" t="str">
+      <x:c r="D62" s="89" t="str">
         <x:v>3:48 PM</x:v>
       </x:c>
-      <x:c r="E62" s="62" t="str">
+      <x:c r="E62" s="89" t="str">
         <x:v>3:49 PM</x:v>
       </x:c>
-      <x:c r="F62" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G62" s="63" t="str"/>
+      <x:c r="F62" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G62" s="90" t="str"/>
     </x:row>
     <x:row r="63" ht="20" customHeight="1">
-      <x:c r="A63" s="57" t="str">
+      <x:c r="A63" s="84" t="str">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B63" s="60" t="str">
+      <x:c r="B63" s="87" t="str">
         <x:v>Haunted Heist</x:v>
       </x:c>
-      <x:c r="C63" s="58" t="str">
+      <x:c r="C63" s="85" t="str">
         <x:v>autotroph games · Booth L09</x:v>
       </x:c>
-      <x:c r="D63" s="58" t="str">
+      <x:c r="D63" s="85" t="str">
         <x:v>3:49 PM</x:v>
       </x:c>
-      <x:c r="E63" s="58" t="str">
+      <x:c r="E63" s="85" t="str">
         <x:v>3:55 PM</x:v>
       </x:c>
-      <x:c r="F63" s="58" t="str">
+      <x:c r="F63" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G63" s="59" t="str"/>
+      <x:c r="G63" s="86" t="str"/>
     </x:row>
     <x:row r="64" ht="20" customHeight="1">
-      <x:c r="A64" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B64" s="64" t="str">
+      <x:c r="A64" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B64" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C64" s="62" t="str">
+      <x:c r="C64" s="89" t="str">
         <x:v>Block F</x:v>
       </x:c>
-      <x:c r="D64" s="62" t="str">
+      <x:c r="D64" s="89" t="str">
         <x:v>3:55 PM</x:v>
       </x:c>
-      <x:c r="E64" s="62" t="str">
+      <x:c r="E64" s="89" t="str">
         <x:v>3:56 PM</x:v>
       </x:c>
-      <x:c r="F64" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G64" s="63" t="str"/>
+      <x:c r="F64" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G64" s="90" t="str"/>
     </x:row>
     <x:row r="65" ht="20" customHeight="1">
-      <x:c r="A65" s="57" t="str">
+      <x:c r="A65" s="84" t="str">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B65" s="60" t="str">
+      <x:c r="B65" s="87" t="str">
         <x:v>RUNE GUNNER</x:v>
       </x:c>
-      <x:c r="C65" s="58" t="str">
+      <x:c r="C65" s="85" t="str">
         <x:v>False Summit · Booth L08</x:v>
       </x:c>
-      <x:c r="D65" s="58" t="str">
+      <x:c r="D65" s="85" t="str">
         <x:v>3:56 PM</x:v>
       </x:c>
-      <x:c r="E65" s="58" t="str">
+      <x:c r="E65" s="85" t="str">
         <x:v>4:02 PM</x:v>
       </x:c>
-      <x:c r="F65" s="58" t="str">
+      <x:c r="F65" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G65" s="59" t="str"/>
+      <x:c r="G65" s="86" t="str"/>
     </x:row>
     <x:row r="66" ht="20" customHeight="1">
-      <x:c r="A66" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B66" s="64" t="str">
+      <x:c r="A66" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B66" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C66" s="62" t="str">
+      <x:c r="C66" s="89" t="str">
         <x:v>Block F</x:v>
       </x:c>
-      <x:c r="D66" s="62" t="str">
+      <x:c r="D66" s="89" t="str">
         <x:v>4:02 PM</x:v>
       </x:c>
-      <x:c r="E66" s="62" t="str">
+      <x:c r="E66" s="89" t="str">
         <x:v>4:03 PM</x:v>
       </x:c>
-      <x:c r="F66" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G66" s="63" t="str"/>
+      <x:c r="F66" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G66" s="90" t="str"/>
     </x:row>
     <x:row r="67" ht="20" customHeight="1">
-      <x:c r="A67" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B67" s="68" t="str">
+      <x:c r="A67" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B67" s="95" t="str">
         <x:v>11 Bit Studios Sponsor Segment</x:v>
       </x:c>
-      <x:c r="C67" s="66" t="str">
+      <x:c r="C67" s="93" t="str">
         <x:v>Sponsor segment · L06</x:v>
       </x:c>
-      <x:c r="D67" s="66" t="str">
+      <x:c r="D67" s="93" t="str">
         <x:v>4:03 PM</x:v>
       </x:c>
-      <x:c r="E67" s="66" t="str">
+      <x:c r="E67" s="93" t="str">
         <x:v>4:10 PM</x:v>
       </x:c>
-      <x:c r="F67" s="66" t="str">
+      <x:c r="F67" s="93" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G67" s="94" t="str"/>
+    </x:row>
+    <x:row r="68" ht="20" customHeight="1">
+      <x:c r="A68" s="84" t="str">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B68" s="87" t="str">
+        <x:v>Telera</x:v>
+      </x:c>
+      <x:c r="C68" s="85" t="str">
+        <x:v>Entropico · Booth U21</x:v>
+      </x:c>
+      <x:c r="D68" s="85" t="str">
+        <x:v>4:10 PM</x:v>
+      </x:c>
+      <x:c r="E68" s="85" t="str">
+        <x:v>4:16 PM</x:v>
+      </x:c>
+      <x:c r="F68" s="85" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G68" s="86" t="str"/>
+    </x:row>
+    <x:row r="69" ht="20" customHeight="1">
+      <x:c r="A69" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B69" s="91" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C69" s="89" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D69" s="89" t="str">
+        <x:v>4:16 PM</x:v>
+      </x:c>
+      <x:c r="E69" s="89" t="str">
+        <x:v>4:17 PM</x:v>
+      </x:c>
+      <x:c r="F69" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G69" s="90" t="str"/>
+    </x:row>
+    <x:row r="70" ht="20" customHeight="1">
+      <x:c r="A70" s="84" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B70" s="87" t="str">
+        <x:v>Hogen</x:v>
+      </x:c>
+      <x:c r="C70" s="85" t="str">
+        <x:v>Scrappyard Games · Booth U22</x:v>
+      </x:c>
+      <x:c r="D70" s="85" t="str">
+        <x:v>4:17 PM</x:v>
+      </x:c>
+      <x:c r="E70" s="85" t="str">
+        <x:v>4:23 PM</x:v>
+      </x:c>
+      <x:c r="F70" s="85" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G70" s="86" t="str"/>
+    </x:row>
+    <x:row r="71" ht="20" customHeight="1">
+      <x:c r="A71" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B71" s="91" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C71" s="89" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D71" s="89" t="str">
+        <x:v>4:23 PM</x:v>
+      </x:c>
+      <x:c r="E71" s="89" t="str">
+        <x:v>4:24 PM</x:v>
+      </x:c>
+      <x:c r="F71" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G71" s="90" t="str"/>
+    </x:row>
+    <x:row r="72" ht="20" customHeight="1">
+      <x:c r="A72" s="84" t="str">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B72" s="87" t="str">
+        <x:v>WILL: Follow The Light</x:v>
+      </x:c>
+      <x:c r="C72" s="85" t="str">
+        <x:v>TomorrowHead Studio · Booth U23</x:v>
+      </x:c>
+      <x:c r="D72" s="85" t="str">
+        <x:v>4:24 PM</x:v>
+      </x:c>
+      <x:c r="E72" s="85" t="str">
+        <x:v>4:30 PM</x:v>
+      </x:c>
+      <x:c r="F72" s="85" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G72" s="86" t="str"/>
+    </x:row>
+    <x:row r="73" ht="20" customHeight="1">
+      <x:c r="A73" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B73" s="91" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C73" s="89" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D73" s="89" t="str">
+        <x:v>4:30 PM</x:v>
+      </x:c>
+      <x:c r="E73" s="89" t="str">
+        <x:v>4:31 PM</x:v>
+      </x:c>
+      <x:c r="F73" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G73" s="90" t="str"/>
+    </x:row>
+    <x:row r="74" ht="20" customHeight="1">
+      <x:c r="A74" s="84" t="str">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B74" s="87" t="str">
+        <x:v>Turning Manor</x:v>
+      </x:c>
+      <x:c r="C74" s="85" t="str">
+        <x:v>Sabbatical Games · Booth U24</x:v>
+      </x:c>
+      <x:c r="D74" s="85" t="str">
+        <x:v>4:31 PM</x:v>
+      </x:c>
+      <x:c r="E74" s="85" t="str">
+        <x:v>4:37 PM</x:v>
+      </x:c>
+      <x:c r="F74" s="85" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="G74" s="86" t="str"/>
+    </x:row>
+    <x:row r="75" ht="20" customHeight="1">
+      <x:c r="A75" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B75" s="91" t="str">
+        <x:v>Break / Transition</x:v>
+      </x:c>
+      <x:c r="C75" s="89" t="str">
+        <x:v>Block G</x:v>
+      </x:c>
+      <x:c r="D75" s="89" t="str">
+        <x:v>4:37 PM</x:v>
+      </x:c>
+      <x:c r="E75" s="89" t="str">
+        <x:v>4:38 PM</x:v>
+      </x:c>
+      <x:c r="F75" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G75" s="90" t="str"/>
+    </x:row>
+    <x:row r="76" ht="20" customHeight="1">
+      <x:c r="A76" s="84" t="str">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B76" s="87" t="str">
+        <x:v>Steel Swarm: SURVIVOR</x:v>
+      </x:c>
+      <x:c r="C76" s="85" t="str">
+        <x:v>Clay Token Game Studio, Inc. · Booth U25</x:v>
+      </x:c>
+      <x:c r="D76" s="85" t="str">
+        <x:v>4:38 PM</x:v>
+      </x:c>
+      <x:c r="E76" s="85" t="str">
+        <x:v>4:44 PM</x:v>
+      </x:c>
+      <x:c r="F76" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G67" s="67" t="str"/>
-    </x:row>
-    <x:row r="68" ht="20" customHeight="1">
-      <x:c r="A68" s="57" t="str">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B68" s="60" t="str">
-        <x:v>Telera</x:v>
-      </x:c>
-      <x:c r="C68" s="58" t="str">
-        <x:v>Entropico · Booth U21</x:v>
-      </x:c>
-      <x:c r="D68" s="58" t="str">
-        <x:v>4:10 PM</x:v>
-      </x:c>
-      <x:c r="E68" s="58" t="str">
-        <x:v>4:16 PM</x:v>
-      </x:c>
-      <x:c r="F68" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G68" s="59" t="str"/>
-    </x:row>
-    <x:row r="69" ht="20" customHeight="1">
-      <x:c r="A69" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B69" s="64" t="str">
+      <x:c r="G76" s="86" t="str"/>
+    </x:row>
+    <x:row r="77" ht="20" customHeight="1">
+      <x:c r="A77" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B77" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C69" s="62" t="str">
+      <x:c r="C77" s="89" t="str">
         <x:v>Block G</x:v>
       </x:c>
-      <x:c r="D69" s="62" t="str">
-        <x:v>4:16 PM</x:v>
-      </x:c>
-      <x:c r="E69" s="62" t="str">
-        <x:v>4:17 PM</x:v>
-      </x:c>
-      <x:c r="F69" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G69" s="63" t="str"/>
-    </x:row>
-    <x:row r="70" ht="20" customHeight="1">
-      <x:c r="A70" s="57" t="str">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B70" s="60" t="str">
-        <x:v>Hogen</x:v>
-      </x:c>
-      <x:c r="C70" s="58" t="str">
-        <x:v>Scrappyard Games · Booth U22</x:v>
-      </x:c>
-      <x:c r="D70" s="58" t="str">
-        <x:v>4:17 PM</x:v>
-      </x:c>
-      <x:c r="E70" s="58" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="F70" s="58" t="str">
+      <x:c r="D77" s="89" t="str">
+        <x:v>4:44 PM</x:v>
+      </x:c>
+      <x:c r="E77" s="89" t="str">
+        <x:v>4:45 PM</x:v>
+      </x:c>
+      <x:c r="F77" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G77" s="90" t="str"/>
+    </x:row>
+    <x:row r="78" ht="20" customHeight="1">
+      <x:c r="A78" s="92" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B78" s="95" t="str">
+        <x:v>NDVisibility Sponsor Segment</x:v>
+      </x:c>
+      <x:c r="C78" s="93" t="str">
+        <x:v>Sponsor segment · 000</x:v>
+      </x:c>
+      <x:c r="D78" s="93" t="str">
+        <x:v>4:45 PM</x:v>
+      </x:c>
+      <x:c r="E78" s="93" t="str">
+        <x:v>4:55 PM</x:v>
+      </x:c>
+      <x:c r="F78" s="93" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G78" s="94" t="str"/>
+    </x:row>
+    <x:row r="79" ht="20" customHeight="1">
+      <x:c r="A79" s="84" t="str">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B79" s="87" t="str">
+        <x:v>HYPERFIST</x:v>
+      </x:c>
+      <x:c r="C79" s="85" t="str">
+        <x:v>Chirality · Booth U15</x:v>
+      </x:c>
+      <x:c r="D79" s="85" t="str">
+        <x:v>4:55 PM</x:v>
+      </x:c>
+      <x:c r="E79" s="85" t="str">
+        <x:v>5:01 PM</x:v>
+      </x:c>
+      <x:c r="F79" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G70" s="59" t="str"/>
-    </x:row>
-    <x:row r="71" ht="20" customHeight="1">
-      <x:c r="A71" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B71" s="64" t="str">
+      <x:c r="G79" s="86" t="str"/>
+    </x:row>
+    <x:row r="80" ht="20" customHeight="1">
+      <x:c r="A80" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B80" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C71" s="62" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D71" s="62" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="E71" s="62" t="str">
-        <x:v>4:24 PM</x:v>
-      </x:c>
-      <x:c r="F71" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G71" s="63" t="str"/>
-    </x:row>
-    <x:row r="72" ht="20" customHeight="1">
-      <x:c r="A72" s="57" t="str">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B72" s="60" t="str">
-        <x:v>WILL: Follow The Light</x:v>
-      </x:c>
-      <x:c r="C72" s="58" t="str">
-        <x:v>TomorrowHead Studio · Booth U23</x:v>
-      </x:c>
-      <x:c r="D72" s="58" t="str">
-        <x:v>4:24 PM</x:v>
-      </x:c>
-      <x:c r="E72" s="58" t="str">
-        <x:v>4:30 PM</x:v>
-      </x:c>
-      <x:c r="F72" s="58" t="str">
+      <x:c r="C80" s="89" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D80" s="89" t="str">
+        <x:v>5:01 PM</x:v>
+      </x:c>
+      <x:c r="E80" s="89" t="str">
+        <x:v>5:02 PM</x:v>
+      </x:c>
+      <x:c r="F80" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G80" s="90" t="str"/>
+    </x:row>
+    <x:row r="81" ht="20" customHeight="1">
+      <x:c r="A81" s="84" t="str">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B81" s="87" t="str">
+        <x:v>Nightmare Kitchen</x:v>
+      </x:c>
+      <x:c r="C81" s="85" t="str">
+        <x:v>Byteback Studios · Booth U16</x:v>
+      </x:c>
+      <x:c r="D81" s="85" t="str">
+        <x:v>5:02 PM</x:v>
+      </x:c>
+      <x:c r="E81" s="85" t="str">
+        <x:v>5:08 PM</x:v>
+      </x:c>
+      <x:c r="F81" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G72" s="59" t="str"/>
-    </x:row>
-    <x:row r="73" ht="20" customHeight="1">
-      <x:c r="A73" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B73" s="64" t="str">
+      <x:c r="G81" s="86" t="str"/>
+    </x:row>
+    <x:row r="82" ht="20" customHeight="1">
+      <x:c r="A82" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B82" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C73" s="62" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D73" s="62" t="str">
-        <x:v>4:30 PM</x:v>
-      </x:c>
-      <x:c r="E73" s="62" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="F73" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G73" s="63" t="str"/>
-    </x:row>
-    <x:row r="74" ht="20" customHeight="1">
-      <x:c r="A74" s="57" t="str">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B74" s="60" t="str">
-        <x:v>Turning Manor</x:v>
-      </x:c>
-      <x:c r="C74" s="58" t="str">
-        <x:v>Sabbatical Games · Booth U24</x:v>
-      </x:c>
-      <x:c r="D74" s="58" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="E74" s="58" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="F74" s="58" t="str">
+      <x:c r="C82" s="89" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D82" s="89" t="str">
+        <x:v>5:08 PM</x:v>
+      </x:c>
+      <x:c r="E82" s="89" t="str">
+        <x:v>5:09 PM</x:v>
+      </x:c>
+      <x:c r="F82" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G82" s="90" t="str"/>
+    </x:row>
+    <x:row r="83" ht="20" customHeight="1">
+      <x:c r="A83" s="84" t="str">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B83" s="87" t="str">
+        <x:v>Shroomwood</x:v>
+      </x:c>
+      <x:c r="C83" s="85" t="str">
+        <x:v>Sporelite Games · Booth U17</x:v>
+      </x:c>
+      <x:c r="D83" s="85" t="str">
+        <x:v>5:09 PM</x:v>
+      </x:c>
+      <x:c r="E83" s="85" t="str">
+        <x:v>5:15 PM</x:v>
+      </x:c>
+      <x:c r="F83" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G74" s="59" t="str"/>
-    </x:row>
-    <x:row r="75" ht="20" customHeight="1">
-      <x:c r="A75" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B75" s="64" t="str">
+      <x:c r="G83" s="86" t="str"/>
+    </x:row>
+    <x:row r="84" ht="20" customHeight="1">
+      <x:c r="A84" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B84" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C75" s="62" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D75" s="62" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="E75" s="62" t="str">
-        <x:v>4:38 PM</x:v>
-      </x:c>
-      <x:c r="F75" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G75" s="63" t="str"/>
-    </x:row>
-    <x:row r="76" ht="20" customHeight="1">
-      <x:c r="A76" s="57" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B76" s="60" t="str">
-        <x:v>Steel Swarm: SURVIVOR</x:v>
-      </x:c>
-      <x:c r="C76" s="58" t="str">
-        <x:v>Clay Token Game Studio, Inc. · Booth U25</x:v>
-      </x:c>
-      <x:c r="D76" s="58" t="str">
-        <x:v>4:38 PM</x:v>
-      </x:c>
-      <x:c r="E76" s="58" t="str">
-        <x:v>4:44 PM</x:v>
-      </x:c>
-      <x:c r="F76" s="58" t="str">
+      <x:c r="C84" s="89" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D84" s="89" t="str">
+        <x:v>5:15 PM</x:v>
+      </x:c>
+      <x:c r="E84" s="89" t="str">
+        <x:v>5:16 PM</x:v>
+      </x:c>
+      <x:c r="F84" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G84" s="90" t="str"/>
+    </x:row>
+    <x:row r="85" ht="20" customHeight="1">
+      <x:c r="A85" s="84" t="str">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B85" s="87" t="str">
+        <x:v>Knockout 2: Wrath of the Karen</x:v>
+      </x:c>
+      <x:c r="C85" s="85" t="str">
+        <x:v>ExceptioNULL Games · Booth U18</x:v>
+      </x:c>
+      <x:c r="D85" s="85" t="str">
+        <x:v>5:16 PM</x:v>
+      </x:c>
+      <x:c r="E85" s="85" t="str">
+        <x:v>5:22 PM</x:v>
+      </x:c>
+      <x:c r="F85" s="85" t="str">
         <x:v>E</x:v>
       </x:c>
-      <x:c r="G76" s="59" t="str"/>
-    </x:row>
-    <x:row r="77" ht="20" customHeight="1">
-      <x:c r="A77" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B77" s="64" t="str">
+      <x:c r="G85" s="86" t="str"/>
+    </x:row>
+    <x:row r="86" ht="20" customHeight="1">
+      <x:c r="A86" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B86" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C77" s="62" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D77" s="62" t="str">
-        <x:v>4:44 PM</x:v>
-      </x:c>
-      <x:c r="E77" s="62" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="F77" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G77" s="63" t="str"/>
-    </x:row>
-    <x:row r="78" ht="20" customHeight="1">
-      <x:c r="A78" s="65" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B78" s="68" t="str">
-        <x:v>NDVisibility Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C78" s="66" t="str">
-        <x:v>Sponsor segment · 000</x:v>
-      </x:c>
-      <x:c r="D78" s="66" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="E78" s="66" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="F78" s="66" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G78" s="67" t="str"/>
-    </x:row>
-    <x:row r="79" ht="20" customHeight="1">
-      <x:c r="A79" s="57" t="str">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B79" s="60" t="str">
-        <x:v>HYPERFIST</x:v>
-      </x:c>
-      <x:c r="C79" s="58" t="str">
-        <x:v>Chirality · Booth U15</x:v>
-      </x:c>
-      <x:c r="D79" s="58" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="E79" s="58" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="F79" s="58" t="str">
+      <x:c r="C86" s="89" t="str">
+        <x:v>Block H</x:v>
+      </x:c>
+      <x:c r="D86" s="89" t="str">
+        <x:v>5:22 PM</x:v>
+      </x:c>
+      <x:c r="E86" s="89" t="str">
+        <x:v>5:23 PM</x:v>
+      </x:c>
+      <x:c r="F86" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G86" s="90" t="str"/>
+    </x:row>
+    <x:row r="87" ht="20" customHeight="1">
+      <x:c r="A87" s="84" t="str">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B87" s="87" t="str">
+        <x:v>Cooking Fist</x:v>
+      </x:c>
+      <x:c r="C87" s="85" t="str">
+        <x:v>Spaghetti Code LLC · Booth U19</x:v>
+      </x:c>
+      <x:c r="D87" s="85" t="str">
+        <x:v>5:23 PM</x:v>
+      </x:c>
+      <x:c r="E87" s="85" t="str">
+        <x:v>5:29 PM</x:v>
+      </x:c>
+      <x:c r="F87" s="85" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G79" s="59" t="str"/>
-    </x:row>
-    <x:row r="80" ht="20" customHeight="1">
-      <x:c r="A80" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B80" s="64" t="str">
+      <x:c r="G87" s="86" t="str"/>
+    </x:row>
+    <x:row r="88" ht="20" customHeight="1">
+      <x:c r="A88" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B88" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C80" s="62" t="str">
+      <x:c r="C88" s="89" t="str">
         <x:v>Block H</x:v>
       </x:c>
-      <x:c r="D80" s="62" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="E80" s="62" t="str">
-        <x:v>5:02 PM</x:v>
-      </x:c>
-      <x:c r="F80" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G80" s="63" t="str"/>
-    </x:row>
-    <x:row r="81" ht="20" customHeight="1">
-      <x:c r="A81" s="57" t="str">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B81" s="60" t="str">
-        <x:v>Nightmare Kitchen</x:v>
-      </x:c>
-      <x:c r="C81" s="58" t="str">
-        <x:v>Byteback Studios · Booth U16</x:v>
-      </x:c>
-      <x:c r="D81" s="58" t="str">
-        <x:v>5:02 PM</x:v>
-      </x:c>
-      <x:c r="E81" s="58" t="str">
-        <x:v>5:08 PM</x:v>
-      </x:c>
-      <x:c r="F81" s="58" t="str">
+      <x:c r="D88" s="89" t="str">
+        <x:v>5:29 PM</x:v>
+      </x:c>
+      <x:c r="E88" s="89" t="str">
+        <x:v>5:30 PM</x:v>
+      </x:c>
+      <x:c r="F88" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G88" s="90" t="str"/>
+    </x:row>
+    <x:row r="89" ht="20" customHeight="1">
+      <x:c r="A89" s="96" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B89" s="99" t="str">
+        <x:v>Ukrainian Games Videos</x:v>
+      </x:c>
+      <x:c r="C89" s="97" t="str">
+        <x:v>International showcase · 000</x:v>
+      </x:c>
+      <x:c r="D89" s="97" t="str">
+        <x:v>5:30 PM</x:v>
+      </x:c>
+      <x:c r="E89" s="97" t="str">
+        <x:v>5:35 PM</x:v>
+      </x:c>
+      <x:c r="F89" s="97" t="str">
+        <x:v>Prerecorded</x:v>
+      </x:c>
+      <x:c r="G89" s="98" t="str"/>
+    </x:row>
+    <x:row r="90" ht="20" customHeight="1">
+      <x:c r="A90" s="84" t="str">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B90" s="87" t="str">
+        <x:v>Killing Baby Hitler</x:v>
+      </x:c>
+      <x:c r="C90" s="85" t="str">
+        <x:v>The Coffee Industrial Complex · Booth U14</x:v>
+      </x:c>
+      <x:c r="D90" s="85" t="str">
+        <x:v>5:35 PM</x:v>
+      </x:c>
+      <x:c r="E90" s="85" t="str">
+        <x:v>5:41 PM</x:v>
+      </x:c>
+      <x:c r="F90" s="85" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="G81" s="59" t="str"/>
-    </x:row>
-    <x:row r="82" ht="20" customHeight="1">
-      <x:c r="A82" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B82" s="64" t="str">
+      <x:c r="G90" s="86" t="str"/>
+    </x:row>
+    <x:row r="91" ht="20" customHeight="1">
+      <x:c r="A91" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B91" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C82" s="62" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D82" s="62" t="str">
-        <x:v>5:08 PM</x:v>
-      </x:c>
-      <x:c r="E82" s="62" t="str">
-        <x:v>5:09 PM</x:v>
-      </x:c>
-      <x:c r="F82" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G82" s="63" t="str"/>
-    </x:row>
-    <x:row r="83" ht="20" customHeight="1">
-      <x:c r="A83" s="57" t="str">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B83" s="60" t="str">
-        <x:v>Shroomwood</x:v>
-      </x:c>
-      <x:c r="C83" s="58" t="str">
-        <x:v>Sporelite Games · Booth U17</x:v>
-      </x:c>
-      <x:c r="D83" s="58" t="str">
-        <x:v>5:09 PM</x:v>
-      </x:c>
-      <x:c r="E83" s="58" t="str">
-        <x:v>5:15 PM</x:v>
-      </x:c>
-      <x:c r="F83" s="58" t="str">
+      <x:c r="C91" s="89" t="str">
+        <x:v>Block I</x:v>
+      </x:c>
+      <x:c r="D91" s="89" t="str">
+        <x:v>5:41 PM</x:v>
+      </x:c>
+      <x:c r="E91" s="89" t="str">
+        <x:v>5:42 PM</x:v>
+      </x:c>
+      <x:c r="F91" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G91" s="90" t="str"/>
+    </x:row>
+    <x:row r="92" ht="20" customHeight="1">
+      <x:c r="A92" s="84" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B92" s="87" t="str">
+        <x:v>The Assessment</x:v>
+      </x:c>
+      <x:c r="C92" s="85" t="str">
+        <x:v>Miga Games · Booth U11</x:v>
+      </x:c>
+      <x:c r="D92" s="85" t="str">
+        <x:v>5:42 PM</x:v>
+      </x:c>
+      <x:c r="E92" s="85" t="str">
+        <x:v>5:48 PM</x:v>
+      </x:c>
+      <x:c r="F92" s="85" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="G83" s="59" t="str"/>
-    </x:row>
-    <x:row r="84" ht="20" customHeight="1">
-      <x:c r="A84" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B84" s="64" t="str">
+      <x:c r="G92" s="86" t="str"/>
+    </x:row>
+    <x:row r="93" ht="20" customHeight="1">
+      <x:c r="A93" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B93" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C84" s="62" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D84" s="62" t="str">
-        <x:v>5:15 PM</x:v>
-      </x:c>
-      <x:c r="E84" s="62" t="str">
-        <x:v>5:16 PM</x:v>
-      </x:c>
-      <x:c r="F84" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G84" s="63" t="str"/>
-    </x:row>
-    <x:row r="85" ht="20" customHeight="1">
-      <x:c r="A85" s="57" t="str">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B85" s="60" t="str">
-        <x:v>Knockout 2: Wrath of the Karen</x:v>
-      </x:c>
-      <x:c r="C85" s="58" t="str">
-        <x:v>ExceptioNULL Games · Booth U18</x:v>
-      </x:c>
-      <x:c r="D85" s="58" t="str">
-        <x:v>5:16 PM</x:v>
-      </x:c>
-      <x:c r="E85" s="58" t="str">
-        <x:v>5:22 PM</x:v>
-      </x:c>
-      <x:c r="F85" s="58" t="str">
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="G85" s="59" t="str"/>
-    </x:row>
-    <x:row r="86" ht="20" customHeight="1">
-      <x:c r="A86" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B86" s="64" t="str">
+      <x:c r="C93" s="89" t="str">
+        <x:v>Block I</x:v>
+      </x:c>
+      <x:c r="D93" s="89" t="str">
+        <x:v>5:48 PM</x:v>
+      </x:c>
+      <x:c r="E93" s="89" t="str">
+        <x:v>5:49 PM</x:v>
+      </x:c>
+      <x:c r="F93" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G93" s="90" t="str"/>
+    </x:row>
+    <x:row r="94" ht="20" customHeight="1">
+      <x:c r="A94" s="96" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B94" s="99" t="str">
+        <x:v>Chile Games Showcase Video</x:v>
+      </x:c>
+      <x:c r="C94" s="97" t="str">
+        <x:v>International showcase · 000</x:v>
+      </x:c>
+      <x:c r="D94" s="97" t="str">
+        <x:v>5:49 PM</x:v>
+      </x:c>
+      <x:c r="E94" s="97" t="str">
+        <x:v>5:54 PM</x:v>
+      </x:c>
+      <x:c r="F94" s="97" t="str">
+        <x:v>Prerecorded</x:v>
+      </x:c>
+      <x:c r="G94" s="98" t="str"/>
+    </x:row>
+    <x:row r="95" ht="20" customHeight="1">
+      <x:c r="A95" s="88" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="B95" s="91" t="str">
         <x:v>Break / Transition</x:v>
       </x:c>
-      <x:c r="C86" s="62" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D86" s="62" t="str">
-        <x:v>5:22 PM</x:v>
-      </x:c>
-      <x:c r="E86" s="62" t="str">
-        <x:v>5:23 PM</x:v>
-      </x:c>
-      <x:c r="F86" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G86" s="63" t="str"/>
-    </x:row>
-    <x:row r="87" ht="20" customHeight="1">
-      <x:c r="A87" s="57" t="str">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B87" s="60" t="str">
-        <x:v>Cooking Fist</x:v>
-      </x:c>
-      <x:c r="C87" s="58" t="str">
-        <x:v>Spaghetti Code LLC · Booth U19</x:v>
-      </x:c>
-      <x:c r="D87" s="58" t="str">
-        <x:v>5:23 PM</x:v>
-      </x:c>
-      <x:c r="E87" s="58" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="F87" s="58" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G87" s="59" t="str"/>
-    </x:row>
-    <x:row r="88" ht="20" customHeight="1">
-      <x:c r="A88" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B88" s="64" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C88" s="62" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D88" s="62" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="E88" s="62" t="str">
-        <x:v>5:30 PM</x:v>
-      </x:c>
-      <x:c r="F88" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G88" s="63" t="str"/>
-    </x:row>
-    <x:row r="89" ht="20" customHeight="1">
-      <x:c r="A89" s="69" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B89" s="72" t="str">
-        <x:v>Ukrainian Games Videos</x:v>
-      </x:c>
-      <x:c r="C89" s="70" t="str">
-        <x:v>International showcase · 000</x:v>
-      </x:c>
-      <x:c r="D89" s="70" t="str">
-        <x:v>5:30 PM</x:v>
-      </x:c>
-      <x:c r="E89" s="70" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="F89" s="70" t="str">
-        <x:v>Prerecorded</x:v>
-      </x:c>
-      <x:c r="G89" s="71" t="str"/>
-    </x:row>
-    <x:row r="90" ht="20" customHeight="1">
-      <x:c r="A90" s="57" t="str">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B90" s="60" t="str">
-        <x:v>Killing Baby Hitler</x:v>
-      </x:c>
-      <x:c r="C90" s="58" t="str">
-        <x:v>The Coffee Industrial Complex · Booth U14</x:v>
-      </x:c>
-      <x:c r="D90" s="58" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="E90" s="58" t="str">
-        <x:v>5:41 PM</x:v>
-      </x:c>
-      <x:c r="F90" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G90" s="59" t="str"/>
-    </x:row>
-    <x:row r="91" ht="20" customHeight="1">
-      <x:c r="A91" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B91" s="64" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C91" s="62" t="str">
+      <x:c r="C95" s="89" t="str">
         <x:v>Block I</x:v>
       </x:c>
-      <x:c r="D91" s="62" t="str">
-        <x:v>5:41 PM</x:v>
-      </x:c>
-      <x:c r="E91" s="62" t="str">
-        <x:v>5:42 PM</x:v>
-      </x:c>
-      <x:c r="F91" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G91" s="63" t="str"/>
-    </x:row>
-    <x:row r="92" ht="20" customHeight="1">
-      <x:c r="A92" s="57" t="str">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B92" s="60" t="str">
-        <x:v>The Assessment</x:v>
-      </x:c>
-      <x:c r="C92" s="58" t="str">
-        <x:v>Miga Games · Booth U11</x:v>
-      </x:c>
-      <x:c r="D92" s="58" t="str">
-        <x:v>5:42 PM</x:v>
-      </x:c>
-      <x:c r="E92" s="58" t="str">
-        <x:v>5:48 PM</x:v>
-      </x:c>
-      <x:c r="F92" s="58" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G92" s="59" t="str"/>
-    </x:row>
-    <x:row r="93" ht="20" customHeight="1">
-      <x:c r="A93" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B93" s="64" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C93" s="62" t="str">
-        <x:v>Block I</x:v>
-      </x:c>
-      <x:c r="D93" s="62" t="str">
-        <x:v>5:48 PM</x:v>
-      </x:c>
-      <x:c r="E93" s="62" t="str">
-        <x:v>5:49 PM</x:v>
-      </x:c>
-      <x:c r="F93" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G93" s="63" t="str"/>
-    </x:row>
-    <x:row r="94" ht="20" customHeight="1">
-      <x:c r="A94" s="69" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B94" s="72" t="str">
-        <x:v>Chile Games Showcase Video</x:v>
-      </x:c>
-      <x:c r="C94" s="70" t="str">
-        <x:v>International showcase · 000</x:v>
-      </x:c>
-      <x:c r="D94" s="70" t="str">
-        <x:v>5:49 PM</x:v>
-      </x:c>
-      <x:c r="E94" s="70" t="str">
+      <x:c r="D95" s="89" t="str">
         <x:v>5:54 PM</x:v>
       </x:c>
-      <x:c r="F94" s="70" t="str">
-        <x:v>Prerecorded</x:v>
-      </x:c>
-      <x:c r="G94" s="71" t="str"/>
-    </x:row>
-    <x:row r="95" ht="20" customHeight="1">
-      <x:c r="A95" s="61" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B95" s="64" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C95" s="62" t="str">
-        <x:v>Block I</x:v>
-      </x:c>
-      <x:c r="D95" s="62" t="str">
-        <x:v>5:54 PM</x:v>
-      </x:c>
-      <x:c r="E95" s="62" t="str">
+      <x:c r="E95" s="89" t="str">
         <x:v>5:55 PM</x:v>
       </x:c>
-      <x:c r="F95" s="62" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G95" s="63" t="str"/>
+      <x:c r="F95" s="89" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G95" s="90" t="str"/>
     </x:row>
     <x:row r="96" ht="20" customHeight="1">
-      <x:c r="A96" s="73" t="str">
+      <x:c r="A96" s="100" t="str">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B96" s="76" t="str">
+      <x:c r="B96" s="103" t="str">
         <x:v>Closing / Thank You</x:v>
       </x:c>
-      <x:c r="C96" s="74" t="str">
+      <x:c r="C96" s="101" t="str">
         <x:v>Seattle Indies</x:v>
       </x:c>
-      <x:c r="D96" s="74" t="str">
+      <x:c r="D96" s="101" t="str">
         <x:v>5:55 PM</x:v>
       </x:c>
-      <x:c r="E96" s="74" t="str">
+      <x:c r="E96" s="101" t="str">
         <x:v>6:05 PM</x:v>
       </x:c>
-      <x:c r="F96" s="74" t="str">
+      <x:c r="F96" s="101" t="str">
         <x:v>All Hosts</x:v>
       </x:c>
-      <x:c r="G96" s="75" t="str"/>
+      <x:c r="G96" s="102" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2868,72 +3026,72 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
-      <x:c r="A3" s="41" t="inlineStr">
+      <x:c r="A3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Name</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="41" t="inlineStr">
+      <x:c r="B3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer / Publisher</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="41" t="inlineStr">
+      <x:c r="C3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Platforms</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="41" t="inlineStr">
+      <x:c r="D3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Display Platforms</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" s="41" t="inlineStr">
+      <x:c r="E3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Availability</x:t>
         </x:is>
       </x:c>
-      <x:c r="F3" s="41" t="inlineStr">
+      <x:c r="F3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Release</x:t>
         </x:is>
       </x:c>
-      <x:c r="G3" s="41" t="inlineStr">
+      <x:c r="G3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Demo / Build</x:t>
         </x:is>
       </x:c>
-      <x:c r="H3" s="41" t="inlineStr">
+      <x:c r="H3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Quick Overview</x:t>
         </x:is>
       </x:c>
-      <x:c r="I3" s="41" t="inlineStr">
+      <x:c r="I3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Full Description</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" s="41" t="inlineStr">
+      <x:c r="J3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Official URL</x:t>
         </x:is>
       </x:c>
-      <x:c r="K3" s="41" t="inlineStr">
+      <x:c r="K3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Steam App ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="L3" s="41" t="inlineStr">
+      <x:c r="L3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">YouTube Video ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="M3" s="41" t="inlineStr">
+      <x:c r="M3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Media Slug</x:t>
         </x:is>
       </x:c>
-      <x:c r="N3" s="41" t="inlineStr">
+      <x:c r="N3" s="79" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Media Folder</x:t>
         </x:is>

</xml_diff>

<commit_message>
Remove The Assessment from run of show
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -981,2014 +981,1993 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="7" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="77" t="str">
-        <x:v>Seattle Indies Expo - SIX 2026 | Run of Show</x:v>
-      </x:c>
-      <x:c r="B1" s="77"/>
-      <x:c r="C1" s="77"/>
-      <x:c r="D1" s="77"/>
-      <x:c r="E1" s="77"/>
-      <x:c r="F1" s="77"/>
-      <x:c r="G1" s="77"/>
-    </x:row>
-    <x:row r="2" ht="21" customHeight="1">
-      <x:c r="A2" s="78" t="str">
-        <x:v>Run of Show - Production Schedule</x:v>
-      </x:c>
-      <x:c r="B2" s="78"/>
-      <x:c r="C2" s="78"/>
-      <x:c r="D2" s="78"/>
-      <x:c r="E2" s="78"/>
-      <x:c r="F2" s="78"/>
-      <x:c r="G2" s="78"/>
-    </x:row>
-    <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="38" t="str">
-        <x:v>Host A = Unavailable | Host B = AbdallahSmash | Host C = MacnCheesep1z | Host D = Rockagoth | Host E = AlchemistJoker</x:v>
-      </x:c>
-      <x:c r="B3" s="39"/>
-      <x:c r="C3" s="39"/>
-      <x:c r="D3" s="39"/>
-      <x:c r="E3" s="39"/>
-      <x:c r="F3" s="39"/>
-      <x:c r="G3" s="39"/>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="79" t="str">
-        <x:v>SEG</x:v>
-      </x:c>
-      <x:c r="B4" s="79" t="str">
-        <x:v>GAME / BREAK</x:v>
-      </x:c>
-      <x:c r="C4" s="79" t="str">
-        <x:v>DEVELOPER / PUBLISHER</x:v>
-      </x:c>
-      <x:c r="D4" s="79" t="str">
-        <x:v>START</x:v>
-      </x:c>
-      <x:c r="E4" s="79" t="str">
-        <x:v>END</x:v>
-      </x:c>
-      <x:c r="F4" s="79" t="str">
-        <x:v>HOST</x:v>
-      </x:c>
-      <x:c r="G4" s="79" t="str">
-        <x:v>PRODUCTION NOTES</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="80" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B5" s="83" t="str">
-        <x:v>SIX Hype Hour</x:v>
-      </x:c>
-      <x:c r="C5" s="81" t="str">
-        <x:v>Seattle Indies</x:v>
-      </x:c>
-      <x:c r="D5" s="81" t="str">
-        <x:v>10:00 AM</x:v>
-      </x:c>
-      <x:c r="E5" s="81" t="str">
-        <x:v>12:00 PM</x:v>
-      </x:c>
-      <x:c r="F5" s="81" t="str">
-        <x:v>Prerecorded</x:v>
-      </x:c>
-      <x:c r="G5" s="82" t="str"/>
-    </x:row>
-    <x:row r="6" ht="20" customHeight="1">
-      <x:c r="A6" s="84" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B6" s="87" t="str">
-        <x:v>Tricky and the Dream Caster</x:v>
-      </x:c>
-      <x:c r="C6" s="85" t="str">
-        <x:v>PossQueen · Booth L27</x:v>
-      </x:c>
-      <x:c r="D6" s="85" t="str">
-        <x:v>12:00 PM</x:v>
-      </x:c>
-      <x:c r="E6" s="85" t="str">
-        <x:v>12:06 PM</x:v>
-      </x:c>
-      <x:c r="F6" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G6" s="86" t="str"/>
-    </x:row>
-    <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B7" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C7" s="89" t="str">
-        <x:v>Block A</x:v>
-      </x:c>
-      <x:c r="D7" s="89" t="str">
-        <x:v>12:06 PM</x:v>
-      </x:c>
-      <x:c r="E7" s="89" t="str">
-        <x:v>12:07 PM</x:v>
-      </x:c>
-      <x:c r="F7" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G7" s="90" t="str"/>
-    </x:row>
-    <x:row r="8" ht="20" customHeight="1">
-      <x:c r="A8" s="84" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B8" s="87" t="str">
-        <x:v>TileShire</x:v>
-      </x:c>
-      <x:c r="C8" s="85" t="str">
-        <x:v>Boss Blob · Booth L28</x:v>
-      </x:c>
-      <x:c r="D8" s="85" t="str">
-        <x:v>12:07 PM</x:v>
-      </x:c>
-      <x:c r="E8" s="85" t="str">
-        <x:v>12:13 PM</x:v>
-      </x:c>
-      <x:c r="F8" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G8" s="86" t="str"/>
-    </x:row>
-    <x:row r="9" ht="20" customHeight="1">
-      <x:c r="A9" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B9" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C9" s="89" t="str">
-        <x:v>Block A</x:v>
-      </x:c>
-      <x:c r="D9" s="89" t="str">
-        <x:v>12:13 PM</x:v>
-      </x:c>
-      <x:c r="E9" s="89" t="str">
-        <x:v>12:14 PM</x:v>
-      </x:c>
-      <x:c r="F9" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G9" s="90" t="str"/>
-    </x:row>
-    <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="84" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B10" s="87" t="str">
-        <x:v>Wrestle Story</x:v>
-      </x:c>
-      <x:c r="C10" s="85" t="str">
-        <x:v>Tic Toc Games · Booth L29</x:v>
-      </x:c>
-      <x:c r="D10" s="85" t="str">
-        <x:v>12:14 PM</x:v>
-      </x:c>
-      <x:c r="E10" s="85" t="str">
-        <x:v>12:20 PM</x:v>
-      </x:c>
-      <x:c r="F10" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="86" t="str"/>
-    </x:row>
-    <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B11" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C11" s="89" t="str">
-        <x:v>Block A</x:v>
-      </x:c>
-      <x:c r="D11" s="89" t="str">
-        <x:v>12:20 PM</x:v>
-      </x:c>
-      <x:c r="E11" s="89" t="str">
-        <x:v>12:21 PM</x:v>
-      </x:c>
-      <x:c r="F11" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G11" s="90" t="str"/>
-    </x:row>
-    <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="84" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B12" s="87" t="str">
-        <x:v>Breach Of Contract</x:v>
-      </x:c>
-      <x:c r="C12" s="85" t="str">
-        <x:v>Fern Sprout Studios · Booth L30</x:v>
-      </x:c>
-      <x:c r="D12" s="85" t="str">
-        <x:v>12:21 PM</x:v>
-      </x:c>
-      <x:c r="E12" s="85" t="str">
-        <x:v>12:27 PM</x:v>
-      </x:c>
-      <x:c r="F12" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G12" s="86" t="str"/>
-    </x:row>
-    <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B13" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C13" s="89" t="str">
-        <x:v>Block A</x:v>
-      </x:c>
-      <x:c r="D13" s="89" t="str">
-        <x:v>12:27 PM</x:v>
-      </x:c>
-      <x:c r="E13" s="89" t="str">
-        <x:v>12:28 PM</x:v>
-      </x:c>
-      <x:c r="F13" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G13" s="90" t="str"/>
-    </x:row>
-    <x:row r="14" ht="20" customHeight="1">
-      <x:c r="A14" s="84" t="str">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B14" s="87" t="str">
-        <x:v>Dungeon Bodega Simulator</x:v>
-      </x:c>
-      <x:c r="C14" s="85" t="str">
-        <x:v>Alien Fruit Games · Booth L31</x:v>
-      </x:c>
-      <x:c r="D14" s="85" t="str">
-        <x:v>12:28 PM</x:v>
-      </x:c>
-      <x:c r="E14" s="85" t="str">
-        <x:v>12:34 PM</x:v>
-      </x:c>
-      <x:c r="F14" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G14" s="86" t="str"/>
-    </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B15" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C15" s="89" t="str">
-        <x:v>Block A</x:v>
-      </x:c>
-      <x:c r="D15" s="89" t="str">
-        <x:v>12:34 PM</x:v>
-      </x:c>
-      <x:c r="E15" s="89" t="str">
-        <x:v>12:35 PM</x:v>
-      </x:c>
-      <x:c r="F15" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G15" s="90" t="str"/>
-    </x:row>
-    <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B16" s="95" t="str">
-        <x:v>DigiPen Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C16" s="93" t="str">
-        <x:v>Sponsor segment · L01</x:v>
-      </x:c>
-      <x:c r="D16" s="93" t="str">
-        <x:v>12:35 PM</x:v>
-      </x:c>
-      <x:c r="E16" s="93" t="str">
-        <x:v>12:45 PM</x:v>
-      </x:c>
-      <x:c r="F16" s="93" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G16" s="94" t="str"/>
-    </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="84" t="str">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B17" s="87" t="str">
-        <x:v>SCP: Antimemetics Division</x:v>
-      </x:c>
-      <x:c r="C17" s="85" t="str">
-        <x:v>Quadrant Five · Booth L22</x:v>
-      </x:c>
-      <x:c r="D17" s="85" t="str">
-        <x:v>12:45 PM</x:v>
-      </x:c>
-      <x:c r="E17" s="85" t="str">
-        <x:v>12:51 PM</x:v>
-      </x:c>
-      <x:c r="F17" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G17" s="86" t="str"/>
-    </x:row>
-    <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B18" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C18" s="89" t="str">
-        <x:v>Block B</x:v>
-      </x:c>
-      <x:c r="D18" s="89" t="str">
-        <x:v>12:51 PM</x:v>
-      </x:c>
-      <x:c r="E18" s="89" t="str">
-        <x:v>12:52 PM</x:v>
-      </x:c>
-      <x:c r="F18" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G18" s="90" t="str"/>
-    </x:row>
-    <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="84" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B19" s="87" t="str">
-        <x:v>Manafinder II</x:v>
-      </x:c>
-      <x:c r="C19" s="85" t="str">
-        <x:v>Wolfsden LLC · Booth L23</x:v>
-      </x:c>
-      <x:c r="D19" s="85" t="str">
-        <x:v>12:52 PM</x:v>
-      </x:c>
-      <x:c r="E19" s="85" t="str">
-        <x:v>12:58 PM</x:v>
-      </x:c>
-      <x:c r="F19" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G19" s="86" t="str"/>
-    </x:row>
-    <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B20" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C20" s="89" t="str">
-        <x:v>Block B</x:v>
-      </x:c>
-      <x:c r="D20" s="89" t="str">
-        <x:v>12:58 PM</x:v>
-      </x:c>
-      <x:c r="E20" s="89" t="str">
-        <x:v>12:59 PM</x:v>
-      </x:c>
-      <x:c r="F20" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G20" s="90" t="str"/>
-    </x:row>
-    <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="84" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B21" s="87" t="str">
-        <x:v>Malice In Wonderland</x:v>
-      </x:c>
-      <x:c r="C21" s="85" t="str">
-        <x:v>Slyglass Games · Booth L24</x:v>
-      </x:c>
-      <x:c r="D21" s="85" t="str">
-        <x:v>12:59 PM</x:v>
-      </x:c>
-      <x:c r="E21" s="85" t="str">
-        <x:v>1:05 PM</x:v>
-      </x:c>
-      <x:c r="F21" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G21" s="86" t="str"/>
-    </x:row>
-    <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B22" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C22" s="89" t="str">
-        <x:v>Block B</x:v>
-      </x:c>
-      <x:c r="D22" s="89" t="str">
-        <x:v>1:05 PM</x:v>
-      </x:c>
-      <x:c r="E22" s="89" t="str">
-        <x:v>1:06 PM</x:v>
-      </x:c>
-      <x:c r="F22" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G22" s="90" t="str"/>
-    </x:row>
-    <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="84" t="str">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B23" s="87" t="str">
-        <x:v>Project Cradle</x:v>
-      </x:c>
-      <x:c r="C23" s="85" t="str">
-        <x:v>ShazySoft · Booth L25</x:v>
-      </x:c>
-      <x:c r="D23" s="85" t="str">
-        <x:v>1:06 PM</x:v>
-      </x:c>
-      <x:c r="E23" s="85" t="str">
-        <x:v>1:12 PM</x:v>
-      </x:c>
-      <x:c r="F23" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G23" s="86" t="str"/>
-    </x:row>
-    <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B24" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C24" s="89" t="str">
-        <x:v>Block B</x:v>
-      </x:c>
-      <x:c r="D24" s="89" t="str">
-        <x:v>1:12 PM</x:v>
-      </x:c>
-      <x:c r="E24" s="89" t="str">
-        <x:v>1:13 PM</x:v>
-      </x:c>
-      <x:c r="F24" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G24" s="90" t="str"/>
-    </x:row>
-    <x:row r="25" ht="20" customHeight="1">
-      <x:c r="A25" s="84" t="str">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B25" s="87" t="str">
-        <x:v>Diabolocracy</x:v>
-      </x:c>
-      <x:c r="C25" s="85" t="str">
-        <x:v>Chaos Gremlin Games · Booth L26</x:v>
-      </x:c>
-      <x:c r="D25" s="85" t="str">
-        <x:v>1:13 PM</x:v>
-      </x:c>
-      <x:c r="E25" s="85" t="str">
-        <x:v>1:19 PM</x:v>
-      </x:c>
-      <x:c r="F25" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G25" s="86" t="str"/>
-    </x:row>
-    <x:row r="26" ht="20" customHeight="1">
-      <x:c r="A26" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B26" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C26" s="89" t="str">
-        <x:v>Block B</x:v>
-      </x:c>
-      <x:c r="D26" s="89" t="str">
-        <x:v>1:19 PM</x:v>
-      </x:c>
-      <x:c r="E26" s="89" t="str">
-        <x:v>1:20 PM</x:v>
-      </x:c>
-      <x:c r="F26" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G26" s="90" t="str"/>
-    </x:row>
-    <x:row r="27" ht="20" customHeight="1">
-      <x:c r="A27" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B27" s="95" t="str">
-        <x:v>AIE Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C27" s="93" t="str">
-        <x:v>Sponsor segment · L02</x:v>
-      </x:c>
-      <x:c r="D27" s="93" t="str">
-        <x:v>1:20 PM</x:v>
-      </x:c>
-      <x:c r="E27" s="93" t="str">
-        <x:v>1:30 PM</x:v>
-      </x:c>
-      <x:c r="F27" s="93" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G27" s="94" t="str"/>
-    </x:row>
-    <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="84" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B28" s="87" t="str">
-        <x:v>Seedborne Soldiers</x:v>
-      </x:c>
-      <x:c r="C28" s="85" t="str">
-        <x:v>Hat Wobble Games · Booth L17</x:v>
-      </x:c>
-      <x:c r="D28" s="85" t="str">
-        <x:v>1:30 PM</x:v>
-      </x:c>
-      <x:c r="E28" s="85" t="str">
-        <x:v>1:36 PM</x:v>
-      </x:c>
-      <x:c r="F28" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G28" s="86" t="str"/>
-    </x:row>
-    <x:row r="29" ht="20" customHeight="1">
-      <x:c r="A29" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B29" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C29" s="89" t="str">
-        <x:v>Block C</x:v>
-      </x:c>
-      <x:c r="D29" s="89" t="str">
-        <x:v>1:36 PM</x:v>
-      </x:c>
-      <x:c r="E29" s="89" t="str">
-        <x:v>1:37 PM</x:v>
-      </x:c>
-      <x:c r="F29" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G29" s="90" t="str"/>
-    </x:row>
-    <x:row r="30" ht="20" customHeight="1">
-      <x:c r="A30" s="84" t="str">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B30" s="87" t="str">
-        <x:v>Super Choppy</x:v>
-      </x:c>
-      <x:c r="C30" s="85" t="str">
-        <x:v>Sumoshell Bombfunk · Booth L18</x:v>
-      </x:c>
-      <x:c r="D30" s="85" t="str">
-        <x:v>1:37 PM</x:v>
-      </x:c>
-      <x:c r="E30" s="85" t="str">
-        <x:v>1:43 PM</x:v>
-      </x:c>
-      <x:c r="F30" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G30" s="86" t="str"/>
-    </x:row>
-    <x:row r="31" ht="20" customHeight="1">
-      <x:c r="A31" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B31" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C31" s="89" t="str">
-        <x:v>Block C</x:v>
-      </x:c>
-      <x:c r="D31" s="89" t="str">
-        <x:v>1:43 PM</x:v>
-      </x:c>
-      <x:c r="E31" s="89" t="str">
-        <x:v>1:44 PM</x:v>
-      </x:c>
-      <x:c r="F31" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G31" s="90" t="str"/>
-    </x:row>
-    <x:row r="32" ht="20" customHeight="1">
-      <x:c r="A32" s="84" t="str">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B32" s="87" t="str">
-        <x:v>Dig Too Deep</x:v>
-      </x:c>
-      <x:c r="C32" s="85" t="str">
-        <x:v>Punch Up Games · Booth L19</x:v>
-      </x:c>
-      <x:c r="D32" s="85" t="str">
-        <x:v>1:44 PM</x:v>
-      </x:c>
-      <x:c r="E32" s="85" t="str">
-        <x:v>1:50 PM</x:v>
-      </x:c>
-      <x:c r="F32" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G32" s="86" t="str"/>
-    </x:row>
-    <x:row r="33" ht="20" customHeight="1">
-      <x:c r="A33" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B33" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C33" s="89" t="str">
-        <x:v>Block C</x:v>
-      </x:c>
-      <x:c r="D33" s="89" t="str">
-        <x:v>1:50 PM</x:v>
-      </x:c>
-      <x:c r="E33" s="89" t="str">
-        <x:v>1:51 PM</x:v>
-      </x:c>
-      <x:c r="F33" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G33" s="90" t="str"/>
-    </x:row>
-    <x:row r="34" ht="20" customHeight="1">
-      <x:c r="A34" s="84" t="str">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B34" s="87" t="str">
-        <x:v>Nimbit Frontier</x:v>
-      </x:c>
-      <x:c r="C34" s="85" t="str">
-        <x:v>Megasploot · Booth L20</x:v>
-      </x:c>
-      <x:c r="D34" s="85" t="str">
-        <x:v>1:51 PM</x:v>
-      </x:c>
-      <x:c r="E34" s="85" t="str">
-        <x:v>1:57 PM</x:v>
-      </x:c>
-      <x:c r="F34" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G34" s="86" t="str"/>
-    </x:row>
-    <x:row r="35" ht="20" customHeight="1">
-      <x:c r="A35" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B35" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C35" s="89" t="str">
-        <x:v>Block C</x:v>
-      </x:c>
-      <x:c r="D35" s="89" t="str">
-        <x:v>1:57 PM</x:v>
-      </x:c>
-      <x:c r="E35" s="89" t="str">
-        <x:v>1:58 PM</x:v>
-      </x:c>
-      <x:c r="F35" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G35" s="90" t="str"/>
-    </x:row>
-    <x:row r="36" ht="20" customHeight="1">
-      <x:c r="A36" s="84" t="str">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B36" s="87" t="str">
-        <x:v>We Need An Army</x:v>
-      </x:c>
-      <x:c r="C36" s="85" t="str">
-        <x:v>Elder Bear Games · Booth L21</x:v>
-      </x:c>
-      <x:c r="D36" s="85" t="str">
-        <x:v>1:58 PM</x:v>
-      </x:c>
-      <x:c r="E36" s="85" t="str">
-        <x:v>2:04 PM</x:v>
-      </x:c>
-      <x:c r="F36" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G36" s="86" t="str"/>
-    </x:row>
-    <x:row r="37" ht="20" customHeight="1">
-      <x:c r="A37" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B37" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C37" s="89" t="str">
-        <x:v>Block C</x:v>
-      </x:c>
-      <x:c r="D37" s="89" t="str">
-        <x:v>2:04 PM</x:v>
-      </x:c>
-      <x:c r="E37" s="89" t="str">
-        <x:v>2:05 PM</x:v>
-      </x:c>
-      <x:c r="F37" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G37" s="90" t="str"/>
-    </x:row>
-    <x:row r="38" ht="20" customHeight="1">
-      <x:c r="A38" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B38" s="95" t="str">
-        <x:v>Unity Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C38" s="93" t="str">
-        <x:v>Sponsor segment · L03</x:v>
-      </x:c>
-      <x:c r="D38" s="93" t="str">
-        <x:v>2:05 PM</x:v>
-      </x:c>
-      <x:c r="E38" s="93" t="str">
-        <x:v>2:15 PM</x:v>
-      </x:c>
-      <x:c r="F38" s="93" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G38" s="94" t="str"/>
-    </x:row>
-    <x:row r="39" ht="20" customHeight="1">
-      <x:c r="A39" s="84" t="str">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B39" s="87" t="str">
-        <x:v>Feeding Gooble</x:v>
-      </x:c>
-      <x:c r="C39" s="85" t="str">
-        <x:v>Displacer Labs · Booth L12</x:v>
-      </x:c>
-      <x:c r="D39" s="85" t="str">
-        <x:v>2:15 PM</x:v>
-      </x:c>
-      <x:c r="E39" s="85" t="str">
-        <x:v>2:21 PM</x:v>
-      </x:c>
-      <x:c r="F39" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G39" s="86" t="str"/>
-    </x:row>
-    <x:row r="40" ht="20" customHeight="1">
-      <x:c r="A40" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B40" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C40" s="89" t="str">
-        <x:v>Block D</x:v>
-      </x:c>
-      <x:c r="D40" s="89" t="str">
-        <x:v>2:21 PM</x:v>
-      </x:c>
-      <x:c r="E40" s="89" t="str">
-        <x:v>2:22 PM</x:v>
-      </x:c>
-      <x:c r="F40" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G40" s="90" t="str"/>
-    </x:row>
-    <x:row r="41" ht="20" customHeight="1">
-      <x:c r="A41" s="84" t="str">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B41" s="87" t="str">
-        <x:v>BroomSweeper</x:v>
-      </x:c>
-      <x:c r="C41" s="85" t="str">
-        <x:v>BandWidth Games · Booth L13</x:v>
-      </x:c>
-      <x:c r="D41" s="85" t="str">
-        <x:v>2:22 PM</x:v>
-      </x:c>
-      <x:c r="E41" s="85" t="str">
-        <x:v>2:28 PM</x:v>
-      </x:c>
-      <x:c r="F41" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G41" s="86" t="str"/>
-    </x:row>
-    <x:row r="42" ht="20" customHeight="1">
-      <x:c r="A42" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B42" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C42" s="89" t="str">
-        <x:v>Block D</x:v>
-      </x:c>
-      <x:c r="D42" s="89" t="str">
-        <x:v>2:28 PM</x:v>
-      </x:c>
-      <x:c r="E42" s="89" t="str">
-        <x:v>2:29 PM</x:v>
-      </x:c>
-      <x:c r="F42" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G42" s="90" t="str"/>
-    </x:row>
-    <x:row r="43" ht="20" customHeight="1">
-      <x:c r="A43" s="84" t="str">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B43" s="87" t="str">
-        <x:v>Fairy Circle</x:v>
-      </x:c>
-      <x:c r="C43" s="85" t="str">
-        <x:v>Play Hooky · Booth L14</x:v>
-      </x:c>
-      <x:c r="D43" s="85" t="str">
-        <x:v>2:29 PM</x:v>
-      </x:c>
-      <x:c r="E43" s="85" t="str">
-        <x:v>2:35 PM</x:v>
-      </x:c>
-      <x:c r="F43" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G43" s="86" t="str"/>
-    </x:row>
-    <x:row r="44" ht="20" customHeight="1">
-      <x:c r="A44" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B44" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C44" s="89" t="str">
-        <x:v>Block D</x:v>
-      </x:c>
-      <x:c r="D44" s="89" t="str">
-        <x:v>2:35 PM</x:v>
-      </x:c>
-      <x:c r="E44" s="89" t="str">
-        <x:v>2:36 PM</x:v>
-      </x:c>
-      <x:c r="F44" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G44" s="90" t="str"/>
-    </x:row>
-    <x:row r="45" ht="20" customHeight="1">
-      <x:c r="A45" s="84" t="str">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B45" s="87" t="str">
-        <x:v>MYRIORAMA</x:v>
-      </x:c>
-      <x:c r="C45" s="85" t="str">
-        <x:v>J&amp;K Games · Booth L15</x:v>
-      </x:c>
-      <x:c r="D45" s="85" t="str">
-        <x:v>2:36 PM</x:v>
-      </x:c>
-      <x:c r="E45" s="85" t="str">
-        <x:v>2:42 PM</x:v>
-      </x:c>
-      <x:c r="F45" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G45" s="86" t="str"/>
-    </x:row>
-    <x:row r="46" ht="20" customHeight="1">
-      <x:c r="A46" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B46" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C46" s="89" t="str">
-        <x:v>Block D</x:v>
-      </x:c>
-      <x:c r="D46" s="89" t="str">
-        <x:v>2:42 PM</x:v>
-      </x:c>
-      <x:c r="E46" s="89" t="str">
-        <x:v>2:43 PM</x:v>
-      </x:c>
-      <x:c r="F46" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G46" s="90" t="str"/>
-    </x:row>
-    <x:row r="47" ht="20" customHeight="1">
-      <x:c r="A47" s="84" t="str">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B47" s="87" t="str">
-        <x:v>Dittori</x:v>
-      </x:c>
-      <x:c r="C47" s="85" t="str">
-        <x:v>Blookerstein · Booth L16</x:v>
-      </x:c>
-      <x:c r="D47" s="85" t="str">
-        <x:v>2:43 PM</x:v>
-      </x:c>
-      <x:c r="E47" s="85" t="str">
-        <x:v>2:49 PM</x:v>
-      </x:c>
-      <x:c r="F47" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G47" s="86" t="str"/>
-    </x:row>
-    <x:row r="48" ht="20" customHeight="1">
-      <x:c r="A48" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B48" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C48" s="89" t="str">
-        <x:v>Block D</x:v>
-      </x:c>
-      <x:c r="D48" s="89" t="str">
-        <x:v>2:49 PM</x:v>
-      </x:c>
-      <x:c r="E48" s="89" t="str">
-        <x:v>2:50 PM</x:v>
-      </x:c>
-      <x:c r="F48" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G48" s="90" t="str"/>
-    </x:row>
-    <x:row r="49" ht="20" customHeight="1">
-      <x:c r="A49" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B49" s="95" t="str">
-        <x:v>Forge Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C49" s="93" t="str">
-        <x:v>Sponsor segment · L05</x:v>
-      </x:c>
-      <x:c r="D49" s="93" t="str">
-        <x:v>2:50 PM</x:v>
-      </x:c>
-      <x:c r="E49" s="93" t="str">
-        <x:v>3:00 PM</x:v>
-      </x:c>
-      <x:c r="F49" s="93" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G49" s="94" t="str"/>
-    </x:row>
-    <x:row r="50" ht="20" customHeight="1">
-      <x:c r="A50" s="84" t="str">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B50" s="87" t="str">
-        <x:v>End of Garbage</x:v>
-      </x:c>
-      <x:c r="C50" s="85" t="str">
-        <x:v>Joshua Rosen (Rakelock LLC) · Booth L35</x:v>
-      </x:c>
-      <x:c r="D50" s="85" t="str">
-        <x:v>3:00 PM</x:v>
-      </x:c>
-      <x:c r="E50" s="85" t="str">
-        <x:v>3:06 PM</x:v>
-      </x:c>
-      <x:c r="F50" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G50" s="86" t="str"/>
-    </x:row>
-    <x:row r="51" ht="20" customHeight="1">
-      <x:c r="A51" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B51" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C51" s="89" t="str">
-        <x:v>Block E</x:v>
-      </x:c>
-      <x:c r="D51" s="89" t="str">
-        <x:v>3:06 PM</x:v>
-      </x:c>
-      <x:c r="E51" s="89" t="str">
-        <x:v>3:07 PM</x:v>
-      </x:c>
-      <x:c r="F51" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G51" s="90" t="str"/>
-    </x:row>
-    <x:row r="52" ht="20" customHeight="1">
-      <x:c r="A52" s="84" t="str">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B52" s="87" t="str">
-        <x:v>Gravity Goblins</x:v>
-      </x:c>
-      <x:c r="C52" s="85" t="str">
-        <x:v>The Rat Zone · Booth L34</x:v>
-      </x:c>
-      <x:c r="D52" s="85" t="str">
-        <x:v>3:07 PM</x:v>
-      </x:c>
-      <x:c r="E52" s="85" t="str">
-        <x:v>3:13 PM</x:v>
-      </x:c>
-      <x:c r="F52" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G52" s="86" t="str"/>
-    </x:row>
-    <x:row r="53" ht="20" customHeight="1">
-      <x:c r="A53" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B53" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C53" s="89" t="str">
-        <x:v>Block E</x:v>
-      </x:c>
-      <x:c r="D53" s="89" t="str">
-        <x:v>3:13 PM</x:v>
-      </x:c>
-      <x:c r="E53" s="89" t="str">
-        <x:v>3:14 PM</x:v>
-      </x:c>
-      <x:c r="F53" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G53" s="90" t="str"/>
-    </x:row>
-    <x:row r="54" ht="20" customHeight="1">
-      <x:c r="A54" s="84" t="str">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B54" s="87" t="str">
-        <x:v>Creature Kitchen</x:v>
-      </x:c>
-      <x:c r="C54" s="85" t="str">
-        <x:v>The Rat Zone · Booth L33</x:v>
-      </x:c>
-      <x:c r="D54" s="85" t="str">
-        <x:v>3:14 PM</x:v>
-      </x:c>
-      <x:c r="E54" s="85" t="str">
-        <x:v>3:20 PM</x:v>
-      </x:c>
-      <x:c r="F54" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G54" s="86" t="str"/>
-    </x:row>
-    <x:row r="55" ht="20" customHeight="1">
-      <x:c r="A55" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B55" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C55" s="89" t="str">
-        <x:v>Block E</x:v>
-      </x:c>
-      <x:c r="D55" s="89" t="str">
-        <x:v>3:20 PM</x:v>
-      </x:c>
-      <x:c r="E55" s="89" t="str">
-        <x:v>3:21 PM</x:v>
-      </x:c>
-      <x:c r="F55" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G55" s="90" t="str"/>
-    </x:row>
-    <x:row r="56" ht="20" customHeight="1">
-      <x:c r="A56" s="84" t="str">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B56" s="87" t="str">
-        <x:v>Desolus</x:v>
-      </x:c>
-      <x:c r="C56" s="85" t="str">
-        <x:v>Mark J. Mayers · Booth L32</x:v>
-      </x:c>
-      <x:c r="D56" s="85" t="str">
-        <x:v>3:21 PM</x:v>
-      </x:c>
-      <x:c r="E56" s="85" t="str">
-        <x:v>3:27 PM</x:v>
-      </x:c>
-      <x:c r="F56" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G56" s="86" t="str"/>
-    </x:row>
-    <x:row r="57" ht="20" customHeight="1">
-      <x:c r="A57" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B57" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C57" s="89" t="str">
-        <x:v>Block E</x:v>
-      </x:c>
-      <x:c r="D57" s="89" t="str">
-        <x:v>3:27 PM</x:v>
-      </x:c>
-      <x:c r="E57" s="89" t="str">
-        <x:v>3:28 PM</x:v>
-      </x:c>
-      <x:c r="F57" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G57" s="90" t="str"/>
-    </x:row>
-    <x:row r="58" ht="20" customHeight="1">
-      <x:c r="A58" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B58" s="95" t="str">
-        <x:v>GeekGirlCon Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C58" s="93" t="str">
-        <x:v>Sponsor segment · L04</x:v>
-      </x:c>
-      <x:c r="D58" s="93" t="str">
-        <x:v>3:28 PM</x:v>
-      </x:c>
-      <x:c r="E58" s="93" t="str">
-        <x:v>3:35 PM</x:v>
-      </x:c>
-      <x:c r="F58" s="93" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G58" s="94" t="str"/>
-    </x:row>
-    <x:row r="59" ht="20" customHeight="1">
-      <x:c r="A59" s="84" t="str">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B59" s="87" t="str">
-        <x:v>Ascent Rivals</x:v>
-      </x:c>
-      <x:c r="C59" s="85" t="str">
-        <x:v>GENUN Games · Booth L11</x:v>
-      </x:c>
-      <x:c r="D59" s="85" t="str">
-        <x:v>3:35 PM</x:v>
-      </x:c>
-      <x:c r="E59" s="85" t="str">
-        <x:v>3:41 PM</x:v>
-      </x:c>
-      <x:c r="F59" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G59" s="86" t="str"/>
-    </x:row>
-    <x:row r="60" ht="20" customHeight="1">
-      <x:c r="A60" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B60" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C60" s="89" t="str">
-        <x:v>Block F</x:v>
-      </x:c>
-      <x:c r="D60" s="89" t="str">
-        <x:v>3:41 PM</x:v>
-      </x:c>
-      <x:c r="E60" s="89" t="str">
-        <x:v>3:42 PM</x:v>
-      </x:c>
-      <x:c r="F60" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G60" s="90" t="str"/>
-    </x:row>
-    <x:row r="61" ht="20" customHeight="1">
-      <x:c r="A61" s="84" t="str">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B61" s="87" t="str">
-        <x:v>Hamsteria</x:v>
-      </x:c>
-      <x:c r="C61" s="85" t="str">
-        <x:v>2WheelerDev · Booth L10</x:v>
-      </x:c>
-      <x:c r="D61" s="85" t="str">
-        <x:v>3:42 PM</x:v>
-      </x:c>
-      <x:c r="E61" s="85" t="str">
-        <x:v>3:48 PM</x:v>
-      </x:c>
-      <x:c r="F61" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G61" s="86" t="str"/>
-    </x:row>
-    <x:row r="62" ht="20" customHeight="1">
-      <x:c r="A62" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B62" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C62" s="89" t="str">
-        <x:v>Block F</x:v>
-      </x:c>
-      <x:c r="D62" s="89" t="str">
-        <x:v>3:48 PM</x:v>
-      </x:c>
-      <x:c r="E62" s="89" t="str">
-        <x:v>3:49 PM</x:v>
-      </x:c>
-      <x:c r="F62" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G62" s="90" t="str"/>
-    </x:row>
-    <x:row r="63" ht="20" customHeight="1">
-      <x:c r="A63" s="84" t="str">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B63" s="87" t="str">
-        <x:v>Haunted Heist</x:v>
-      </x:c>
-      <x:c r="C63" s="85" t="str">
-        <x:v>autotroph games · Booth L09</x:v>
-      </x:c>
-      <x:c r="D63" s="85" t="str">
-        <x:v>3:49 PM</x:v>
-      </x:c>
-      <x:c r="E63" s="85" t="str">
-        <x:v>3:55 PM</x:v>
-      </x:c>
-      <x:c r="F63" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G63" s="86" t="str"/>
-    </x:row>
-    <x:row r="64" ht="20" customHeight="1">
-      <x:c r="A64" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B64" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C64" s="89" t="str">
-        <x:v>Block F</x:v>
-      </x:c>
-      <x:c r="D64" s="89" t="str">
-        <x:v>3:55 PM</x:v>
-      </x:c>
-      <x:c r="E64" s="89" t="str">
-        <x:v>3:56 PM</x:v>
-      </x:c>
-      <x:c r="F64" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G64" s="90" t="str"/>
-    </x:row>
-    <x:row r="65" ht="20" customHeight="1">
-      <x:c r="A65" s="84" t="str">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B65" s="87" t="str">
-        <x:v>RUNE GUNNER</x:v>
-      </x:c>
-      <x:c r="C65" s="85" t="str">
-        <x:v>False Summit · Booth L08</x:v>
-      </x:c>
-      <x:c r="D65" s="85" t="str">
-        <x:v>3:56 PM</x:v>
-      </x:c>
-      <x:c r="E65" s="85" t="str">
-        <x:v>4:02 PM</x:v>
-      </x:c>
-      <x:c r="F65" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G65" s="86" t="str"/>
-    </x:row>
-    <x:row r="66" ht="20" customHeight="1">
-      <x:c r="A66" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B66" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C66" s="89" t="str">
-        <x:v>Block F</x:v>
-      </x:c>
-      <x:c r="D66" s="89" t="str">
-        <x:v>4:02 PM</x:v>
-      </x:c>
-      <x:c r="E66" s="89" t="str">
-        <x:v>4:03 PM</x:v>
-      </x:c>
-      <x:c r="F66" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G66" s="90" t="str"/>
-    </x:row>
-    <x:row r="67" ht="20" customHeight="1">
-      <x:c r="A67" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B67" s="95" t="str">
-        <x:v>11 Bit Studios Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C67" s="93" t="str">
-        <x:v>Sponsor segment · L06</x:v>
-      </x:c>
-      <x:c r="D67" s="93" t="str">
-        <x:v>4:03 PM</x:v>
-      </x:c>
-      <x:c r="E67" s="93" t="str">
-        <x:v>4:10 PM</x:v>
-      </x:c>
-      <x:c r="F67" s="93" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G67" s="94" t="str"/>
-    </x:row>
-    <x:row r="68" ht="20" customHeight="1">
-      <x:c r="A68" s="84" t="str">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B68" s="87" t="str">
-        <x:v>Telera</x:v>
-      </x:c>
-      <x:c r="C68" s="85" t="str">
-        <x:v>Entropico · Booth U21</x:v>
-      </x:c>
-      <x:c r="D68" s="85" t="str">
-        <x:v>4:10 PM</x:v>
-      </x:c>
-      <x:c r="E68" s="85" t="str">
-        <x:v>4:16 PM</x:v>
-      </x:c>
-      <x:c r="F68" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G68" s="86" t="str"/>
-    </x:row>
-    <x:row r="69" ht="20" customHeight="1">
-      <x:c r="A69" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B69" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C69" s="89" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D69" s="89" t="str">
-        <x:v>4:16 PM</x:v>
-      </x:c>
-      <x:c r="E69" s="89" t="str">
-        <x:v>4:17 PM</x:v>
-      </x:c>
-      <x:c r="F69" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G69" s="90" t="str"/>
-    </x:row>
-    <x:row r="70" ht="20" customHeight="1">
-      <x:c r="A70" s="84" t="str">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B70" s="87" t="str">
-        <x:v>Hogen</x:v>
-      </x:c>
-      <x:c r="C70" s="85" t="str">
-        <x:v>Scrappyard Games · Booth U22</x:v>
-      </x:c>
-      <x:c r="D70" s="85" t="str">
-        <x:v>4:17 PM</x:v>
-      </x:c>
-      <x:c r="E70" s="85" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="F70" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G70" s="86" t="str"/>
-    </x:row>
-    <x:row r="71" ht="20" customHeight="1">
-      <x:c r="A71" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B71" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C71" s="89" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D71" s="89" t="str">
-        <x:v>4:23 PM</x:v>
-      </x:c>
-      <x:c r="E71" s="89" t="str">
-        <x:v>4:24 PM</x:v>
-      </x:c>
-      <x:c r="F71" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G71" s="90" t="str"/>
-    </x:row>
-    <x:row r="72" ht="20" customHeight="1">
-      <x:c r="A72" s="84" t="str">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B72" s="87" t="str">
-        <x:v>WILL: Follow The Light</x:v>
-      </x:c>
-      <x:c r="C72" s="85" t="str">
-        <x:v>TomorrowHead Studio · Booth U23</x:v>
-      </x:c>
-      <x:c r="D72" s="85" t="str">
-        <x:v>4:24 PM</x:v>
-      </x:c>
-      <x:c r="E72" s="85" t="str">
-        <x:v>4:30 PM</x:v>
-      </x:c>
-      <x:c r="F72" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G72" s="86" t="str"/>
-    </x:row>
-    <x:row r="73" ht="20" customHeight="1">
-      <x:c r="A73" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B73" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C73" s="89" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D73" s="89" t="str">
-        <x:v>4:30 PM</x:v>
-      </x:c>
-      <x:c r="E73" s="89" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="F73" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G73" s="90" t="str"/>
-    </x:row>
-    <x:row r="74" ht="20" customHeight="1">
-      <x:c r="A74" s="84" t="str">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B74" s="87" t="str">
-        <x:v>Turning Manor</x:v>
-      </x:c>
-      <x:c r="C74" s="85" t="str">
-        <x:v>Sabbatical Games · Booth U24</x:v>
-      </x:c>
-      <x:c r="D74" s="85" t="str">
-        <x:v>4:31 PM</x:v>
-      </x:c>
-      <x:c r="E74" s="85" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="F74" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G74" s="86" t="str"/>
-    </x:row>
-    <x:row r="75" ht="20" customHeight="1">
-      <x:c r="A75" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B75" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C75" s="89" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D75" s="89" t="str">
-        <x:v>4:37 PM</x:v>
-      </x:c>
-      <x:c r="E75" s="89" t="str">
-        <x:v>4:38 PM</x:v>
-      </x:c>
-      <x:c r="F75" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G75" s="90" t="str"/>
-    </x:row>
-    <x:row r="76" ht="20" customHeight="1">
-      <x:c r="A76" s="84" t="str">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B76" s="87" t="str">
-        <x:v>Steel Swarm: SURVIVOR</x:v>
-      </x:c>
-      <x:c r="C76" s="85" t="str">
-        <x:v>Clay Token Game Studio, Inc. · Booth U25</x:v>
-      </x:c>
-      <x:c r="D76" s="85" t="str">
-        <x:v>4:38 PM</x:v>
-      </x:c>
-      <x:c r="E76" s="85" t="str">
-        <x:v>4:44 PM</x:v>
-      </x:c>
-      <x:c r="F76" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G76" s="86" t="str"/>
-    </x:row>
-    <x:row r="77" ht="20" customHeight="1">
-      <x:c r="A77" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B77" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C77" s="89" t="str">
-        <x:v>Block G</x:v>
-      </x:c>
-      <x:c r="D77" s="89" t="str">
-        <x:v>4:44 PM</x:v>
-      </x:c>
-      <x:c r="E77" s="89" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="F77" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G77" s="90" t="str"/>
-    </x:row>
-    <x:row r="78" ht="20" customHeight="1">
-      <x:c r="A78" s="92" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B78" s="95" t="str">
-        <x:v>NDVisibility Sponsor Segment</x:v>
-      </x:c>
-      <x:c r="C78" s="93" t="str">
-        <x:v>Sponsor segment · 000</x:v>
-      </x:c>
-      <x:c r="D78" s="93" t="str">
-        <x:v>4:45 PM</x:v>
-      </x:c>
-      <x:c r="E78" s="93" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="F78" s="93" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G78" s="94" t="str"/>
-    </x:row>
-    <x:row r="79" ht="20" customHeight="1">
-      <x:c r="A79" s="84" t="str">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B79" s="87" t="str">
-        <x:v>HYPERFIST</x:v>
-      </x:c>
-      <x:c r="C79" s="85" t="str">
-        <x:v>Chirality · Booth U15</x:v>
-      </x:c>
-      <x:c r="D79" s="85" t="str">
-        <x:v>4:55 PM</x:v>
-      </x:c>
-      <x:c r="E79" s="85" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="F79" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G79" s="86" t="str"/>
-    </x:row>
-    <x:row r="80" ht="20" customHeight="1">
-      <x:c r="A80" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B80" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C80" s="89" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D80" s="89" t="str">
-        <x:v>5:01 PM</x:v>
-      </x:c>
-      <x:c r="E80" s="89" t="str">
-        <x:v>5:02 PM</x:v>
-      </x:c>
-      <x:c r="F80" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G80" s="90" t="str"/>
-    </x:row>
-    <x:row r="81" ht="20" customHeight="1">
-      <x:c r="A81" s="84" t="str">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B81" s="87" t="str">
-        <x:v>Nightmare Kitchen</x:v>
-      </x:c>
-      <x:c r="C81" s="85" t="str">
-        <x:v>Byteback Studios · Booth U16</x:v>
-      </x:c>
-      <x:c r="D81" s="85" t="str">
-        <x:v>5:02 PM</x:v>
-      </x:c>
-      <x:c r="E81" s="85" t="str">
-        <x:v>5:08 PM</x:v>
-      </x:c>
-      <x:c r="F81" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G81" s="86" t="str"/>
-    </x:row>
-    <x:row r="82" ht="20" customHeight="1">
-      <x:c r="A82" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B82" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C82" s="89" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D82" s="89" t="str">
-        <x:v>5:08 PM</x:v>
-      </x:c>
-      <x:c r="E82" s="89" t="str">
-        <x:v>5:09 PM</x:v>
-      </x:c>
-      <x:c r="F82" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G82" s="90" t="str"/>
-    </x:row>
-    <x:row r="83" ht="20" customHeight="1">
-      <x:c r="A83" s="84" t="str">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B83" s="87" t="str">
-        <x:v>Shroomwood</x:v>
-      </x:c>
-      <x:c r="C83" s="85" t="str">
-        <x:v>Sporelite Games · Booth U17</x:v>
-      </x:c>
-      <x:c r="D83" s="85" t="str">
-        <x:v>5:09 PM</x:v>
-      </x:c>
-      <x:c r="E83" s="85" t="str">
-        <x:v>5:15 PM</x:v>
-      </x:c>
-      <x:c r="F83" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G83" s="86" t="str"/>
-    </x:row>
-    <x:row r="84" ht="20" customHeight="1">
-      <x:c r="A84" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B84" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C84" s="89" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D84" s="89" t="str">
-        <x:v>5:15 PM</x:v>
-      </x:c>
-      <x:c r="E84" s="89" t="str">
-        <x:v>5:16 PM</x:v>
-      </x:c>
-      <x:c r="F84" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G84" s="90" t="str"/>
-    </x:row>
-    <x:row r="85" ht="20" customHeight="1">
-      <x:c r="A85" s="84" t="str">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B85" s="87" t="str">
-        <x:v>Knockout 2: Wrath of the Karen</x:v>
-      </x:c>
-      <x:c r="C85" s="85" t="str">
-        <x:v>ExceptioNULL Games · Booth U18</x:v>
-      </x:c>
-      <x:c r="D85" s="85" t="str">
-        <x:v>5:16 PM</x:v>
-      </x:c>
-      <x:c r="E85" s="85" t="str">
-        <x:v>5:22 PM</x:v>
-      </x:c>
-      <x:c r="F85" s="85" t="str">
-        <x:v>E</x:v>
-      </x:c>
-      <x:c r="G85" s="86" t="str"/>
-    </x:row>
-    <x:row r="86" ht="20" customHeight="1">
-      <x:c r="A86" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B86" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C86" s="89" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D86" s="89" t="str">
-        <x:v>5:22 PM</x:v>
-      </x:c>
-      <x:c r="E86" s="89" t="str">
-        <x:v>5:23 PM</x:v>
-      </x:c>
-      <x:c r="F86" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G86" s="90" t="str"/>
-    </x:row>
-    <x:row r="87" ht="20" customHeight="1">
-      <x:c r="A87" s="84" t="str">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B87" s="87" t="str">
-        <x:v>Cooking Fist</x:v>
-      </x:c>
-      <x:c r="C87" s="85" t="str">
-        <x:v>Spaghetti Code LLC · Booth U19</x:v>
-      </x:c>
-      <x:c r="D87" s="85" t="str">
-        <x:v>5:23 PM</x:v>
-      </x:c>
-      <x:c r="E87" s="85" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="F87" s="85" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G87" s="86" t="str"/>
-    </x:row>
-    <x:row r="88" ht="20" customHeight="1">
-      <x:c r="A88" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B88" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C88" s="89" t="str">
-        <x:v>Block H</x:v>
-      </x:c>
-      <x:c r="D88" s="89" t="str">
-        <x:v>5:29 PM</x:v>
-      </x:c>
-      <x:c r="E88" s="89" t="str">
-        <x:v>5:30 PM</x:v>
-      </x:c>
-      <x:c r="F88" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G88" s="90" t="str"/>
-    </x:row>
-    <x:row r="89" ht="20" customHeight="1">
-      <x:c r="A89" s="96" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B89" s="99" t="str">
-        <x:v>Ukrainian Games Videos</x:v>
-      </x:c>
-      <x:c r="C89" s="97" t="str">
-        <x:v>International showcase · 000</x:v>
-      </x:c>
-      <x:c r="D89" s="97" t="str">
-        <x:v>5:30 PM</x:v>
-      </x:c>
-      <x:c r="E89" s="97" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="F89" s="97" t="str">
-        <x:v>Prerecorded</x:v>
-      </x:c>
-      <x:c r="G89" s="98" t="str"/>
-    </x:row>
-    <x:row r="90" ht="20" customHeight="1">
-      <x:c r="A90" s="84" t="str">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B90" s="87" t="str">
-        <x:v>Killing Baby Hitler</x:v>
-      </x:c>
-      <x:c r="C90" s="85" t="str">
-        <x:v>The Coffee Industrial Complex · Booth U14</x:v>
-      </x:c>
-      <x:c r="D90" s="85" t="str">
-        <x:v>5:35 PM</x:v>
-      </x:c>
-      <x:c r="E90" s="85" t="str">
-        <x:v>5:41 PM</x:v>
-      </x:c>
-      <x:c r="F90" s="85" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G90" s="86" t="str"/>
-    </x:row>
-    <x:row r="91" ht="20" customHeight="1">
-      <x:c r="A91" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B91" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C91" s="89" t="str">
-        <x:v>Block I</x:v>
-      </x:c>
-      <x:c r="D91" s="89" t="str">
-        <x:v>5:41 PM</x:v>
-      </x:c>
-      <x:c r="E91" s="89" t="str">
-        <x:v>5:42 PM</x:v>
-      </x:c>
-      <x:c r="F91" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G91" s="90" t="str"/>
-    </x:row>
-    <x:row r="92" ht="20" customHeight="1">
-      <x:c r="A92" s="84" t="str">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B92" s="87" t="str">
-        <x:v>The Assessment</x:v>
-      </x:c>
-      <x:c r="C92" s="85" t="str">
-        <x:v>Miga Games · Booth U11</x:v>
-      </x:c>
-      <x:c r="D92" s="85" t="str">
-        <x:v>5:42 PM</x:v>
-      </x:c>
-      <x:c r="E92" s="85" t="str">
-        <x:v>5:48 PM</x:v>
-      </x:c>
-      <x:c r="F92" s="85" t="str">
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="G92" s="86" t="str"/>
-    </x:row>
-    <x:row r="93" ht="20" customHeight="1">
-      <x:c r="A93" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B93" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C93" s="89" t="str">
-        <x:v>Block I</x:v>
-      </x:c>
-      <x:c r="D93" s="89" t="str">
-        <x:v>5:48 PM</x:v>
-      </x:c>
-      <x:c r="E93" s="89" t="str">
-        <x:v>5:49 PM</x:v>
-      </x:c>
-      <x:c r="F93" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G93" s="90" t="str"/>
-    </x:row>
-    <x:row r="94" ht="20" customHeight="1">
-      <x:c r="A94" s="96" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B94" s="99" t="str">
-        <x:v>Chile Games Showcase Video</x:v>
-      </x:c>
-      <x:c r="C94" s="97" t="str">
-        <x:v>International showcase · 000</x:v>
-      </x:c>
-      <x:c r="D94" s="97" t="str">
-        <x:v>5:49 PM</x:v>
-      </x:c>
-      <x:c r="E94" s="97" t="str">
-        <x:v>5:54 PM</x:v>
-      </x:c>
-      <x:c r="F94" s="97" t="str">
-        <x:v>Prerecorded</x:v>
-      </x:c>
-      <x:c r="G94" s="98" t="str"/>
-    </x:row>
-    <x:row r="95" ht="20" customHeight="1">
-      <x:c r="A95" s="88" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="B95" s="91" t="str">
-        <x:v>Break / Transition</x:v>
-      </x:c>
-      <x:c r="C95" s="89" t="str">
-        <x:v>Block I</x:v>
-      </x:c>
-      <x:c r="D95" s="89" t="str">
-        <x:v>5:54 PM</x:v>
-      </x:c>
-      <x:c r="E95" s="89" t="str">
-        <x:v>5:55 PM</x:v>
-      </x:c>
-      <x:c r="F95" s="89" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G95" s="90" t="str"/>
-    </x:row>
-    <x:row r="96" ht="20" customHeight="1">
-      <x:c r="A96" s="100" t="str">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B96" s="103" t="str">
-        <x:v>Closing / Thank You</x:v>
-      </x:c>
-      <x:c r="C96" s="101" t="str">
-        <x:v>Seattle Indies</x:v>
-      </x:c>
-      <x:c r="D96" s="101" t="str">
-        <x:v>5:55 PM</x:v>
-      </x:c>
-      <x:c r="E96" s="101" t="str">
-        <x:v>6:05 PM</x:v>
-      </x:c>
-      <x:c r="F96" s="101" t="str">
-        <x:v>All Hosts</x:v>
-      </x:c>
-      <x:c r="G96" s="102" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A3:G3"/>
-    <x:mergeCell ref="A2:G2"/>
-    <x:mergeCell ref="A1:G1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="7" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="77" t="str">
+        <v>Seattle Indies Expo - SIX 2026 | Run of Show</v>
+      </c>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+    </row>
+    <row r="2" ht="21" customHeight="1">
+      <c r="A2" s="78" t="str">
+        <v>Run of Show - Production Schedule</v>
+      </c>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="38" t="str">
+        <v>Host A = Unavailable | Host B = AbdallahSmash | Host C = MacnCheesep1z | Host D = Rockagoth | Host E = AlchemistJoker</v>
+      </c>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="79" t="str">
+        <v>SEG</v>
+      </c>
+      <c r="B4" s="79" t="str">
+        <v>GAME / BREAK</v>
+      </c>
+      <c r="C4" s="79" t="str">
+        <v>DEVELOPER / PUBLISHER</v>
+      </c>
+      <c r="D4" s="79" t="str">
+        <v>START</v>
+      </c>
+      <c r="E4" s="79" t="str">
+        <v>END</v>
+      </c>
+      <c r="F4" s="79" t="str">
+        <v>HOST</v>
+      </c>
+      <c r="G4" s="79" t="str">
+        <v>PRODUCTION NOTES</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="80" t="str">
+        <v>-</v>
+      </c>
+      <c r="B5" s="83" t="str">
+        <v>SIX Hype Hour</v>
+      </c>
+      <c r="C5" s="81" t="str">
+        <v>Seattle Indies</v>
+      </c>
+      <c r="D5" s="81" t="str">
+        <v>10:00 AM</v>
+      </c>
+      <c r="E5" s="81" t="str">
+        <v>12:00 PM</v>
+      </c>
+      <c r="F5" s="81" t="str">
+        <v>Prerecorded</v>
+      </c>
+      <c r="G5" s="82" t="str"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="84" t="str">
+        <v>1</v>
+      </c>
+      <c r="B6" s="87" t="str">
+        <v>Tricky and the Dream Caster</v>
+      </c>
+      <c r="C6" s="85" t="str">
+        <v>PossQueen · Booth L27</v>
+      </c>
+      <c r="D6" s="85" t="str">
+        <v>12:00 PM</v>
+      </c>
+      <c r="E6" s="85" t="str">
+        <v>12:06 PM</v>
+      </c>
+      <c r="F6" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G6" s="86" t="str"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B7" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C7" s="89" t="str">
+        <v>Block A</v>
+      </c>
+      <c r="D7" s="89" t="str">
+        <v>12:06 PM</v>
+      </c>
+      <c r="E7" s="89" t="str">
+        <v>12:07 PM</v>
+      </c>
+      <c r="F7" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G7" s="90" t="str"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="84" t="str">
+        <v>2</v>
+      </c>
+      <c r="B8" s="87" t="str">
+        <v>TileShire</v>
+      </c>
+      <c r="C8" s="85" t="str">
+        <v>Boss Blob · Booth L28</v>
+      </c>
+      <c r="D8" s="85" t="str">
+        <v>12:07 PM</v>
+      </c>
+      <c r="E8" s="85" t="str">
+        <v>12:13 PM</v>
+      </c>
+      <c r="F8" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G8" s="86" t="str"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B9" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C9" s="89" t="str">
+        <v>Block A</v>
+      </c>
+      <c r="D9" s="89" t="str">
+        <v>12:13 PM</v>
+      </c>
+      <c r="E9" s="89" t="str">
+        <v>12:14 PM</v>
+      </c>
+      <c r="F9" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G9" s="90" t="str"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="84" t="str">
+        <v>3</v>
+      </c>
+      <c r="B10" s="87" t="str">
+        <v>Wrestle Story</v>
+      </c>
+      <c r="C10" s="85" t="str">
+        <v>Tic Toc Games · Booth L29</v>
+      </c>
+      <c r="D10" s="85" t="str">
+        <v>12:14 PM</v>
+      </c>
+      <c r="E10" s="85" t="str">
+        <v>12:20 PM</v>
+      </c>
+      <c r="F10" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G10" s="86" t="str"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B11" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C11" s="89" t="str">
+        <v>Block A</v>
+      </c>
+      <c r="D11" s="89" t="str">
+        <v>12:20 PM</v>
+      </c>
+      <c r="E11" s="89" t="str">
+        <v>12:21 PM</v>
+      </c>
+      <c r="F11" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G11" s="90" t="str"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="84" t="str">
+        <v>4</v>
+      </c>
+      <c r="B12" s="87" t="str">
+        <v>Breach Of Contract</v>
+      </c>
+      <c r="C12" s="85" t="str">
+        <v>Fern Sprout Studios · Booth L30</v>
+      </c>
+      <c r="D12" s="85" t="str">
+        <v>12:21 PM</v>
+      </c>
+      <c r="E12" s="85" t="str">
+        <v>12:27 PM</v>
+      </c>
+      <c r="F12" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G12" s="86" t="str"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B13" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C13" s="89" t="str">
+        <v>Block A</v>
+      </c>
+      <c r="D13" s="89" t="str">
+        <v>12:27 PM</v>
+      </c>
+      <c r="E13" s="89" t="str">
+        <v>12:28 PM</v>
+      </c>
+      <c r="F13" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G13" s="90" t="str"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="84" t="str">
+        <v>5</v>
+      </c>
+      <c r="B14" s="87" t="str">
+        <v>Dungeon Bodega Simulator</v>
+      </c>
+      <c r="C14" s="85" t="str">
+        <v>Alien Fruit Games · Booth L31</v>
+      </c>
+      <c r="D14" s="85" t="str">
+        <v>12:28 PM</v>
+      </c>
+      <c r="E14" s="85" t="str">
+        <v>12:34 PM</v>
+      </c>
+      <c r="F14" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G14" s="86" t="str"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B15" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C15" s="89" t="str">
+        <v>Block A</v>
+      </c>
+      <c r="D15" s="89" t="str">
+        <v>12:34 PM</v>
+      </c>
+      <c r="E15" s="89" t="str">
+        <v>12:35 PM</v>
+      </c>
+      <c r="F15" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G15" s="90" t="str"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B16" s="95" t="str">
+        <v>DigiPen Sponsor Segment</v>
+      </c>
+      <c r="C16" s="93" t="str">
+        <v>Sponsor segment · L01</v>
+      </c>
+      <c r="D16" s="93" t="str">
+        <v>12:35 PM</v>
+      </c>
+      <c r="E16" s="93" t="str">
+        <v>12:45 PM</v>
+      </c>
+      <c r="F16" s="93" t="str">
+        <v>B</v>
+      </c>
+      <c r="G16" s="94" t="str"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="84" t="str">
+        <v>6</v>
+      </c>
+      <c r="B17" s="87" t="str">
+        <v>SCP: Antimemetics Division</v>
+      </c>
+      <c r="C17" s="85" t="str">
+        <v>Quadrant Five · Booth L22</v>
+      </c>
+      <c r="D17" s="85" t="str">
+        <v>12:45 PM</v>
+      </c>
+      <c r="E17" s="85" t="str">
+        <v>12:51 PM</v>
+      </c>
+      <c r="F17" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G17" s="86" t="str"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B18" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C18" s="89" t="str">
+        <v>Block B</v>
+      </c>
+      <c r="D18" s="89" t="str">
+        <v>12:51 PM</v>
+      </c>
+      <c r="E18" s="89" t="str">
+        <v>12:52 PM</v>
+      </c>
+      <c r="F18" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G18" s="90" t="str"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="84" t="str">
+        <v>7</v>
+      </c>
+      <c r="B19" s="87" t="str">
+        <v>Manafinder II</v>
+      </c>
+      <c r="C19" s="85" t="str">
+        <v>Wolfsden LLC · Booth L23</v>
+      </c>
+      <c r="D19" s="85" t="str">
+        <v>12:52 PM</v>
+      </c>
+      <c r="E19" s="85" t="str">
+        <v>12:58 PM</v>
+      </c>
+      <c r="F19" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G19" s="86" t="str"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B20" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C20" s="89" t="str">
+        <v>Block B</v>
+      </c>
+      <c r="D20" s="89" t="str">
+        <v>12:58 PM</v>
+      </c>
+      <c r="E20" s="89" t="str">
+        <v>12:59 PM</v>
+      </c>
+      <c r="F20" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G20" s="90" t="str"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="84" t="str">
+        <v>8</v>
+      </c>
+      <c r="B21" s="87" t="str">
+        <v>Malice In Wonderland</v>
+      </c>
+      <c r="C21" s="85" t="str">
+        <v>Slyglass Games · Booth L24</v>
+      </c>
+      <c r="D21" s="85" t="str">
+        <v>12:59 PM</v>
+      </c>
+      <c r="E21" s="85" t="str">
+        <v>1:05 PM</v>
+      </c>
+      <c r="F21" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G21" s="86" t="str"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B22" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C22" s="89" t="str">
+        <v>Block B</v>
+      </c>
+      <c r="D22" s="89" t="str">
+        <v>1:05 PM</v>
+      </c>
+      <c r="E22" s="89" t="str">
+        <v>1:06 PM</v>
+      </c>
+      <c r="F22" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G22" s="90" t="str"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="84" t="str">
+        <v>9</v>
+      </c>
+      <c r="B23" s="87" t="str">
+        <v>Project Cradle</v>
+      </c>
+      <c r="C23" s="85" t="str">
+        <v>ShazySoft · Booth L25</v>
+      </c>
+      <c r="D23" s="85" t="str">
+        <v>1:06 PM</v>
+      </c>
+      <c r="E23" s="85" t="str">
+        <v>1:12 PM</v>
+      </c>
+      <c r="F23" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G23" s="86" t="str"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B24" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C24" s="89" t="str">
+        <v>Block B</v>
+      </c>
+      <c r="D24" s="89" t="str">
+        <v>1:12 PM</v>
+      </c>
+      <c r="E24" s="89" t="str">
+        <v>1:13 PM</v>
+      </c>
+      <c r="F24" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G24" s="90" t="str"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="84" t="str">
+        <v>10</v>
+      </c>
+      <c r="B25" s="87" t="str">
+        <v>Diabolocracy</v>
+      </c>
+      <c r="C25" s="85" t="str">
+        <v>Chaos Gremlin Games · Booth L26</v>
+      </c>
+      <c r="D25" s="85" t="str">
+        <v>1:13 PM</v>
+      </c>
+      <c r="E25" s="85" t="str">
+        <v>1:19 PM</v>
+      </c>
+      <c r="F25" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G25" s="86" t="str"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B26" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C26" s="89" t="str">
+        <v>Block B</v>
+      </c>
+      <c r="D26" s="89" t="str">
+        <v>1:19 PM</v>
+      </c>
+      <c r="E26" s="89" t="str">
+        <v>1:20 PM</v>
+      </c>
+      <c r="F26" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G26" s="90" t="str"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B27" s="95" t="str">
+        <v>AIE Sponsor Segment</v>
+      </c>
+      <c r="C27" s="93" t="str">
+        <v>Sponsor segment · L02</v>
+      </c>
+      <c r="D27" s="93" t="str">
+        <v>1:20 PM</v>
+      </c>
+      <c r="E27" s="93" t="str">
+        <v>1:30 PM</v>
+      </c>
+      <c r="F27" s="93" t="str">
+        <v>B</v>
+      </c>
+      <c r="G27" s="94" t="str"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="84" t="str">
+        <v>11</v>
+      </c>
+      <c r="B28" s="87" t="str">
+        <v>Seedborne Soldiers</v>
+      </c>
+      <c r="C28" s="85" t="str">
+        <v>Hat Wobble Games · Booth L17</v>
+      </c>
+      <c r="D28" s="85" t="str">
+        <v>1:30 PM</v>
+      </c>
+      <c r="E28" s="85" t="str">
+        <v>1:36 PM</v>
+      </c>
+      <c r="F28" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G28" s="86" t="str"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B29" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C29" s="89" t="str">
+        <v>Block C</v>
+      </c>
+      <c r="D29" s="89" t="str">
+        <v>1:36 PM</v>
+      </c>
+      <c r="E29" s="89" t="str">
+        <v>1:37 PM</v>
+      </c>
+      <c r="F29" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G29" s="90" t="str"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="84" t="str">
+        <v>12</v>
+      </c>
+      <c r="B30" s="87" t="str">
+        <v>Super Choppy</v>
+      </c>
+      <c r="C30" s="85" t="str">
+        <v>Sumoshell Bombfunk · Booth L18</v>
+      </c>
+      <c r="D30" s="85" t="str">
+        <v>1:37 PM</v>
+      </c>
+      <c r="E30" s="85" t="str">
+        <v>1:43 PM</v>
+      </c>
+      <c r="F30" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G30" s="86" t="str"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B31" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C31" s="89" t="str">
+        <v>Block C</v>
+      </c>
+      <c r="D31" s="89" t="str">
+        <v>1:43 PM</v>
+      </c>
+      <c r="E31" s="89" t="str">
+        <v>1:44 PM</v>
+      </c>
+      <c r="F31" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G31" s="90" t="str"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="84" t="str">
+        <v>13</v>
+      </c>
+      <c r="B32" s="87" t="str">
+        <v>Dig Too Deep</v>
+      </c>
+      <c r="C32" s="85" t="str">
+        <v>Punch Up Games · Booth L19</v>
+      </c>
+      <c r="D32" s="85" t="str">
+        <v>1:44 PM</v>
+      </c>
+      <c r="E32" s="85" t="str">
+        <v>1:50 PM</v>
+      </c>
+      <c r="F32" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G32" s="86" t="str"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B33" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C33" s="89" t="str">
+        <v>Block C</v>
+      </c>
+      <c r="D33" s="89" t="str">
+        <v>1:50 PM</v>
+      </c>
+      <c r="E33" s="89" t="str">
+        <v>1:51 PM</v>
+      </c>
+      <c r="F33" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G33" s="90" t="str"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="84" t="str">
+        <v>14</v>
+      </c>
+      <c r="B34" s="87" t="str">
+        <v>Nimbit Frontier</v>
+      </c>
+      <c r="C34" s="85" t="str">
+        <v>Megasploot · Booth L20</v>
+      </c>
+      <c r="D34" s="85" t="str">
+        <v>1:51 PM</v>
+      </c>
+      <c r="E34" s="85" t="str">
+        <v>1:57 PM</v>
+      </c>
+      <c r="F34" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G34" s="86" t="str"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B35" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C35" s="89" t="str">
+        <v>Block C</v>
+      </c>
+      <c r="D35" s="89" t="str">
+        <v>1:57 PM</v>
+      </c>
+      <c r="E35" s="89" t="str">
+        <v>1:58 PM</v>
+      </c>
+      <c r="F35" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G35" s="90" t="str"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="84" t="str">
+        <v>15</v>
+      </c>
+      <c r="B36" s="87" t="str">
+        <v>We Need An Army</v>
+      </c>
+      <c r="C36" s="85" t="str">
+        <v>Elder Bear Games · Booth L21</v>
+      </c>
+      <c r="D36" s="85" t="str">
+        <v>1:58 PM</v>
+      </c>
+      <c r="E36" s="85" t="str">
+        <v>2:04 PM</v>
+      </c>
+      <c r="F36" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G36" s="86" t="str"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B37" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C37" s="89" t="str">
+        <v>Block C</v>
+      </c>
+      <c r="D37" s="89" t="str">
+        <v>2:04 PM</v>
+      </c>
+      <c r="E37" s="89" t="str">
+        <v>2:05 PM</v>
+      </c>
+      <c r="F37" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G37" s="90" t="str"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B38" s="95" t="str">
+        <v>Unity Sponsor Segment</v>
+      </c>
+      <c r="C38" s="93" t="str">
+        <v>Sponsor segment · L03</v>
+      </c>
+      <c r="D38" s="93" t="str">
+        <v>2:05 PM</v>
+      </c>
+      <c r="E38" s="93" t="str">
+        <v>2:15 PM</v>
+      </c>
+      <c r="F38" s="93" t="str">
+        <v>C</v>
+      </c>
+      <c r="G38" s="94" t="str"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="84" t="str">
+        <v>16</v>
+      </c>
+      <c r="B39" s="87" t="str">
+        <v>Feeding Gooble</v>
+      </c>
+      <c r="C39" s="85" t="str">
+        <v>Displacer Labs · Booth L12</v>
+      </c>
+      <c r="D39" s="85" t="str">
+        <v>2:15 PM</v>
+      </c>
+      <c r="E39" s="85" t="str">
+        <v>2:21 PM</v>
+      </c>
+      <c r="F39" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G39" s="86" t="str"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B40" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C40" s="89" t="str">
+        <v>Block D</v>
+      </c>
+      <c r="D40" s="89" t="str">
+        <v>2:21 PM</v>
+      </c>
+      <c r="E40" s="89" t="str">
+        <v>2:22 PM</v>
+      </c>
+      <c r="F40" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G40" s="90" t="str"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="84" t="str">
+        <v>17</v>
+      </c>
+      <c r="B41" s="87" t="str">
+        <v>BroomSweeper</v>
+      </c>
+      <c r="C41" s="85" t="str">
+        <v>BandWidth Games · Booth L13</v>
+      </c>
+      <c r="D41" s="85" t="str">
+        <v>2:22 PM</v>
+      </c>
+      <c r="E41" s="85" t="str">
+        <v>2:28 PM</v>
+      </c>
+      <c r="F41" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G41" s="86" t="str"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B42" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C42" s="89" t="str">
+        <v>Block D</v>
+      </c>
+      <c r="D42" s="89" t="str">
+        <v>2:28 PM</v>
+      </c>
+      <c r="E42" s="89" t="str">
+        <v>2:29 PM</v>
+      </c>
+      <c r="F42" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G42" s="90" t="str"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="84" t="str">
+        <v>18</v>
+      </c>
+      <c r="B43" s="87" t="str">
+        <v>Fairy Circle</v>
+      </c>
+      <c r="C43" s="85" t="str">
+        <v>Play Hooky · Booth L14</v>
+      </c>
+      <c r="D43" s="85" t="str">
+        <v>2:29 PM</v>
+      </c>
+      <c r="E43" s="85" t="str">
+        <v>2:35 PM</v>
+      </c>
+      <c r="F43" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G43" s="86" t="str"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B44" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C44" s="89" t="str">
+        <v>Block D</v>
+      </c>
+      <c r="D44" s="89" t="str">
+        <v>2:35 PM</v>
+      </c>
+      <c r="E44" s="89" t="str">
+        <v>2:36 PM</v>
+      </c>
+      <c r="F44" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G44" s="90" t="str"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="84" t="str">
+        <v>19</v>
+      </c>
+      <c r="B45" s="87" t="str">
+        <v>MYRIORAMA</v>
+      </c>
+      <c r="C45" s="85" t="str">
+        <v>J&amp;K Games · Booth L15</v>
+      </c>
+      <c r="D45" s="85" t="str">
+        <v>2:36 PM</v>
+      </c>
+      <c r="E45" s="85" t="str">
+        <v>2:42 PM</v>
+      </c>
+      <c r="F45" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G45" s="86" t="str"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B46" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C46" s="89" t="str">
+        <v>Block D</v>
+      </c>
+      <c r="D46" s="89" t="str">
+        <v>2:42 PM</v>
+      </c>
+      <c r="E46" s="89" t="str">
+        <v>2:43 PM</v>
+      </c>
+      <c r="F46" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G46" s="90" t="str"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="84" t="str">
+        <v>20</v>
+      </c>
+      <c r="B47" s="87" t="str">
+        <v>Dittori</v>
+      </c>
+      <c r="C47" s="85" t="str">
+        <v>Blookerstein · Booth L16</v>
+      </c>
+      <c r="D47" s="85" t="str">
+        <v>2:43 PM</v>
+      </c>
+      <c r="E47" s="85" t="str">
+        <v>2:49 PM</v>
+      </c>
+      <c r="F47" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G47" s="86" t="str"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B48" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C48" s="89" t="str">
+        <v>Block D</v>
+      </c>
+      <c r="D48" s="89" t="str">
+        <v>2:49 PM</v>
+      </c>
+      <c r="E48" s="89" t="str">
+        <v>2:50 PM</v>
+      </c>
+      <c r="F48" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G48" s="90" t="str"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B49" s="95" t="str">
+        <v>Forge Sponsor Segment</v>
+      </c>
+      <c r="C49" s="93" t="str">
+        <v>Sponsor segment · L05</v>
+      </c>
+      <c r="D49" s="93" t="str">
+        <v>2:50 PM</v>
+      </c>
+      <c r="E49" s="93" t="str">
+        <v>3:00 PM</v>
+      </c>
+      <c r="F49" s="93" t="str">
+        <v>D</v>
+      </c>
+      <c r="G49" s="94" t="str"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="84" t="str">
+        <v>21</v>
+      </c>
+      <c r="B50" s="87" t="str">
+        <v>End of Garbage</v>
+      </c>
+      <c r="C50" s="85" t="str">
+        <v>Joshua Rosen (Rakelock LLC) · Booth L35</v>
+      </c>
+      <c r="D50" s="85" t="str">
+        <v>3:00 PM</v>
+      </c>
+      <c r="E50" s="85" t="str">
+        <v>3:06 PM</v>
+      </c>
+      <c r="F50" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G50" s="86" t="str"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B51" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C51" s="89" t="str">
+        <v>Block E</v>
+      </c>
+      <c r="D51" s="89" t="str">
+        <v>3:06 PM</v>
+      </c>
+      <c r="E51" s="89" t="str">
+        <v>3:07 PM</v>
+      </c>
+      <c r="F51" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G51" s="90" t="str"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="84" t="str">
+        <v>22</v>
+      </c>
+      <c r="B52" s="87" t="str">
+        <v>Gravity Goblins</v>
+      </c>
+      <c r="C52" s="85" t="str">
+        <v>The Rat Zone · Booth L34</v>
+      </c>
+      <c r="D52" s="85" t="str">
+        <v>3:07 PM</v>
+      </c>
+      <c r="E52" s="85" t="str">
+        <v>3:13 PM</v>
+      </c>
+      <c r="F52" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G52" s="86" t="str"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B53" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C53" s="89" t="str">
+        <v>Block E</v>
+      </c>
+      <c r="D53" s="89" t="str">
+        <v>3:13 PM</v>
+      </c>
+      <c r="E53" s="89" t="str">
+        <v>3:14 PM</v>
+      </c>
+      <c r="F53" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G53" s="90" t="str"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="84" t="str">
+        <v>23</v>
+      </c>
+      <c r="B54" s="87" t="str">
+        <v>Creature Kitchen</v>
+      </c>
+      <c r="C54" s="85" t="str">
+        <v>The Rat Zone · Booth L33</v>
+      </c>
+      <c r="D54" s="85" t="str">
+        <v>3:14 PM</v>
+      </c>
+      <c r="E54" s="85" t="str">
+        <v>3:20 PM</v>
+      </c>
+      <c r="F54" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G54" s="86" t="str"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B55" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C55" s="89" t="str">
+        <v>Block E</v>
+      </c>
+      <c r="D55" s="89" t="str">
+        <v>3:20 PM</v>
+      </c>
+      <c r="E55" s="89" t="str">
+        <v>3:21 PM</v>
+      </c>
+      <c r="F55" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G55" s="90" t="str"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="84" t="str">
+        <v>24</v>
+      </c>
+      <c r="B56" s="87" t="str">
+        <v>Desolus</v>
+      </c>
+      <c r="C56" s="85" t="str">
+        <v>Mark J. Mayers · Booth L32</v>
+      </c>
+      <c r="D56" s="85" t="str">
+        <v>3:21 PM</v>
+      </c>
+      <c r="E56" s="85" t="str">
+        <v>3:27 PM</v>
+      </c>
+      <c r="F56" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G56" s="86" t="str"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B57" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C57" s="89" t="str">
+        <v>Block E</v>
+      </c>
+      <c r="D57" s="89" t="str">
+        <v>3:27 PM</v>
+      </c>
+      <c r="E57" s="89" t="str">
+        <v>3:28 PM</v>
+      </c>
+      <c r="F57" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G57" s="90" t="str"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B58" s="95" t="str">
+        <v>GeekGirlCon Sponsor Segment</v>
+      </c>
+      <c r="C58" s="93" t="str">
+        <v>Sponsor segment · L04</v>
+      </c>
+      <c r="D58" s="93" t="str">
+        <v>3:28 PM</v>
+      </c>
+      <c r="E58" s="93" t="str">
+        <v>3:35 PM</v>
+      </c>
+      <c r="F58" s="93" t="str">
+        <v>E</v>
+      </c>
+      <c r="G58" s="94" t="str"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="84" t="str">
+        <v>25</v>
+      </c>
+      <c r="B59" s="87" t="str">
+        <v>Ascent Rivals</v>
+      </c>
+      <c r="C59" s="85" t="str">
+        <v>GENUN Games · Booth L11</v>
+      </c>
+      <c r="D59" s="85" t="str">
+        <v>3:35 PM</v>
+      </c>
+      <c r="E59" s="85" t="str">
+        <v>3:41 PM</v>
+      </c>
+      <c r="F59" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G59" s="86" t="str"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B60" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C60" s="89" t="str">
+        <v>Block F</v>
+      </c>
+      <c r="D60" s="89" t="str">
+        <v>3:41 PM</v>
+      </c>
+      <c r="E60" s="89" t="str">
+        <v>3:42 PM</v>
+      </c>
+      <c r="F60" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G60" s="90" t="str"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="84" t="str">
+        <v>26</v>
+      </c>
+      <c r="B61" s="87" t="str">
+        <v>Hamsteria</v>
+      </c>
+      <c r="C61" s="85" t="str">
+        <v>2WheelerDev · Booth L10</v>
+      </c>
+      <c r="D61" s="85" t="str">
+        <v>3:42 PM</v>
+      </c>
+      <c r="E61" s="85" t="str">
+        <v>3:48 PM</v>
+      </c>
+      <c r="F61" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G61" s="86" t="str"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B62" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C62" s="89" t="str">
+        <v>Block F</v>
+      </c>
+      <c r="D62" s="89" t="str">
+        <v>3:48 PM</v>
+      </c>
+      <c r="E62" s="89" t="str">
+        <v>3:49 PM</v>
+      </c>
+      <c r="F62" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G62" s="90" t="str"/>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="84" t="str">
+        <v>27</v>
+      </c>
+      <c r="B63" s="87" t="str">
+        <v>Haunted Heist</v>
+      </c>
+      <c r="C63" s="85" t="str">
+        <v>autotroph games · Booth L09</v>
+      </c>
+      <c r="D63" s="85" t="str">
+        <v>3:49 PM</v>
+      </c>
+      <c r="E63" s="85" t="str">
+        <v>3:55 PM</v>
+      </c>
+      <c r="F63" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G63" s="86" t="str"/>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B64" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C64" s="89" t="str">
+        <v>Block F</v>
+      </c>
+      <c r="D64" s="89" t="str">
+        <v>3:55 PM</v>
+      </c>
+      <c r="E64" s="89" t="str">
+        <v>3:56 PM</v>
+      </c>
+      <c r="F64" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G64" s="90" t="str"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="84" t="str">
+        <v>28</v>
+      </c>
+      <c r="B65" s="87" t="str">
+        <v>RUNE GUNNER</v>
+      </c>
+      <c r="C65" s="85" t="str">
+        <v>False Summit · Booth L08</v>
+      </c>
+      <c r="D65" s="85" t="str">
+        <v>3:56 PM</v>
+      </c>
+      <c r="E65" s="85" t="str">
+        <v>4:02 PM</v>
+      </c>
+      <c r="F65" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G65" s="86" t="str"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B66" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C66" s="89" t="str">
+        <v>Block F</v>
+      </c>
+      <c r="D66" s="89" t="str">
+        <v>4:02 PM</v>
+      </c>
+      <c r="E66" s="89" t="str">
+        <v>4:03 PM</v>
+      </c>
+      <c r="F66" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G66" s="90" t="str"/>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B67" s="95" t="str">
+        <v>11 Bit Studios Sponsor Segment</v>
+      </c>
+      <c r="C67" s="93" t="str">
+        <v>Sponsor segment · L06</v>
+      </c>
+      <c r="D67" s="93" t="str">
+        <v>4:03 PM</v>
+      </c>
+      <c r="E67" s="93" t="str">
+        <v>4:10 PM</v>
+      </c>
+      <c r="F67" s="93" t="str">
+        <v>B</v>
+      </c>
+      <c r="G67" s="94" t="str"/>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="84" t="str">
+        <v>29</v>
+      </c>
+      <c r="B68" s="87" t="str">
+        <v>Telera</v>
+      </c>
+      <c r="C68" s="85" t="str">
+        <v>Entropico · Booth U21</v>
+      </c>
+      <c r="D68" s="85" t="str">
+        <v>4:10 PM</v>
+      </c>
+      <c r="E68" s="85" t="str">
+        <v>4:16 PM</v>
+      </c>
+      <c r="F68" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G68" s="86" t="str"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B69" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C69" s="89" t="str">
+        <v>Block G</v>
+      </c>
+      <c r="D69" s="89" t="str">
+        <v>4:16 PM</v>
+      </c>
+      <c r="E69" s="89" t="str">
+        <v>4:17 PM</v>
+      </c>
+      <c r="F69" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G69" s="90" t="str"/>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="84" t="str">
+        <v>30</v>
+      </c>
+      <c r="B70" s="87" t="str">
+        <v>Hogen</v>
+      </c>
+      <c r="C70" s="85" t="str">
+        <v>Scrappyard Games · Booth U22</v>
+      </c>
+      <c r="D70" s="85" t="str">
+        <v>4:17 PM</v>
+      </c>
+      <c r="E70" s="85" t="str">
+        <v>4:23 PM</v>
+      </c>
+      <c r="F70" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G70" s="86" t="str"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B71" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C71" s="89" t="str">
+        <v>Block G</v>
+      </c>
+      <c r="D71" s="89" t="str">
+        <v>4:23 PM</v>
+      </c>
+      <c r="E71" s="89" t="str">
+        <v>4:24 PM</v>
+      </c>
+      <c r="F71" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G71" s="90" t="str"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="84" t="str">
+        <v>31</v>
+      </c>
+      <c r="B72" s="87" t="str">
+        <v>WILL: Follow The Light</v>
+      </c>
+      <c r="C72" s="85" t="str">
+        <v>TomorrowHead Studio · Booth U23</v>
+      </c>
+      <c r="D72" s="85" t="str">
+        <v>4:24 PM</v>
+      </c>
+      <c r="E72" s="85" t="str">
+        <v>4:30 PM</v>
+      </c>
+      <c r="F72" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G72" s="86" t="str"/>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B73" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C73" s="89" t="str">
+        <v>Block G</v>
+      </c>
+      <c r="D73" s="89" t="str">
+        <v>4:30 PM</v>
+      </c>
+      <c r="E73" s="89" t="str">
+        <v>4:31 PM</v>
+      </c>
+      <c r="F73" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G73" s="90" t="str"/>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="84" t="str">
+        <v>32</v>
+      </c>
+      <c r="B74" s="87" t="str">
+        <v>Turning Manor</v>
+      </c>
+      <c r="C74" s="85" t="str">
+        <v>Sabbatical Games · Booth U24</v>
+      </c>
+      <c r="D74" s="85" t="str">
+        <v>4:31 PM</v>
+      </c>
+      <c r="E74" s="85" t="str">
+        <v>4:37 PM</v>
+      </c>
+      <c r="F74" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G74" s="86" t="str"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B75" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C75" s="89" t="str">
+        <v>Block G</v>
+      </c>
+      <c r="D75" s="89" t="str">
+        <v>4:37 PM</v>
+      </c>
+      <c r="E75" s="89" t="str">
+        <v>4:38 PM</v>
+      </c>
+      <c r="F75" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G75" s="90" t="str"/>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="84" t="str">
+        <v>33</v>
+      </c>
+      <c r="B76" s="87" t="str">
+        <v>Steel Swarm: SURVIVOR</v>
+      </c>
+      <c r="C76" s="85" t="str">
+        <v>Clay Token Game Studio, Inc. · Booth U25</v>
+      </c>
+      <c r="D76" s="85" t="str">
+        <v>4:38 PM</v>
+      </c>
+      <c r="E76" s="85" t="str">
+        <v>4:44 PM</v>
+      </c>
+      <c r="F76" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G76" s="86" t="str"/>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B77" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C77" s="89" t="str">
+        <v>Block G</v>
+      </c>
+      <c r="D77" s="89" t="str">
+        <v>4:44 PM</v>
+      </c>
+      <c r="E77" s="89" t="str">
+        <v>4:45 PM</v>
+      </c>
+      <c r="F77" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G77" s="90" t="str"/>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="92" t="str">
+        <v>-</v>
+      </c>
+      <c r="B78" s="95" t="str">
+        <v>NDVisibility Sponsor Segment</v>
+      </c>
+      <c r="C78" s="93" t="str">
+        <v>Sponsor segment · 000</v>
+      </c>
+      <c r="D78" s="93" t="str">
+        <v>4:45 PM</v>
+      </c>
+      <c r="E78" s="93" t="str">
+        <v>4:55 PM</v>
+      </c>
+      <c r="F78" s="93" t="str">
+        <v>C</v>
+      </c>
+      <c r="G78" s="94" t="str"/>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="84" t="str">
+        <v>34</v>
+      </c>
+      <c r="B79" s="87" t="str">
+        <v>HYPERFIST</v>
+      </c>
+      <c r="C79" s="85" t="str">
+        <v>Chirality · Booth U15</v>
+      </c>
+      <c r="D79" s="85" t="str">
+        <v>4:55 PM</v>
+      </c>
+      <c r="E79" s="85" t="str">
+        <v>5:01 PM</v>
+      </c>
+      <c r="F79" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G79" s="86" t="str"/>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B80" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C80" s="89" t="str">
+        <v>Block H</v>
+      </c>
+      <c r="D80" s="89" t="str">
+        <v>5:01 PM</v>
+      </c>
+      <c r="E80" s="89" t="str">
+        <v>5:02 PM</v>
+      </c>
+      <c r="F80" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G80" s="90" t="str"/>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="84" t="str">
+        <v>35</v>
+      </c>
+      <c r="B81" s="87" t="str">
+        <v>Nightmare Kitchen</v>
+      </c>
+      <c r="C81" s="85" t="str">
+        <v>Byteback Studios · Booth U16</v>
+      </c>
+      <c r="D81" s="85" t="str">
+        <v>5:02 PM</v>
+      </c>
+      <c r="E81" s="85" t="str">
+        <v>5:08 PM</v>
+      </c>
+      <c r="F81" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G81" s="86" t="str"/>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B82" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C82" s="89" t="str">
+        <v>Block H</v>
+      </c>
+      <c r="D82" s="89" t="str">
+        <v>5:08 PM</v>
+      </c>
+      <c r="E82" s="89" t="str">
+        <v>5:09 PM</v>
+      </c>
+      <c r="F82" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G82" s="90" t="str"/>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="84" t="str">
+        <v>36</v>
+      </c>
+      <c r="B83" s="87" t="str">
+        <v>Shroomwood</v>
+      </c>
+      <c r="C83" s="85" t="str">
+        <v>Sporelite Games · Booth U17</v>
+      </c>
+      <c r="D83" s="85" t="str">
+        <v>5:09 PM</v>
+      </c>
+      <c r="E83" s="85" t="str">
+        <v>5:15 PM</v>
+      </c>
+      <c r="F83" s="85" t="str">
+        <v>D</v>
+      </c>
+      <c r="G83" s="86" t="str"/>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B84" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C84" s="89" t="str">
+        <v>Block H</v>
+      </c>
+      <c r="D84" s="89" t="str">
+        <v>5:15 PM</v>
+      </c>
+      <c r="E84" s="89" t="str">
+        <v>5:16 PM</v>
+      </c>
+      <c r="F84" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G84" s="90" t="str"/>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="84" t="str">
+        <v>37</v>
+      </c>
+      <c r="B85" s="87" t="str">
+        <v>Knockout 2: Wrath of the Karen</v>
+      </c>
+      <c r="C85" s="85" t="str">
+        <v>ExceptioNULL Games · Booth U18</v>
+      </c>
+      <c r="D85" s="85" t="str">
+        <v>5:16 PM</v>
+      </c>
+      <c r="E85" s="85" t="str">
+        <v>5:22 PM</v>
+      </c>
+      <c r="F85" s="85" t="str">
+        <v>E</v>
+      </c>
+      <c r="G85" s="86" t="str"/>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B86" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C86" s="89" t="str">
+        <v>Block H</v>
+      </c>
+      <c r="D86" s="89" t="str">
+        <v>5:22 PM</v>
+      </c>
+      <c r="E86" s="89" t="str">
+        <v>5:23 PM</v>
+      </c>
+      <c r="F86" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G86" s="90" t="str"/>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="84" t="str">
+        <v>38</v>
+      </c>
+      <c r="B87" s="87" t="str">
+        <v>Cooking Fist</v>
+      </c>
+      <c r="C87" s="85" t="str">
+        <v>Spaghetti Code LLC · Booth U19</v>
+      </c>
+      <c r="D87" s="85" t="str">
+        <v>5:23 PM</v>
+      </c>
+      <c r="E87" s="85" t="str">
+        <v>5:29 PM</v>
+      </c>
+      <c r="F87" s="85" t="str">
+        <v>B</v>
+      </c>
+      <c r="G87" s="86" t="str"/>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B88" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C88" s="89" t="str">
+        <v>Block H</v>
+      </c>
+      <c r="D88" s="89" t="str">
+        <v>5:29 PM</v>
+      </c>
+      <c r="E88" s="89" t="str">
+        <v>5:30 PM</v>
+      </c>
+      <c r="F88" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G88" s="90" t="str"/>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="96" t="str">
+        <v>-</v>
+      </c>
+      <c r="B89" s="99" t="str">
+        <v>Ukrainian Games Videos</v>
+      </c>
+      <c r="C89" s="97" t="str">
+        <v>International showcase · 000</v>
+      </c>
+      <c r="D89" s="97" t="str">
+        <v>5:30 PM</v>
+      </c>
+      <c r="E89" s="97" t="str">
+        <v>5:35 PM</v>
+      </c>
+      <c r="F89" s="97" t="str">
+        <v>Prerecorded</v>
+      </c>
+      <c r="G89" s="98" t="str"/>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="84" t="str">
+        <v>39</v>
+      </c>
+      <c r="B90" s="87" t="str">
+        <v>Killing Baby Hitler</v>
+      </c>
+      <c r="C90" s="85" t="str">
+        <v>The Coffee Industrial Complex · Booth U14</v>
+      </c>
+      <c r="D90" s="85" t="str">
+        <v>5:35 PM</v>
+      </c>
+      <c r="E90" s="85" t="str">
+        <v>5:41 PM</v>
+      </c>
+      <c r="F90" s="85" t="str">
+        <v>C</v>
+      </c>
+      <c r="G90" s="86" t="str"/>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B91" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C91" s="89" t="str">
+        <v>Block I</v>
+      </c>
+      <c r="D91" s="89" t="str">
+        <v>5:41 PM</v>
+      </c>
+      <c r="E91" s="89" t="str">
+        <v>5:42 PM</v>
+      </c>
+      <c r="F91" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G91" s="90" t="str"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B92" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C92" s="89" t="str">
+        <v>Block I</v>
+      </c>
+      <c r="D92" s="89" t="str">
+        <v>5:48 PM</v>
+      </c>
+      <c r="E92" s="89" t="str">
+        <v>5:49 PM</v>
+      </c>
+      <c r="F92" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G92" s="90" t="str"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="96" t="str">
+        <v>-</v>
+      </c>
+      <c r="B93" s="99" t="str">
+        <v>Chile Games Showcase Video</v>
+      </c>
+      <c r="C93" s="97" t="str">
+        <v>International showcase · 000</v>
+      </c>
+      <c r="D93" s="97" t="str">
+        <v>5:49 PM</v>
+      </c>
+      <c r="E93" s="97" t="str">
+        <v>5:54 PM</v>
+      </c>
+      <c r="F93" s="97" t="str">
+        <v>Prerecorded</v>
+      </c>
+      <c r="G93" s="98" t="str"/>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B94" s="91" t="str">
+        <v>Break / Transition</v>
+      </c>
+      <c r="C94" s="89" t="str">
+        <v>Block I</v>
+      </c>
+      <c r="D94" s="89" t="str">
+        <v>5:54 PM</v>
+      </c>
+      <c r="E94" s="89" t="str">
+        <v>5:55 PM</v>
+      </c>
+      <c r="F94" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G94" s="90" t="str"/>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="100" t="str">
+        <v>41</v>
+      </c>
+      <c r="B95" s="103" t="str">
+        <v>Closing / Thank You</v>
+      </c>
+      <c r="C95" s="101" t="str">
+        <v>Seattle Indies</v>
+      </c>
+      <c r="D95" s="101" t="str">
+        <v>5:55 PM</v>
+      </c>
+      <c r="E95" s="101" t="str">
+        <v>6:05 PM</v>
+      </c>
+      <c r="F95" s="101" t="str">
+        <v>All Hosts</v>
+      </c>
+      <c r="G95" s="102" t="str"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Remove redundant run of show break
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -2877,88 +2877,67 @@
       <c r="G91" s="90" t="str"/>
     </row>
     <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="88" t="str">
-        <v>-</v>
-      </c>
-      <c r="B92" s="91" t="str">
+      <c r="A92" s="96" t="str">
+        <v>-</v>
+      </c>
+      <c r="B92" s="99" t="str">
+        <v>Chile Games Showcase Video</v>
+      </c>
+      <c r="C92" s="97" t="str">
+        <v>International showcase · 000</v>
+      </c>
+      <c r="D92" s="97" t="str">
+        <v>5:49 PM</v>
+      </c>
+      <c r="E92" s="97" t="str">
+        <v>5:54 PM</v>
+      </c>
+      <c r="F92" s="97" t="str">
+        <v>Prerecorded</v>
+      </c>
+      <c r="G92" s="98" t="str"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="88" t="str">
+        <v>-</v>
+      </c>
+      <c r="B93" s="91" t="str">
         <v>Break / Transition</v>
       </c>
-      <c r="C92" s="89" t="str">
+      <c r="C93" s="89" t="str">
         <v>Block I</v>
       </c>
-      <c r="D92" s="89" t="str">
-        <v>5:48 PM</v>
-      </c>
-      <c r="E92" s="89" t="str">
-        <v>5:49 PM</v>
-      </c>
-      <c r="F92" s="89" t="str">
-        <v>-</v>
-      </c>
-      <c r="G92" s="90" t="str"/>
-    </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="96" t="str">
-        <v>-</v>
-      </c>
-      <c r="B93" s="99" t="str">
-        <v>Chile Games Showcase Video</v>
-      </c>
-      <c r="C93" s="97" t="str">
-        <v>International showcase · 000</v>
-      </c>
-      <c r="D93" s="97" t="str">
-        <v>5:49 PM</v>
-      </c>
-      <c r="E93" s="97" t="str">
+      <c r="D93" s="89" t="str">
         <v>5:54 PM</v>
       </c>
-      <c r="F93" s="97" t="str">
-        <v>Prerecorded</v>
-      </c>
-      <c r="G93" s="98" t="str"/>
+      <c r="E93" s="89" t="str">
+        <v>5:55 PM</v>
+      </c>
+      <c r="F93" s="89" t="str">
+        <v>-</v>
+      </c>
+      <c r="G93" s="90" t="str"/>
     </row>
     <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="88" t="str">
-        <v>-</v>
-      </c>
-      <c r="B94" s="91" t="str">
-        <v>Break / Transition</v>
-      </c>
-      <c r="C94" s="89" t="str">
-        <v>Block I</v>
-      </c>
-      <c r="D94" s="89" t="str">
-        <v>5:54 PM</v>
-      </c>
-      <c r="E94" s="89" t="str">
+      <c r="A94" s="100" t="str">
+        <v>41</v>
+      </c>
+      <c r="B94" s="103" t="str">
+        <v>Closing / Thank You</v>
+      </c>
+      <c r="C94" s="101" t="str">
+        <v>Seattle Indies</v>
+      </c>
+      <c r="D94" s="101" t="str">
         <v>5:55 PM</v>
       </c>
-      <c r="F94" s="89" t="str">
-        <v>-</v>
-      </c>
-      <c r="G94" s="90" t="str"/>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="100" t="str">
-        <v>41</v>
-      </c>
-      <c r="B95" s="103" t="str">
-        <v>Closing / Thank You</v>
-      </c>
-      <c r="C95" s="101" t="str">
-        <v>Seattle Indies</v>
-      </c>
-      <c r="D95" s="101" t="str">
-        <v>5:55 PM</v>
-      </c>
-      <c r="E95" s="101" t="str">
+      <c r="E94" s="101" t="str">
         <v>6:05 PM</v>
       </c>
-      <c r="F95" s="101" t="str">
+      <c r="F94" s="101" t="str">
         <v>All Hosts</v>
       </c>
-      <c r="G95" s="102" t="str"/>
+      <c r="G94" s="102" t="str"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>

<commit_message>
Shift final run of show segments earlier
</commit_message>
<xml_diff>
--- a/public/SIX-2026-Run-of-Show.xlsx
+++ b/public/SIX-2026-Run-of-Show.xlsx
@@ -2869,7 +2869,7 @@
         <v>5:41 PM</v>
       </c>
       <c r="E91" s="89" t="str">
-        <v>5:49 PM</v>
+        <v>5:42 PM</v>
       </c>
       <c r="F91" s="89" t="str">
         <v>-</v>
@@ -2887,10 +2887,10 @@
         <v>International showcase · 000</v>
       </c>
       <c r="D92" s="97" t="str">
-        <v>5:49 PM</v>
+        <v>5:42 PM</v>
       </c>
       <c r="E92" s="97" t="str">
-        <v>5:54 PM</v>
+        <v>5:47 PM</v>
       </c>
       <c r="F92" s="97" t="str">
         <v>Prerecorded</v>
@@ -2908,10 +2908,10 @@
         <v>Block I</v>
       </c>
       <c r="D93" s="89" t="str">
-        <v>5:54 PM</v>
+        <v>5:47 PM</v>
       </c>
       <c r="E93" s="89" t="str">
-        <v>5:55 PM</v>
+        <v>5:48 PM</v>
       </c>
       <c r="F93" s="89" t="str">
         <v>-</v>
@@ -2929,10 +2929,10 @@
         <v>Seattle Indies</v>
       </c>
       <c r="D94" s="101" t="str">
-        <v>5:55 PM</v>
+        <v>5:48 PM</v>
       </c>
       <c r="E94" s="101" t="str">
-        <v>6:05 PM</v>
+        <v>5:58 PM</v>
       </c>
       <c r="F94" s="101" t="str">
         <v>All Hosts</v>

</xml_diff>